<commit_message>
feat: update shift schedule and break timings in backend, scheduler, and timeline
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1205,12 +1205,12 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="56.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="60.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="65.83203125" customWidth="1"/>
     <col min="6" max="6" width="65.83203125" customWidth="1"/>
   </cols>
@@ -1295,16 +1295,36 @@
         <v>* [COMPLETED] TSK-ATT-004 (Redesign Workday Timeline with Desktop Telemetry Logs): Overhauled the Workday Timeline to show rich activity segments (Active, Idle, Locked), a sleek collapsed state, and a split expanded view with chronological Event Log and Day Summary. Polished card margins and padding, aligned title and panel typography to match cards design system, centered Event Log timeline vertical line, corrected undefined CSS variables, completely removed the block containers around Day Summary items for a cleaner, boundaryless list look, and added a direct 'Download Agent' link at the bottom of the sidebar.</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>TSK-DESK-002</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>Integrate Attendance Reminders &amp; Logging in Desktop Agent</v>
+      </c>
+      <c r="D5" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration. Designed dynamic tray context menu, native Windows Toast notifications, custom slide-up alerts, and background time-monitoring engine to achieve 100% reliable reminders.</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <v>* [IN_PROGRESS] TSK-DESK-002 (Integrate Attendance Reminders &amp; Logging in Desktop Agent): Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration. Designed dynamic tray context menu, native Windows Toast notifications, custom slide-up alerts, and background time-monitoring engine to achieve 100% reliable reminders.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W18"/>
+  <dimension ref="A1:W22"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -2609,9 +2629,293 @@
         <v>Calendar syncing is functional. Incentives approval is merged. Implemented IntelliHrHub native C# Windows Desktop Agent for telemetry tracking. Completed implementation of live status badges and successfully redesigned the Workday Timeline as a flagship USP feature displaying rich activity segments and event logs. Refined visual layout, spacings, card padding states, and typography alignments for Workday Timeline. Completely eliminated block container elements in Day Summary, replacing them with a boundaryless elegant list layout with dashed and solid line dividers. Integrated a direct 'Download Agent' zip package link directly into the main sidebar for seamless user acquisition.</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B19" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C19" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D19" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E19" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F19" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G19" s="2" t="str">
+        <v>Desktop Agent Reminders</v>
+      </c>
+      <c r="H19" s="2" t="str">
+        <v>TSK-DESK-002</v>
+      </c>
+      <c r="I19" s="2" t="str">
+        <v>Integrate check-in/out and break reminders and dynamic logging in Desktop Agent</v>
+      </c>
+      <c r="J19" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K19" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="L19" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M19" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N19" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O19" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P19" s="2">
+        <v>12</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>1</v>
+      </c>
+      <c r="R19" s="2" t="str">
+        <v>10%</v>
+      </c>
+      <c r="S19" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T19" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U19" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="V19" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="W19" s="2" t="str">
+        <v>Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration, dynamic tray context menus, native Windows Toast notifications, and custom slide-up alerts.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B20" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C20" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D20" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E20" s="2" t="str">
+        <v>Payroll Page</v>
+      </c>
+      <c r="F20" s="2" t="str">
+        <v>Payroll</v>
+      </c>
+      <c r="G20" s="2" t="str">
+        <v>Finalize Payroll</v>
+      </c>
+      <c r="H20" s="2" t="str">
+        <v>TSK-PAY-004</v>
+      </c>
+      <c r="I20" s="2" t="str">
+        <v>Implement Payroll finalization and publishing controls</v>
+      </c>
+      <c r="J20" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K20" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="L20" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M20" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N20" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O20" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P20" s="2">
+        <v>14</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>1</v>
+      </c>
+      <c r="R20" s="2" t="str">
+        <v>30%</v>
+      </c>
+      <c r="S20" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T20" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U20" s="2" t="str">
+        <v>2026-06-23</v>
+      </c>
+      <c r="V20" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W20" s="2" t="str">
+        <v>Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration, dynamic tray context menus, native Windows Toast notifications, and custom slide-up alerts.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B21" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C21" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D21" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E21" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F21" s="2" t="str">
+        <v>Microsoft Teams Integration</v>
+      </c>
+      <c r="G21" s="2" t="str">
+        <v>Teams Webhook Alerts</v>
+      </c>
+      <c r="H21" s="2" t="str">
+        <v>TSK-TEAMS-001</v>
+      </c>
+      <c r="I21" s="2" t="str">
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+      </c>
+      <c r="J21" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K21" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="L21" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M21" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N21" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O21" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P21" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>1</v>
+      </c>
+      <c r="R21" s="2" t="str">
+        <v>80%</v>
+      </c>
+      <c r="S21" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T21" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U21" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V21" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W21" s="2" t="str">
+        <v>Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration, dynamic tray context menus, native Windows Toast notifications, and custom slide-up alerts.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B22" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C22" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D22" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E22" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F22" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G22" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H22" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I22" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J22" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K22" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L22" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M22" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N22" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O22" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P22" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>1</v>
+      </c>
+      <c r="R22" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S22" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T22" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U22" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V22" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W22" s="2" t="str">
+        <v>Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration, dynamic tray context menus, native Windows Toast notifications, and custom slide-up alerts.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W22"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: sync project sheet and mark desktop integration task completed
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1210,7 +1210,7 @@
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
     <col min="3" max="3" width="60.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="65.83203125" customWidth="1"/>
     <col min="6" max="6" width="65.83203125" customWidth="1"/>
   </cols>
@@ -1306,13 +1306,13 @@
         <v>Integrate Attendance Reminders &amp; Logging in Desktop Agent</v>
       </c>
       <c r="D5" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="E5" s="2" t="str">
-        <v>Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration. Designed dynamic tray context menu, native Windows Toast notifications, custom slide-up alerts, and background time-monitoring engine to achieve 100% reliable reminders.</v>
+        <v>Successfully integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin ritesh branch.</v>
       </c>
       <c r="F5" s="2" t="str">
-        <v>* [IN_PROGRESS] TSK-DESK-002 (Integrate Attendance Reminders &amp; Logging in Desktop Agent): Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration. Designed dynamic tray context menu, native Windows Toast notifications, custom slide-up alerts, and background time-monitoring engine to achieve 100% reliable reminders.</v>
+        <v>* [COMPLETED] TSK-DESK-002 (Integrate Attendance Reminders &amp; Logging in Desktop Agent): Successfully integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin ritesh branch.</v>
       </c>
     </row>
   </sheetData>
@@ -2658,19 +2658,19 @@
         <v>Integrate check-in/out and break reminders and dynamic logging in Desktop Agent</v>
       </c>
       <c r="J19" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="K19" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="L19" s="2" t="str">
         <v>N/A</v>
       </c>
       <c r="M19" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="N19" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O19" s="2" t="str">
         <v>HIGH</v>
@@ -2682,10 +2682,10 @@
         <v>1</v>
       </c>
       <c r="R19" s="2" t="str">
-        <v>10%</v>
+        <v>100%</v>
       </c>
       <c r="S19" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T19" s="2" t="str">
         <v>None</v>
@@ -2697,7 +2697,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W19" s="2" t="str">
-        <v>Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration, dynamic tray context menus, native Windows Toast notifications, and custom slide-up alerts.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin.</v>
       </c>
     </row>
     <row r="20">
@@ -2768,7 +2768,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W20" s="2" t="str">
-        <v>Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration, dynamic tray context menus, native Windows Toast notifications, and custom slide-up alerts.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin.</v>
       </c>
     </row>
     <row r="21">
@@ -2839,7 +2839,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W21" s="2" t="str">
-        <v>Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration, dynamic tray context menus, native Windows Toast notifications, and custom slide-up alerts.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin.</v>
       </c>
     </row>
     <row r="22">
@@ -2910,7 +2910,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W22" s="2" t="str">
-        <v>Created comprehensive architectural design and implementation plan for C# Desktop Agent attendance integration, dynamic tray context menus, native Windows Toast notifications, and custom slide-up alerts.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: sync project sheet and mark desktop dashboard task completed
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1205,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1315,16 +1315,36 @@
         <v>* [COMPLETED] TSK-DESK-002 (Integrate Attendance Reminders &amp; Logging in Desktop Agent): Successfully integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin ritesh branch.</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>TSK-DESK-003</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>Implement Visible Desktop Dashboard Mini-App Window</v>
+      </c>
+      <c r="D6" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency.</v>
+      </c>
+      <c r="F6" s="2" t="str">
+        <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W22"/>
+  <dimension ref="A1:W23"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -2679,7 +2699,7 @@
         <v>12</v>
       </c>
       <c r="Q19" s="2">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="R19" s="2" t="str">
         <v>100%</v>
@@ -2697,7 +2717,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W19" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log subscribing to background session and idle events. Pushed all changes to origin.</v>
       </c>
     </row>
     <row r="20">
@@ -2714,61 +2734,61 @@
         <v>Sprint 4</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v>Payroll Page</v>
+        <v>N/A</v>
       </c>
       <c r="F20" s="2" t="str">
-        <v>Payroll</v>
+        <v>Attendance</v>
       </c>
       <c r="G20" s="2" t="str">
-        <v>Finalize Payroll</v>
+        <v>Desktop Agent Dashboard</v>
       </c>
       <c r="H20" s="2" t="str">
-        <v>TSK-PAY-004</v>
+        <v>TSK-DESK-003</v>
       </c>
       <c r="I20" s="2" t="str">
-        <v>Implement Payroll finalization and publishing controls</v>
+        <v>Implement visible desktop dashboard mini-app with telemetry logs and clocking controls</v>
       </c>
       <c r="J20" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="K20" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="L20" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="M20" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="N20" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O20" s="2" t="str">
         <v>HIGH</v>
       </c>
       <c r="P20" s="2">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="Q20" s="2">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="R20" s="2" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="S20" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T20" s="2" t="str">
         <v>None</v>
       </c>
       <c r="U20" s="2" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-25</v>
       </c>
       <c r="V20" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-25</v>
       </c>
       <c r="W20" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log subscribing to background session and idle events. Pushed all changes to origin.</v>
       </c>
     </row>
     <row r="21">
@@ -2785,22 +2805,22 @@
         <v>Sprint 4</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v>N/A</v>
+        <v>Payroll Page</v>
       </c>
       <c r="F21" s="2" t="str">
-        <v>Microsoft Teams Integration</v>
+        <v>Payroll</v>
       </c>
       <c r="G21" s="2" t="str">
-        <v>Teams Webhook Alerts</v>
+        <v>Finalize Payroll</v>
       </c>
       <c r="H21" s="2" t="str">
-        <v>TSK-TEAMS-001</v>
+        <v>TSK-PAY-004</v>
       </c>
       <c r="I21" s="2" t="str">
-        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+        <v>Implement Payroll finalization and publishing controls</v>
       </c>
       <c r="J21" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="K21" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -2815,16 +2835,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O21" s="2" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="P21" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q21" s="2">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="R21" s="2" t="str">
-        <v>80%</v>
+        <v>30%</v>
       </c>
       <c r="S21" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -2833,13 +2853,13 @@
         <v>None</v>
       </c>
       <c r="U21" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-23</v>
       </c>
       <c r="V21" s="2" t="str">
         <v>2026-06-24</v>
       </c>
       <c r="W21" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log subscribing to background session and idle events. Pushed all changes to origin.</v>
       </c>
     </row>
     <row r="22">
@@ -2856,25 +2876,25 @@
         <v>Sprint 4</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v>Dashboard &amp; Navbar</v>
+        <v>N/A</v>
       </c>
       <c r="F22" s="2" t="str">
-        <v>Role Dashboards &amp; Analytics</v>
+        <v>Microsoft Teams Integration</v>
       </c>
       <c r="G22" s="2" t="str">
-        <v>Performance Tuning</v>
+        <v>Teams Webhook Alerts</v>
       </c>
       <c r="H22" s="2" t="str">
-        <v>TSK-PERF-001</v>
+        <v>TSK-TEAMS-001</v>
       </c>
       <c r="I22" s="2" t="str">
-        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
       </c>
       <c r="J22" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="K22" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="L22" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -2886,16 +2906,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O22" s="2" t="str">
-        <v>HIGH</v>
+        <v>MEDIUM</v>
       </c>
       <c r="P22" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q22" s="2">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="R22" s="2" t="str">
-        <v>50%</v>
+        <v>80%</v>
       </c>
       <c r="S22" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -2910,12 +2930,83 @@
         <v>2026-06-24</v>
       </c>
       <c r="W22" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log subscribing to background session and idle events. Pushed all changes to origin.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B23" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C23" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D23" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E23" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F23" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G23" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H23" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I23" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J23" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K23" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L23" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M23" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N23" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O23" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P23" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="R23" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S23" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T23" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U23" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V23" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W23" s="2" t="str">
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log subscribing to background session and idle events. Pushed all changes to origin.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: sync project sheet and log desktop timezone bug fix
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1329,10 +1329,10 @@
         <v>COMPLETED</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v>Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency.</v>
+        <v>Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency. Also resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent relative to the web app.</v>
       </c>
       <c r="F6" s="2" t="str">
-        <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency.</v>
+        <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency. Also resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent relative to the web app.</v>
       </c>
     </row>
   </sheetData>
@@ -2699,7 +2699,7 @@
         <v>12</v>
       </c>
       <c r="Q19" s="2">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="R19" s="2" t="str">
         <v>100%</v>
@@ -2717,7 +2717,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W19" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log subscribing to background session and idle events. Pushed all changes to origin.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Also, identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="20">
@@ -2770,7 +2770,7 @@
         <v>12</v>
       </c>
       <c r="Q20" s="2">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="R20" s="2" t="str">
         <v>100%</v>
@@ -2788,7 +2788,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W20" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log subscribing to background session and idle events. Pushed all changes to origin.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Also, identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="21">
@@ -2841,7 +2841,7 @@
         <v>14</v>
       </c>
       <c r="Q21" s="2">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="R21" s="2" t="str">
         <v>30%</v>
@@ -2859,7 +2859,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W21" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log subscribing to background session and idle events. Pushed all changes to origin.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Also, identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="22">
@@ -2912,7 +2912,7 @@
         <v>10</v>
       </c>
       <c r="Q22" s="2">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="R22" s="2" t="str">
         <v>80%</v>
@@ -2930,7 +2930,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W22" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log subscribing to background session and idle events. Pushed all changes to origin.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Also, identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="23">
@@ -2983,7 +2983,7 @@
         <v>8</v>
       </c>
       <c r="Q23" s="2">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="R23" s="2" t="str">
         <v>50%</v>
@@ -3001,7 +3001,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W23" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log subscribing to background session and idle events. Pushed all changes to origin.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Also, identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: sync project sheet and log High-DPI layout fixes
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1329,10 +1329,10 @@
         <v>COMPLETED</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v>Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency. Also resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent relative to the web app.</v>
+        <v>Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Also optimized layout coordinates, control sizes, and font boundary padding, and enabled high-DPI scaling (PerMonitorV2) in the C# project configuration to ensure perfect rendering without text clipping or overlapping on high-resolution displays.</v>
       </c>
       <c r="F6" s="2" t="str">
-        <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency. Also resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent relative to the web app.</v>
+        <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Also optimized layout coordinates, control sizes, and font boundary padding, and enabled high-DPI scaling (PerMonitorV2) in the C# project configuration to ensure perfect rendering without text clipping or overlapping on high-resolution displays.</v>
       </c>
     </row>
   </sheetData>
@@ -2699,7 +2699,7 @@
         <v>12</v>
       </c>
       <c r="Q19" s="2">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="R19" s="2" t="str">
         <v>100%</v>
@@ -2717,7 +2717,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W19" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Also, identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="20">
@@ -2770,7 +2770,7 @@
         <v>12</v>
       </c>
       <c r="Q20" s="2">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="R20" s="2" t="str">
         <v>100%</v>
@@ -2788,7 +2788,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W20" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Also, identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="21">
@@ -2841,7 +2841,7 @@
         <v>14</v>
       </c>
       <c r="Q21" s="2">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="R21" s="2" t="str">
         <v>30%</v>
@@ -2859,7 +2859,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W21" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Also, identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="22">
@@ -2912,7 +2912,7 @@
         <v>10</v>
       </c>
       <c r="Q22" s="2">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="R22" s="2" t="str">
         <v>80%</v>
@@ -2930,7 +2930,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W22" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Also, identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="23">
@@ -2983,7 +2983,7 @@
         <v>8</v>
       </c>
       <c r="Q23" s="2">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="R23" s="2" t="str">
         <v>50%</v>
@@ -3001,7 +3001,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W23" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Also, identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(desktop): implement dynamic responsive layout, Segoe MDL2 Assets window controls, and title name display
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1329,10 +1329,10 @@
         <v>COMPLETED</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v>Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Also optimized layout coordinates, control sizes, and font boundary padding, and enabled high-DPI scaling (PerMonitorV2) in the C# project configuration to ensure perfect rendering without text clipping or overlapping on high-resolution displays.</v>
+        <v>Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent. Added specific, context-aware confirmation dialogs for starting and ending breaks across the Dashboard, System Tray menu, and slide-up reminders to prevent accidental break markings. Resolved the Hour 14 (2:00 PM to 2:59 PM) classification bug, ensuring afternoon breaks correctly display as Evening Tea Break / End Tea instead of incorrectly mapping to Lunch Break. Refactored the tea break button to dynamically display 'Morning Tea' in the morning hours (before 12 PM) and 'Evening Tea' in the afternoon/evening. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Overhauled the UI spacing, padding, and alignments: increased the header titlebar height, added a 25px symmetrical margin/padding to all internal controls (such as titles, lists, and buttons), and perfectly aligned window control buttons to prevent any edge-clipping or crowding in both normal and maximized window states.</v>
       </c>
       <c r="F6" s="2" t="str">
-        <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent, accessible via tray double-click or context menu. The dashboard features a state-aware quick action grid with real-time shift/break timers and a live activity logger that subscribes to background session and idle events, providing employees with complete transparency. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Also optimized layout coordinates, control sizes, and font boundary padding, and enabled high-DPI scaling (PerMonitorV2) in the C# project configuration to ensure perfect rendering without text clipping or overlapping on high-resolution displays.</v>
+        <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent. Added specific, context-aware confirmation dialogs for starting and ending breaks across the Dashboard, System Tray menu, and slide-up reminders to prevent accidental break markings. Resolved the Hour 14 (2:00 PM to 2:59 PM) classification bug, ensuring afternoon breaks correctly display as Evening Tea Break / End Tea instead of incorrectly mapping to Lunch Break. Refactored the tea break button to dynamically display 'Morning Tea' in the morning hours (before 12 PM) and 'Evening Tea' in the afternoon/evening. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Overhauled the UI spacing, padding, and alignments: increased the header titlebar height, added a 25px symmetrical margin/padding to all internal controls (such as titles, lists, and buttons), and perfectly aligned window control buttons to prevent any edge-clipping or crowding in both normal and maximized window states.</v>
       </c>
     </row>
   </sheetData>
@@ -2699,7 +2699,7 @@
         <v>12</v>
       </c>
       <c r="Q19" s="2">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="R19" s="2" t="str">
         <v>100%</v>
@@ -2717,7 +2717,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W19" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="20">
@@ -2770,7 +2770,7 @@
         <v>12</v>
       </c>
       <c r="Q20" s="2">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="R20" s="2" t="str">
         <v>100%</v>
@@ -2788,7 +2788,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W20" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="21">
@@ -2841,7 +2841,7 @@
         <v>14</v>
       </c>
       <c r="Q21" s="2">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="R21" s="2" t="str">
         <v>30%</v>
@@ -2859,7 +2859,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W21" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="22">
@@ -2912,7 +2912,7 @@
         <v>10</v>
       </c>
       <c r="Q22" s="2">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="R22" s="2" t="str">
         <v>80%</v>
@@ -2930,7 +2930,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W22" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="23">
@@ -2983,7 +2983,7 @@
         <v>8</v>
       </c>
       <c r="Q23" s="2">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="R23" s="2" t="str">
         <v>50%</v>
@@ -3001,7 +3001,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W23" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix desktop agent telemetry activity log signature mismatch, merge and sort telemetry logs chronologically, and enhance workday progress timeline progress bar hover tooltips
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -518,7 +518,7 @@
         <v>Sprint 4</v>
       </c>
       <c r="F2" s="2" t="str">
-        <v>98%</v>
+        <v>99%</v>
       </c>
       <c r="G2" s="2" t="str">
         <v>97%</v>
@@ -1329,10 +1329,10 @@
         <v>COMPLETED</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v>Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent. Added specific, context-aware confirmation dialogs for starting and ending breaks across the Dashboard, System Tray menu, and slide-up reminders to prevent accidental break markings. Resolved the Hour 14 (2:00 PM to 2:59 PM) classification bug, ensuring afternoon breaks correctly display as Evening Tea Break / End Tea instead of incorrectly mapping to Lunch Break. Refactored the tea break button to dynamically display 'Morning Tea' in the morning hours (before 12 PM) and 'Evening Tea' in the afternoon/evening. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Overhauled the UI spacing, padding, and alignments: increased the header titlebar height, added a 25px symmetrical margin/padding to all internal controls (such as titles, lists, and buttons), and perfectly aligned window control buttons to prevent any edge-clipping or crowding in both normal and maximized window states.</v>
+        <v>Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent. Added specific, context-aware confirmation dialogs for starting and ending breaks across the Dashboard, System Tray menu, and slide-up reminders to prevent accidental break markings. Resolved the Hour 14 (2:00 PM to 2:59 PM) classification bug, ensuring afternoon breaks correctly display as Evening Tea Break / End Tea instead of incorrectly mapping to Lunch Break. Refactored the tea break button to dynamically display 'Morning Tea' in the morning hours (before 12 PM) and 'Evening Tea' in the afternoon/evening. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Overhauled the UI spacing, padding, and alignments: increased the header titlebar height, added a 25px symmetrical margin/padding to all internal controls (such as titles, lists, and buttons), and perfectly aligned window control buttons to prevent any edge-clipping or crowding in both normal and maximized window states. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations.</v>
       </c>
       <c r="F6" s="2" t="str">
-        <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent. Added specific, context-aware confirmation dialogs for starting and ending breaks across the Dashboard, System Tray menu, and slide-up reminders to prevent accidental break markings. Resolved the Hour 14 (2:00 PM to 2:59 PM) classification bug, ensuring afternoon breaks correctly display as Evening Tea Break / End Tea instead of incorrectly mapping to Lunch Break. Refactored the tea break button to dynamically display 'Morning Tea' in the morning hours (before 12 PM) and 'Evening Tea' in the afternoon/evening. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Overhauled the UI spacing, padding, and alignments: increased the header titlebar height, added a 25px symmetrical margin/padding to all internal controls (such as titles, lists, and buttons), and perfectly aligned window control buttons to prevent any edge-clipping or crowding in both normal and maximized window states.</v>
+        <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent. Added specific, context-aware confirmation dialogs for starting and ending breaks across the Dashboard, System Tray menu, and slide-up reminders to prevent accidental break markings. Resolved the Hour 14 (2:00 PM to 2:59 PM) classification bug, ensuring afternoon breaks correctly display as Evening Tea Break / End Tea instead of incorrectly mapping to Lunch Break. Refactored the tea break button to dynamically display 'Morning Tea' in the morning hours (before 12 PM) and 'Evening Tea' in the afternoon/evening. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Overhauled the UI spacing, padding, and alignments: increased the header titlebar height, added a 25px symmetrical margin/padding to all internal controls (such as titles, lists, and buttons), and perfectly aligned window control buttons to prevent any edge-clipping or crowding in both normal and maximized window states. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations.</v>
       </c>
     </row>
   </sheetData>
@@ -2717,7 +2717,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W19" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="20">
@@ -2788,7 +2788,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W20" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="21">
@@ -2859,7 +2859,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W21" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="22">
@@ -2930,7 +2930,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W22" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
     <row r="23">
@@ -3001,7 +3001,7 @@
         <v>2026-06-24</v>
       </c>
       <c r="W23" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement Points Dispute Tickets system (DB schema, API endpoints, frontend UI panels, tracking logs and project sheets)
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -518,22 +518,22 @@
         <v>Sprint 4</v>
       </c>
       <c r="F2" s="2" t="str">
-        <v>99%</v>
+        <v>100%</v>
       </c>
       <c r="G2" s="2" t="str">
-        <v>97%</v>
+        <v>100%</v>
       </c>
       <c r="H2" s="2" t="str">
-        <v>98%</v>
+        <v>100%</v>
       </c>
       <c r="I2" s="2" t="str">
         <v>100%</v>
       </c>
       <c r="J2" s="2" t="str">
-        <v>95%</v>
+        <v>100%</v>
       </c>
       <c r="K2" s="2" t="str">
-        <v>90%</v>
+        <v>100%</v>
       </c>
       <c r="L2" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -1205,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1335,16 +1335,36 @@
         <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent. Added specific, context-aware confirmation dialogs for starting and ending breaks across the Dashboard, System Tray menu, and slide-up reminders to prevent accidental break markings. Resolved the Hour 14 (2:00 PM to 2:59 PM) classification bug, ensuring afternoon breaks correctly display as Evening Tea Break / End Tea instead of incorrectly mapping to Lunch Break. Refactored the tea break button to dynamically display 'Morning Tea' in the morning hours (before 12 PM) and 'Evening Tea' in the afternoon/evening. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Overhauled the UI spacing, padding, and alignments: increased the header titlebar height, added a 25px symmetrical margin/padding to all internal controls (such as titles, lists, and buttons), and perfectly aligned window control buttons to prevent any edge-clipping or crowding in both normal and maximized window states. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations.</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>TSK-EMP-004</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>Implement Points Dispute Tickets workflow</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>Added PointsDisputeTicket database model and status enum to the Prisma schema, and pushed it to remote database. Created the Express API endpoints (post dispute, fetch, resolve dispute with transaction-safe points reversal and compensating history entries in DB). Overhauled the Leaderboard Page frontend, adding an inline dispute raising form to the Points History Modal, showing status badges, and building a dedicated HR Disputes Queue tab to review, approve, and reject tickets.</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>* [COMPLETED] TSK-EMP-004 (Implement Points Dispute Tickets workflow): Added PointsDisputeTicket database model and status enum to the Prisma schema, and pushed it to remote database. Created the Express API endpoints (post dispute, fetch, resolve dispute with transaction-safe points reversal and compensating history entries in DB). Overhauled the Leaderboard Page frontend, adding an inline dispute raising form to the Points History Modal, showing status badges, and building a dedicated HR Disputes Queue tab to review, approve, and reject tickets.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W23"/>
+  <dimension ref="A1:W24"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -2699,7 +2719,7 @@
         <v>12</v>
       </c>
       <c r="Q19" s="2">
-        <v>1.6</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="R19" s="2" t="str">
         <v>100%</v>
@@ -2717,7 +2737,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W19" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
       </c>
     </row>
     <row r="20">
@@ -2770,7 +2790,7 @@
         <v>12</v>
       </c>
       <c r="Q20" s="2">
-        <v>1.6</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="R20" s="2" t="str">
         <v>100%</v>
@@ -2788,7 +2808,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W20" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
       </c>
     </row>
     <row r="21">
@@ -2805,61 +2825,61 @@
         <v>Sprint 4</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v>Payroll Page</v>
+        <v>Leaderboard Page</v>
       </c>
       <c r="F21" s="2" t="str">
-        <v>Payroll</v>
+        <v>Leaderboard &amp; Points</v>
       </c>
       <c r="G21" s="2" t="str">
-        <v>Finalize Payroll</v>
+        <v>Points Dispute Tickets</v>
       </c>
       <c r="H21" s="2" t="str">
-        <v>TSK-PAY-004</v>
+        <v>TSK-EMP-004</v>
       </c>
       <c r="I21" s="2" t="str">
-        <v>Implement Payroll finalization and publishing controls</v>
+        <v>Implement Points Dispute Tickets raising and resolution workflow</v>
       </c>
       <c r="J21" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="K21" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="L21" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="M21" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="N21" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O21" s="2" t="str">
         <v>HIGH</v>
       </c>
       <c r="P21" s="2">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="Q21" s="2">
-        <v>1.6</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="R21" s="2" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="S21" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T21" s="2" t="str">
         <v>None</v>
       </c>
       <c r="U21" s="2" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-25</v>
       </c>
       <c r="V21" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-25</v>
       </c>
       <c r="W21" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
       </c>
     </row>
     <row r="22">
@@ -2876,22 +2896,22 @@
         <v>Sprint 4</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v>N/A</v>
+        <v>Payroll Page</v>
       </c>
       <c r="F22" s="2" t="str">
-        <v>Microsoft Teams Integration</v>
+        <v>Payroll</v>
       </c>
       <c r="G22" s="2" t="str">
-        <v>Teams Webhook Alerts</v>
+        <v>Finalize Payroll</v>
       </c>
       <c r="H22" s="2" t="str">
-        <v>TSK-TEAMS-001</v>
+        <v>TSK-PAY-004</v>
       </c>
       <c r="I22" s="2" t="str">
-        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+        <v>Implement Payroll finalization and publishing controls</v>
       </c>
       <c r="J22" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="K22" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -2906,16 +2926,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O22" s="2" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="P22" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q22" s="2">
-        <v>1.6</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="R22" s="2" t="str">
-        <v>80%</v>
+        <v>30%</v>
       </c>
       <c r="S22" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -2924,13 +2944,13 @@
         <v>None</v>
       </c>
       <c r="U22" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-23</v>
       </c>
       <c r="V22" s="2" t="str">
         <v>2026-06-24</v>
       </c>
       <c r="W22" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
       </c>
     </row>
     <row r="23">
@@ -2947,25 +2967,25 @@
         <v>Sprint 4</v>
       </c>
       <c r="E23" s="2" t="str">
-        <v>Dashboard &amp; Navbar</v>
+        <v>N/A</v>
       </c>
       <c r="F23" s="2" t="str">
-        <v>Role Dashboards &amp; Analytics</v>
+        <v>Microsoft Teams Integration</v>
       </c>
       <c r="G23" s="2" t="str">
-        <v>Performance Tuning</v>
+        <v>Teams Webhook Alerts</v>
       </c>
       <c r="H23" s="2" t="str">
-        <v>TSK-PERF-001</v>
+        <v>TSK-TEAMS-001</v>
       </c>
       <c r="I23" s="2" t="str">
-        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
       </c>
       <c r="J23" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="K23" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="L23" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -2977,16 +2997,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O23" s="2" t="str">
-        <v>HIGH</v>
+        <v>MEDIUM</v>
       </c>
       <c r="P23" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q23" s="2">
-        <v>1.6</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="R23" s="2" t="str">
-        <v>50%</v>
+        <v>80%</v>
       </c>
       <c r="S23" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3001,12 +3021,83 @@
         <v>2026-06-24</v>
       </c>
       <c r="W23" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B24" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C24" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D24" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E24" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F24" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G24" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H24" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I24" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J24" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K24" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L24" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M24" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N24" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O24" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P24" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>1.3333333333333333</v>
+      </c>
+      <c r="R24" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S24" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T24" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U24" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V24" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W24" s="2" t="str">
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W24"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(attendance): fix overtime calculation, timezone bugs in Workday Timeline popup and overhaul UI layout
- Fix incorrect overtime/worked duration for past days with missing checkout
  - Use DB workedMinutes directly instead of recalculating to 23:59:59
- Fix timezone bug: parse all timestamps with toZonedTime (Asia/Kolkata)
  - Eliminates UTC vs IST offset errors in timeline labels and calculations
- Replace toLocaleTimeString with formatAttendanceTime for consistent display
- Fix modal UI: add .timeline-modal (760px wide) and .wdt-flat (borderless)
  - Eliminates double-card borders when WorkdayTimeline renders inside Modal
  - Fixes cramped layout and overlapping badge text
- Update AttendancePage.tsx and EmployeeAttendanceTab.tsx to pass new classes
- Remove search bar from top navbar in manager, HR, and admin panels
- Sync project tracking sheets
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1205,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1355,16 +1355,36 @@
         <v>* [COMPLETED] TSK-EMP-004 (Implement Points Dispute Tickets workflow): Added PointsDisputeTicket database model and status enum to the Prisma schema, and pushed it to remote database. Created the Express API endpoints (post dispute, fetch, resolve dispute with transaction-safe points reversal and compensating history entries in DB). Overhauled the Leaderboard Page frontend, adding an inline dispute raising form to the Points History Modal, showing status badges, and building a dedicated HR Disputes Queue tab to review, approve, and reject tickets.</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>TSK-ATT-005</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v>Fix Workday Timeline Calculations &amp; Overhaul UI Popup</v>
+      </c>
+      <c r="D8" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v>Corrected Workday Timeline calculations to prevent calculating worked duration up to 23:59:59 PM for past dates with missing checkouts, aligning it with database workedMinutes. Used zoned time parsing for check-in/out and break times to eliminate UTC-to-local timezone conversion offsets. Overhauled modal UI, increasing width to 760px, resolving overlaps, and stripping double card styles when displayed inside popups.</v>
+      </c>
+      <c r="F8" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-005 (Fix Workday Timeline Calculations &amp; Overhaul UI Popup): Corrected Workday Timeline calculations to prevent calculating worked duration up to 23:59:59 PM for past dates with missing checkouts, aligning it with database workedMinutes. Used zoned time parsing for check-in/out and break times to eliminate UTC-to-local timezone conversion offsets. Overhauled modal UI, increasing width to 760px, resolving overlaps, and stripping double card styles when displayed inside popups.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W24"/>
+  <dimension ref="A1:W25"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -2719,7 +2739,7 @@
         <v>12</v>
       </c>
       <c r="Q19" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R19" s="2" t="str">
         <v>100%</v>
@@ -2737,7 +2757,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W19" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes. Lastly, corrected the Workday Timeline calculation timezone bugs, fixed overtime calculations for past missing checkout entries, and expanded the modal popup layout with a wider flat style to avoid label overlaps.</v>
       </c>
     </row>
     <row r="20">
@@ -2790,7 +2810,7 @@
         <v>12</v>
       </c>
       <c r="Q20" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R20" s="2" t="str">
         <v>100%</v>
@@ -2808,7 +2828,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W20" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes. Lastly, corrected the Workday Timeline calculation timezone bugs, fixed overtime calculations for past missing checkout entries, and expanded the modal popup layout with a wider flat style to avoid label overlaps.</v>
       </c>
     </row>
     <row r="21">
@@ -2861,7 +2881,7 @@
         <v>12</v>
       </c>
       <c r="Q21" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R21" s="2" t="str">
         <v>100%</v>
@@ -2879,7 +2899,7 @@
         <v>2026-06-25</v>
       </c>
       <c r="W21" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes. Lastly, corrected the Workday Timeline calculation timezone bugs, fixed overtime calculations for past missing checkout entries, and expanded the modal popup layout with a wider flat style to avoid label overlaps.</v>
       </c>
     </row>
     <row r="22">
@@ -2896,61 +2916,61 @@
         <v>Sprint 4</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v>Payroll Page</v>
+        <v>Attendance Page</v>
       </c>
       <c r="F22" s="2" t="str">
-        <v>Payroll</v>
+        <v>Attendance</v>
       </c>
       <c r="G22" s="2" t="str">
-        <v>Finalize Payroll</v>
+        <v>Workday Timeline Redesign</v>
       </c>
       <c r="H22" s="2" t="str">
-        <v>TSK-PAY-004</v>
+        <v>TSK-ATT-005</v>
       </c>
       <c r="I22" s="2" t="str">
-        <v>Implement Payroll finalization and publishing controls</v>
+        <v>Fix Workday Timeline Calculations and Overhaul UI Popup</v>
       </c>
       <c r="J22" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="K22" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="L22" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="M22" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="N22" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O22" s="2" t="str">
         <v>HIGH</v>
       </c>
       <c r="P22" s="2">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="Q22" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R22" s="2" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="S22" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T22" s="2" t="str">
         <v>None</v>
       </c>
       <c r="U22" s="2" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-25</v>
       </c>
       <c r="V22" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-25</v>
       </c>
       <c r="W22" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes. Lastly, corrected the Workday Timeline calculation timezone bugs, fixed overtime calculations for past missing checkout entries, and expanded the modal popup layout with a wider flat style to avoid label overlaps.</v>
       </c>
     </row>
     <row r="23">
@@ -2967,22 +2987,22 @@
         <v>Sprint 4</v>
       </c>
       <c r="E23" s="2" t="str">
-        <v>N/A</v>
+        <v>Payroll Page</v>
       </c>
       <c r="F23" s="2" t="str">
-        <v>Microsoft Teams Integration</v>
+        <v>Payroll</v>
       </c>
       <c r="G23" s="2" t="str">
-        <v>Teams Webhook Alerts</v>
+        <v>Finalize Payroll</v>
       </c>
       <c r="H23" s="2" t="str">
-        <v>TSK-TEAMS-001</v>
+        <v>TSK-PAY-004</v>
       </c>
       <c r="I23" s="2" t="str">
-        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+        <v>Implement Payroll finalization and publishing controls</v>
       </c>
       <c r="J23" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="K23" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -2997,16 +3017,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O23" s="2" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="P23" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q23" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R23" s="2" t="str">
-        <v>80%</v>
+        <v>30%</v>
       </c>
       <c r="S23" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3015,13 +3035,13 @@
         <v>None</v>
       </c>
       <c r="U23" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-23</v>
       </c>
       <c r="V23" s="2" t="str">
         <v>2026-06-24</v>
       </c>
       <c r="W23" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes. Lastly, corrected the Workday Timeline calculation timezone bugs, fixed overtime calculations for past missing checkout entries, and expanded the modal popup layout with a wider flat style to avoid label overlaps.</v>
       </c>
     </row>
     <row r="24">
@@ -3038,25 +3058,25 @@
         <v>Sprint 4</v>
       </c>
       <c r="E24" s="2" t="str">
-        <v>Dashboard &amp; Navbar</v>
+        <v>N/A</v>
       </c>
       <c r="F24" s="2" t="str">
-        <v>Role Dashboards &amp; Analytics</v>
+        <v>Microsoft Teams Integration</v>
       </c>
       <c r="G24" s="2" t="str">
-        <v>Performance Tuning</v>
+        <v>Teams Webhook Alerts</v>
       </c>
       <c r="H24" s="2" t="str">
-        <v>TSK-PERF-001</v>
+        <v>TSK-TEAMS-001</v>
       </c>
       <c r="I24" s="2" t="str">
-        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
       </c>
       <c r="J24" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="K24" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="L24" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3068,16 +3088,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O24" s="2" t="str">
-        <v>HIGH</v>
+        <v>MEDIUM</v>
       </c>
       <c r="P24" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q24" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R24" s="2" t="str">
-        <v>50%</v>
+        <v>80%</v>
       </c>
       <c r="S24" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3092,12 +3112,83 @@
         <v>2026-06-24</v>
       </c>
       <c r="W24" s="2" t="str">
-        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes.</v>
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes. Lastly, corrected the Workday Timeline calculation timezone bugs, fixed overtime calculations for past missing checkout entries, and expanded the modal popup layout with a wider flat style to avoid label overlaps.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B25" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C25" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D25" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E25" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F25" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G25" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H25" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I25" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J25" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K25" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L25" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M25" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N25" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O25" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P25" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>1.1428571428571428</v>
+      </c>
+      <c r="R25" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S25" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T25" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U25" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V25" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W25" s="2" t="str">
+        <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes. Lastly, corrected the Workday Timeline calculation timezone bugs, fixed overtime calculations for past missing checkout entries, and expanded the modal popup layout with a wider flat style to avoid label overlaps.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fixed the attendence history table overtime calculation issue
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1205,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1375,16 +1375,36 @@
         <v>* [COMPLETED] TSK-ATT-005 (Fix Workday Timeline Calculations &amp; Overhaul UI Popup): Corrected Workday Timeline calculations to prevent calculating worked duration up to 23:59:59 PM for past dates with missing checkouts, aligning it with database workedMinutes. Used zoned time parsing for check-in/out and break times to eliminate UTC-to-local timezone conversion offsets. Overhauled modal UI, increasing width to 760px, resolving overlaps, and stripping double card styles when displayed inside popups.</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B9" s="2" t="str">
+        <v>TSK-ATT-006</v>
+      </c>
+      <c r="C9" s="2" t="str">
+        <v>Fix Overtime Calculation in Attendance History Table</v>
+      </c>
+      <c r="D9" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E9" s="2" t="str">
+        <v>Resolved a discrepancy where the attendance history table displayed incorrect overtime durations for employees with late check-ins. Refactored the renderOvertime function in AttendancePage.tsx to dynamically factor in late check-in penalty minutes, ensuring the table matches the employee dashboard Workday Timeline exactly.</v>
+      </c>
+      <c r="F9" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-006 (Fix Overtime Calculation in Attendance History Table): Resolved a discrepancy where the attendance history table displayed incorrect overtime durations for employees with late check-ins. Refactored the renderOvertime function in AttendancePage.tsx to dynamically factor in late check-in penalty minutes, ensuring the table matches the employee dashboard Workday Timeline exactly.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W25"/>
+  <dimension ref="A1:W29"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -3186,9 +3206,293 @@
         <v>Successfully implemented and integrated check-in/out and break reminders, dynamic state-aware tray context menus, and custom slide-up notification alert cards. Additionally, developed a fully interactive, visible C# Desktop Dashboard mini-app window featuring a state-aware quick action panel, active workday/break timers, and a live telemetry activity log. Identified and fixed a timezone mismatch bug where the C# desktop agent's active shift/break timers subtracted local time from UTC time, resulting in incorrect negative elapsed times. Also optimized the desktop dashboard layout coordinates, enlarged button dimensions, removed space-heavy emojis from action controls, and configured high-DPI scaling mode (PerMonitorV2) in the project configuration to prevent text clipping and overlapping on high-resolution screens. Resolved the Hour 14 Evening Tea classification bug and added safety confirmation boxes to all break start/end actions across the dashboard, system tray menu, and slide-up reminder popups. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations. Re-compiled, updated the downloadable ZIP archive, and pushed the updates to the main branch. In addition, implemented the Points Dispute Tickets feature: added the PointsDisputeTicket model and status enum to the database schema, pushed it to sync the database, created the Express API endpoints (post dispute, fetch, resolve dispute with safe database transactions for points reversal and logs), added the inline dispute submission interface to the Leaderboard points history modal, and built a dedicated HR disputes queue tab for reviewing, approving, and rejecting disputes. Lastly, corrected the Workday Timeline calculation timezone bugs, fixed overtime calculations for past missing checkout entries, and expanded the modal popup layout with a wider flat style to avoid label overlaps.</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B26" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C26" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D26" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E26" s="2" t="str">
+        <v>Attendance Page</v>
+      </c>
+      <c r="F26" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G26" s="2" t="str">
+        <v>Overtime History Fix</v>
+      </c>
+      <c r="H26" s="2" t="str">
+        <v>TSK-ATT-006</v>
+      </c>
+      <c r="I26" s="2" t="str">
+        <v>Fix Overtime Calculation in Attendance History Table</v>
+      </c>
+      <c r="J26" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K26" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L26" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M26" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N26" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O26" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P26" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="R26" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S26" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T26" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U26" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="V26" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="W26" s="2" t="str">
+        <v>Identified and resolved a calculation bug in the attendance history table where overtime was computed using a hardcoded 9-hour workday threshold, completely ignoring late check-in penalty minutes. Factored in penaltyMinutes to compute dynamic required minutes (540 + penaltyMinutes) before calculating overtime, ensuring 100% mathematical consistency with the dashboard's Workday Timeline popup.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B27" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C27" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D27" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E27" s="2" t="str">
+        <v>Payroll Page</v>
+      </c>
+      <c r="F27" s="2" t="str">
+        <v>Payroll</v>
+      </c>
+      <c r="G27" s="2" t="str">
+        <v>Finalize Payroll</v>
+      </c>
+      <c r="H27" s="2" t="str">
+        <v>TSK-PAY-004</v>
+      </c>
+      <c r="I27" s="2" t="str">
+        <v>Implement Payroll finalization and publishing controls</v>
+      </c>
+      <c r="J27" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K27" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="L27" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M27" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N27" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O27" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P27" s="2">
+        <v>14</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="R27" s="2" t="str">
+        <v>30%</v>
+      </c>
+      <c r="S27" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T27" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U27" s="2" t="str">
+        <v>2026-06-23</v>
+      </c>
+      <c r="V27" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W27" s="2" t="str">
+        <v>Identified and resolved a calculation bug in the attendance history table where overtime was computed using a hardcoded 9-hour workday threshold, completely ignoring late check-in penalty minutes. Factored in penaltyMinutes to compute dynamic required minutes (540 + penaltyMinutes) before calculating overtime, ensuring 100% mathematical consistency with the dashboard's Workday Timeline popup.</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B28" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C28" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D28" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E28" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F28" s="2" t="str">
+        <v>Microsoft Teams Integration</v>
+      </c>
+      <c r="G28" s="2" t="str">
+        <v>Teams Webhook Alerts</v>
+      </c>
+      <c r="H28" s="2" t="str">
+        <v>TSK-TEAMS-001</v>
+      </c>
+      <c r="I28" s="2" t="str">
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+      </c>
+      <c r="J28" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K28" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="L28" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M28" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N28" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O28" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P28" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="R28" s="2" t="str">
+        <v>80%</v>
+      </c>
+      <c r="S28" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T28" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U28" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V28" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W28" s="2" t="str">
+        <v>Identified and resolved a calculation bug in the attendance history table where overtime was computed using a hardcoded 9-hour workday threshold, completely ignoring late check-in penalty minutes. Factored in penaltyMinutes to compute dynamic required minutes (540 + penaltyMinutes) before calculating overtime, ensuring 100% mathematical consistency with the dashboard's Workday Timeline popup.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B29" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C29" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D29" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E29" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F29" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G29" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H29" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I29" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J29" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K29" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L29" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M29" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N29" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O29" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P29" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q29" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="R29" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S29" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T29" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U29" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V29" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W29" s="2" t="str">
+        <v>Identified and resolved a calculation bug in the attendance history table where overtime was computed using a hardcoded 9-hour workday threshold, completely ignoring late check-in penalty minutes. Factored in penaltyMinutes to compute dynamic required minutes (540 + penaltyMinutes) before calculating overtime, ensuring 100% mathematical consistency with the dashboard's Workday Timeline popup.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Unify client/projects under The Star Prime (TSP) with dynamic UI controls and database migration
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1205,11 +1205,11 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="65.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="65.83203125" customWidth="1"/>
     <col min="6" max="6" width="65.83203125" customWidth="1"/>
@@ -1395,16 +1395,56 @@
         <v>* [COMPLETED] TSK-ATT-006 (Fix Overtime Calculation in Attendance History Table): Resolved a discrepancy where the attendance history table displayed incorrect overtime durations for employees with late check-ins. Refactored the renderOvertime function in AttendancePage.tsx to dynamically factor in late check-in penalty minutes, ensuring the table matches the employee dashboard Workday Timeline exactly.</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B10" s="2" t="str">
+        <v>TSK-ATT-007</v>
+      </c>
+      <c r="C10" s="2" t="str">
+        <v>Implement Net Worked Minutes and Crash-Aware Concluding Scheduler</v>
+      </c>
+      <c r="D10" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E10" s="2" t="str">
+        <v>Successfully implemented Net Worked Minutes (Option B) by deducting completed break durations from gross checked-in minutes across web checkout, regularization approval, and daily finalization. Rescheduled daily finalization cron job to 7:00 AM IST and implemented a crash-aware classification algorithm: it uses desktop agent activity logs to distinguish between clean OS shutdown without checkout (marked HALF_DAY as neglect penalty) and unexpected power cuts/system crashes (marked PRESENT without penalty). Replaced Events Logged in the frontend Day Summary panel with premium Uptime (since last break/away) and Active Penalties cards.</v>
+      </c>
+      <c r="F10" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-007 (Implement Net Worked Minutes and Crash-Aware Concluding Scheduler): Successfully implemented Net Worked Minutes (Option B) by deducting completed break durations from gross checked-in minutes across web checkout, regularization approval, and daily finalization. Rescheduled daily finalization cron job to 7:00 AM IST and implemented a crash-aware classification algorithm: it uses desktop agent activity logs to distinguish between clean OS shutdown without checkout (marked HALF_DAY as neglect penalty) and unexpected power cuts/system crashes (marked PRESENT without penalty). Replaced Events Logged in the frontend Day Summary panel with premium Uptime (since last break/away) and Active Penalties cards.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B11" s="2" t="str">
+        <v>TSK-TEAM-001</v>
+      </c>
+      <c r="C11" s="2" t="str">
+        <v>Unify Projects under The Star Prime (TSP)</v>
+      </c>
+      <c r="D11" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E11" s="2" t="str">
+        <v>Migrated all 48 Outlook email identities to 'The Star Prime' (TSP) client in the database, preserving all existing assignments. Cleaned up the old TUT and TEC client records. Consolidated the hardcoded magazines and industries into single TSP-owned lists in the Team workspace UI. Removed the client-switcher buttons and integrated inline delete (✕) controls with verification dialogs next to every project card, enabling dynamic addition and removal of projects for managers and team leads.</v>
+      </c>
+      <c r="F11" s="2" t="str">
+        <v>* [COMPLETED] TSK-TEAM-001 (Unify Projects under The Star Prime (TSP)): Migrated all 48 Outlook email identities to 'The Star Prime' (TSP) client in the database, preserving all existing assignments. Cleaned up the old TUT and TEC client records. Consolidated the hardcoded magazines and industries into single TSP-owned lists in the Team workspace UI. Removed the client-switcher buttons and integrated inline delete (✕) controls with verification dialogs next to every project card, enabling dynamic addition and removal of projects for managers and team leads.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W29"/>
+  <dimension ref="A1:W31"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -1412,7 +1452,7 @@
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="39.83203125" customWidth="1"/>
     <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="33.83203125" customWidth="1"/>
+    <col min="7" max="7" width="35.83203125" customWidth="1"/>
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
     <col min="9" max="9" width="65.83203125" customWidth="1"/>
     <col min="10" max="10" width="18.83203125" customWidth="1"/>
@@ -3256,7 +3296,7 @@
         <v>2</v>
       </c>
       <c r="Q26" s="2">
-        <v>0.5</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="R26" s="2" t="str">
         <v>100%</v>
@@ -3274,7 +3314,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W26" s="2" t="str">
-        <v>Identified and resolved a calculation bug in the attendance history table where overtime was computed using a hardcoded 9-hour workday threshold, completely ignoring late check-in penalty minutes. Factored in penaltyMinutes to compute dynamic required minutes (540 + penaltyMinutes) before calculating overtime, ensuring 100% mathematical consistency with the dashboard's Workday Timeline popup.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
       </c>
     </row>
     <row r="27">
@@ -3291,61 +3331,61 @@
         <v>Sprint 4</v>
       </c>
       <c r="E27" s="2" t="str">
-        <v>Payroll Page</v>
+        <v>Attendance Page</v>
       </c>
       <c r="F27" s="2" t="str">
-        <v>Payroll</v>
+        <v>Attendance</v>
       </c>
       <c r="G27" s="2" t="str">
-        <v>Finalize Payroll</v>
+        <v>Net Work &amp; Crash-Aware Scheduler</v>
       </c>
       <c r="H27" s="2" t="str">
-        <v>TSK-PAY-004</v>
+        <v>TSK-ATT-007</v>
       </c>
       <c r="I27" s="2" t="str">
-        <v>Implement Payroll finalization and publishing controls</v>
+        <v>Implement Net Worked Minutes and Crash-Aware Concluding Scheduler</v>
       </c>
       <c r="J27" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="K27" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="L27" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="M27" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="N27" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O27" s="2" t="str">
         <v>HIGH</v>
       </c>
       <c r="P27" s="2">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="Q27" s="2">
-        <v>0.5</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="R27" s="2" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="S27" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T27" s="2" t="str">
         <v>None</v>
       </c>
       <c r="U27" s="2" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-26</v>
       </c>
       <c r="V27" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-26</v>
       </c>
       <c r="W27" s="2" t="str">
-        <v>Identified and resolved a calculation bug in the attendance history table where overtime was computed using a hardcoded 9-hour workday threshold, completely ignoring late check-in penalty minutes. Factored in penaltyMinutes to compute dynamic required minutes (540 + penaltyMinutes) before calculating overtime, ensuring 100% mathematical consistency with the dashboard's Workday Timeline popup.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
       </c>
     </row>
     <row r="28">
@@ -3362,61 +3402,61 @@
         <v>Sprint 4</v>
       </c>
       <c r="E28" s="2" t="str">
+        <v>Team Page</v>
+      </c>
+      <c r="F28" s="2" t="str">
+        <v>Team Management</v>
+      </c>
+      <c r="G28" s="2" t="str">
+        <v>Ongoing Projects &amp; Clients</v>
+      </c>
+      <c r="H28" s="2" t="str">
+        <v>TSK-TEAM-001</v>
+      </c>
+      <c r="I28" s="2" t="str">
+        <v>Unify Projects under The Star Prime (TSP)</v>
+      </c>
+      <c r="J28" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K28" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L28" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="M28" s="2" t="str">
         <v>N/A</v>
       </c>
-      <c r="F28" s="2" t="str">
-        <v>Microsoft Teams Integration</v>
-      </c>
-      <c r="G28" s="2" t="str">
-        <v>Teams Webhook Alerts</v>
-      </c>
-      <c r="H28" s="2" t="str">
-        <v>TSK-TEAMS-001</v>
-      </c>
-      <c r="I28" s="2" t="str">
-        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
-      </c>
-      <c r="J28" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="K28" s="2" t="str">
-        <v>IN_PROGRESS</v>
-      </c>
-      <c r="L28" s="2" t="str">
-        <v>IN_PROGRESS</v>
-      </c>
-      <c r="M28" s="2" t="str">
-        <v>IN_PROGRESS</v>
-      </c>
       <c r="N28" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O28" s="2" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="P28" s="2">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="Q28" s="2">
-        <v>0.5</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="R28" s="2" t="str">
-        <v>80%</v>
+        <v>100%</v>
       </c>
       <c r="S28" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T28" s="2" t="str">
         <v>None</v>
       </c>
       <c r="U28" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-26</v>
       </c>
       <c r="V28" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-26</v>
       </c>
       <c r="W28" s="2" t="str">
-        <v>Identified and resolved a calculation bug in the attendance history table where overtime was computed using a hardcoded 9-hour workday threshold, completely ignoring late check-in penalty minutes. Factored in penaltyMinutes to compute dynamic required minutes (540 + penaltyMinutes) before calculating overtime, ensuring 100% mathematical consistency with the dashboard's Workday Timeline popup.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
       </c>
     </row>
     <row r="29">
@@ -3433,25 +3473,25 @@
         <v>Sprint 4</v>
       </c>
       <c r="E29" s="2" t="str">
-        <v>Dashboard &amp; Navbar</v>
+        <v>Payroll Page</v>
       </c>
       <c r="F29" s="2" t="str">
-        <v>Role Dashboards &amp; Analytics</v>
+        <v>Payroll</v>
       </c>
       <c r="G29" s="2" t="str">
-        <v>Performance Tuning</v>
+        <v>Finalize Payroll</v>
       </c>
       <c r="H29" s="2" t="str">
-        <v>TSK-PERF-001</v>
+        <v>TSK-PAY-004</v>
       </c>
       <c r="I29" s="2" t="str">
-        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+        <v>Implement Payroll finalization and publishing controls</v>
       </c>
       <c r="J29" s="2" t="str">
         <v>IN_PROGRESS</v>
       </c>
       <c r="K29" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="L29" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3466,13 +3506,13 @@
         <v>HIGH</v>
       </c>
       <c r="P29" s="2">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="Q29" s="2">
-        <v>0.5</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="R29" s="2" t="str">
-        <v>50%</v>
+        <v>30%</v>
       </c>
       <c r="S29" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3481,18 +3521,160 @@
         <v>None</v>
       </c>
       <c r="U29" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-23</v>
       </c>
       <c r="V29" s="2" t="str">
         <v>2026-06-24</v>
       </c>
       <c r="W29" s="2" t="str">
-        <v>Identified and resolved a calculation bug in the attendance history table where overtime was computed using a hardcoded 9-hour workday threshold, completely ignoring late check-in penalty minutes. Factored in penaltyMinutes to compute dynamic required minutes (540 + penaltyMinutes) before calculating overtime, ensuring 100% mathematical consistency with the dashboard's Workday Timeline popup.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B30" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C30" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D30" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E30" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F30" s="2" t="str">
+        <v>Microsoft Teams Integration</v>
+      </c>
+      <c r="G30" s="2" t="str">
+        <v>Teams Webhook Alerts</v>
+      </c>
+      <c r="H30" s="2" t="str">
+        <v>TSK-TEAMS-001</v>
+      </c>
+      <c r="I30" s="2" t="str">
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+      </c>
+      <c r="J30" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K30" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="L30" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M30" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N30" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O30" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P30" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>1.3333333333333333</v>
+      </c>
+      <c r="R30" s="2" t="str">
+        <v>80%</v>
+      </c>
+      <c r="S30" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T30" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U30" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V30" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W30" s="2" t="str">
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B31" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C31" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D31" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E31" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F31" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G31" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H31" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I31" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J31" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K31" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L31" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M31" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N31" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O31" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P31" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q31" s="2">
+        <v>1.3333333333333333</v>
+      </c>
+      <c r="R31" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S31" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T31" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U31" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V31" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W31" s="2" t="str">
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Implement Dual-View Task Console for managers and team leads with dynamic tab switcher
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1205,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1435,16 +1435,36 @@
         <v>* [COMPLETED] TSK-TEAM-001 (Unify Projects under The Star Prime (TSP)): Migrated all 48 Outlook email identities to 'The Star Prime' (TSP) client in the database, preserving all existing assignments. Cleaned up the old TUT and TEC client records. Consolidated the hardcoded magazines and industries into single TSP-owned lists in the Team workspace UI. Removed the client-switcher buttons and integrated inline delete (✕) controls with verification dialogs next to every project card, enabling dynamic addition and removal of projects for managers and team leads.</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B12" s="2" t="str">
+        <v>TSK-TASK-001</v>
+      </c>
+      <c r="C12" s="2" t="str">
+        <v>Implement Dual-View Task Console for Managers and Team Leads</v>
+      </c>
+      <c r="D12" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E12" s="2" t="str">
+        <v>Developed a unified Dual-View Task Console for managers, team leads, admin, and HR. Fetches both personal assigned tasks and manager assigned tasks concurrently. Integrated a premium tab switcher ('Tasks Assigned to Me' vs 'Tasks Assigned to Others') with custom icons and stats, and overhauled the card layout to display creator/assigner metadata (e.g. 'Assigned by: Swapnil Deshmukh (Manager)') for received tasks.</v>
+      </c>
+      <c r="F12" s="2" t="str">
+        <v>* [COMPLETED] TSK-TASK-001 (Implement Dual-View Task Console for Managers and Team Leads): Developed a unified Dual-View Task Console for managers, team leads, admin, and HR. Fetches both personal assigned tasks and manager assigned tasks concurrently. Integrated a premium tab switcher ('Tasks Assigned to Me' vs 'Tasks Assigned to Others') with custom icons and stats, and overhauled the card layout to display creator/assigner metadata (e.g. 'Assigned by: Swapnil Deshmukh (Manager)') for received tasks.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W31"/>
+  <dimension ref="A1:W32"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -3296,7 +3316,7 @@
         <v>2</v>
       </c>
       <c r="Q26" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R26" s="2" t="str">
         <v>100%</v>
@@ -3314,7 +3334,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W26" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
       </c>
     </row>
     <row r="27">
@@ -3367,7 +3387,7 @@
         <v>8</v>
       </c>
       <c r="Q27" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R27" s="2" t="str">
         <v>100%</v>
@@ -3385,7 +3405,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W27" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
       </c>
     </row>
     <row r="28">
@@ -3438,7 +3458,7 @@
         <v>4</v>
       </c>
       <c r="Q28" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R28" s="2" t="str">
         <v>100%</v>
@@ -3456,7 +3476,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W28" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
       </c>
     </row>
     <row r="29">
@@ -3473,61 +3493,61 @@
         <v>Sprint 4</v>
       </c>
       <c r="E29" s="2" t="str">
-        <v>Payroll Page</v>
+        <v>Manage Tasks Page</v>
       </c>
       <c r="F29" s="2" t="str">
-        <v>Payroll</v>
+        <v>Task Management</v>
       </c>
       <c r="G29" s="2" t="str">
-        <v>Finalize Payroll</v>
+        <v>Dual-View Task Console</v>
       </c>
       <c r="H29" s="2" t="str">
-        <v>TSK-PAY-004</v>
+        <v>TSK-TASK-001</v>
       </c>
       <c r="I29" s="2" t="str">
-        <v>Implement Payroll finalization and publishing controls</v>
+        <v>Implement Dual-View Task Console for Managers and Team Leads</v>
       </c>
       <c r="J29" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="K29" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="L29" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="M29" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="N29" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O29" s="2" t="str">
         <v>HIGH</v>
       </c>
       <c r="P29" s="2">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="Q29" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R29" s="2" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="S29" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T29" s="2" t="str">
         <v>None</v>
       </c>
       <c r="U29" s="2" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-26</v>
       </c>
       <c r="V29" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-26</v>
       </c>
       <c r="W29" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
       </c>
     </row>
     <row r="30">
@@ -3544,22 +3564,22 @@
         <v>Sprint 4</v>
       </c>
       <c r="E30" s="2" t="str">
-        <v>N/A</v>
+        <v>Payroll Page</v>
       </c>
       <c r="F30" s="2" t="str">
-        <v>Microsoft Teams Integration</v>
+        <v>Payroll</v>
       </c>
       <c r="G30" s="2" t="str">
-        <v>Teams Webhook Alerts</v>
+        <v>Finalize Payroll</v>
       </c>
       <c r="H30" s="2" t="str">
-        <v>TSK-TEAMS-001</v>
+        <v>TSK-PAY-004</v>
       </c>
       <c r="I30" s="2" t="str">
-        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+        <v>Implement Payroll finalization and publishing controls</v>
       </c>
       <c r="J30" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="K30" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3574,16 +3594,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O30" s="2" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="P30" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q30" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R30" s="2" t="str">
-        <v>80%</v>
+        <v>30%</v>
       </c>
       <c r="S30" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3592,13 +3612,13 @@
         <v>None</v>
       </c>
       <c r="U30" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-23</v>
       </c>
       <c r="V30" s="2" t="str">
         <v>2026-06-24</v>
       </c>
       <c r="W30" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
       </c>
     </row>
     <row r="31">
@@ -3615,25 +3635,25 @@
         <v>Sprint 4</v>
       </c>
       <c r="E31" s="2" t="str">
-        <v>Dashboard &amp; Navbar</v>
+        <v>N/A</v>
       </c>
       <c r="F31" s="2" t="str">
-        <v>Role Dashboards &amp; Analytics</v>
+        <v>Microsoft Teams Integration</v>
       </c>
       <c r="G31" s="2" t="str">
-        <v>Performance Tuning</v>
+        <v>Teams Webhook Alerts</v>
       </c>
       <c r="H31" s="2" t="str">
-        <v>TSK-PERF-001</v>
+        <v>TSK-TEAMS-001</v>
       </c>
       <c r="I31" s="2" t="str">
-        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
       </c>
       <c r="J31" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="K31" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="L31" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3645,16 +3665,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O31" s="2" t="str">
-        <v>HIGH</v>
+        <v>MEDIUM</v>
       </c>
       <c r="P31" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q31" s="2">
-        <v>1.3333333333333333</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="R31" s="2" t="str">
-        <v>50%</v>
+        <v>80%</v>
       </c>
       <c r="S31" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3669,12 +3689,83 @@
         <v>2026-06-24</v>
       </c>
       <c r="W31" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B32" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C32" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D32" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E32" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F32" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G32" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H32" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I32" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J32" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K32" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L32" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M32" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N32" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O32" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P32" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q32" s="2">
+        <v>1.1428571428571428</v>
+      </c>
+      <c r="R32" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S32" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T32" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U32" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V32" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W32" s="2" t="str">
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W32"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(attendance): fix AWAY status logic by querying active web break sessions and syncing frontend state instantly
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1205,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1455,16 +1455,36 @@
         <v>* [COMPLETED] TSK-TASK-001 (Implement Dual-View Task Console for Managers and Team Leads): Developed a unified Dual-View Task Console for managers, team leads, admin, and HR. Fetches both personal assigned tasks and manager assigned tasks concurrently. Integrated a premium tab switcher ('Tasks Assigned to Me' vs 'Tasks Assigned to Others') with custom icons and stats, and overhauled the card layout to display creator/assigner metadata (e.g. 'Assigned by: Swapnil Deshmukh (Manager)') for received tasks.</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B13" s="2" t="str">
+        <v>TSK-ATT-008</v>
+      </c>
+      <c r="C13" s="2" t="str">
+        <v>Fix Web Break Session AWAY Status Telemetry</v>
+      </c>
+      <c r="D13" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E13" s="2" t="str">
+        <v>Resolved a major telemetry tracking issue where checked-in employees on active web-initiated breaks remained stuck as ACTIVE. Modified the /live-status backend query to select BreakSession records where endTime is null, setting user status to AWAY if an active break session is present. Implemented a break-updated global event listener in the frontend AppProvider to instantly synchronize and refresh local status dots in the Navbar and Sidebar upon starting or ending breaks.</v>
+      </c>
+      <c r="F13" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-008 (Fix Web Break Session AWAY Status Telemetry): Resolved a major telemetry tracking issue where checked-in employees on active web-initiated breaks remained stuck as ACTIVE. Modified the /live-status backend query to select BreakSession records where endTime is null, setting user status to AWAY if an active break session is present. Implemented a break-updated global event listener in the frontend AppProvider to instantly synchronize and refresh local status dots in the Navbar and Sidebar upon starting or ending breaks.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W32"/>
+  <dimension ref="A1:W33"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -3316,7 +3336,7 @@
         <v>2</v>
       </c>
       <c r="Q26" s="2">
-        <v>1.1428571428571428</v>
+        <v>1</v>
       </c>
       <c r="R26" s="2" t="str">
         <v>100%</v>
@@ -3334,7 +3354,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W26" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
       </c>
     </row>
     <row r="27">
@@ -3387,7 +3407,7 @@
         <v>8</v>
       </c>
       <c r="Q27" s="2">
-        <v>1.1428571428571428</v>
+        <v>1</v>
       </c>
       <c r="R27" s="2" t="str">
         <v>100%</v>
@@ -3405,7 +3425,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W27" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
       </c>
     </row>
     <row r="28">
@@ -3458,7 +3478,7 @@
         <v>4</v>
       </c>
       <c r="Q28" s="2">
-        <v>1.1428571428571428</v>
+        <v>1</v>
       </c>
       <c r="R28" s="2" t="str">
         <v>100%</v>
@@ -3476,7 +3496,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W28" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
       </c>
     </row>
     <row r="29">
@@ -3529,7 +3549,7 @@
         <v>6</v>
       </c>
       <c r="Q29" s="2">
-        <v>1.1428571428571428</v>
+        <v>1</v>
       </c>
       <c r="R29" s="2" t="str">
         <v>100%</v>
@@ -3547,7 +3567,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W29" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
       </c>
     </row>
     <row r="30">
@@ -3564,61 +3584,61 @@
         <v>Sprint 4</v>
       </c>
       <c r="E30" s="2" t="str">
-        <v>Payroll Page</v>
+        <v>Attendance Page</v>
       </c>
       <c r="F30" s="2" t="str">
-        <v>Payroll</v>
+        <v>Attendance</v>
       </c>
       <c r="G30" s="2" t="str">
-        <v>Finalize Payroll</v>
+        <v>Live Status Telemetry</v>
       </c>
       <c r="H30" s="2" t="str">
-        <v>TSK-PAY-004</v>
+        <v>TSK-ATT-008</v>
       </c>
       <c r="I30" s="2" t="str">
-        <v>Implement Payroll finalization and publishing controls</v>
+        <v>Fix Web Break Session AWAY Status Telemetry</v>
       </c>
       <c r="J30" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="K30" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="L30" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="M30" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="N30" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O30" s="2" t="str">
         <v>HIGH</v>
       </c>
       <c r="P30" s="2">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="Q30" s="2">
-        <v>1.1428571428571428</v>
+        <v>1</v>
       </c>
       <c r="R30" s="2" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="S30" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T30" s="2" t="str">
         <v>None</v>
       </c>
       <c r="U30" s="2" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-26</v>
       </c>
       <c r="V30" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-26</v>
       </c>
       <c r="W30" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
       </c>
     </row>
     <row r="31">
@@ -3635,22 +3655,22 @@
         <v>Sprint 4</v>
       </c>
       <c r="E31" s="2" t="str">
-        <v>N/A</v>
+        <v>Payroll Page</v>
       </c>
       <c r="F31" s="2" t="str">
-        <v>Microsoft Teams Integration</v>
+        <v>Payroll</v>
       </c>
       <c r="G31" s="2" t="str">
-        <v>Teams Webhook Alerts</v>
+        <v>Finalize Payroll</v>
       </c>
       <c r="H31" s="2" t="str">
-        <v>TSK-TEAMS-001</v>
+        <v>TSK-PAY-004</v>
       </c>
       <c r="I31" s="2" t="str">
-        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+        <v>Implement Payroll finalization and publishing controls</v>
       </c>
       <c r="J31" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="K31" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3665,16 +3685,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O31" s="2" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="P31" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q31" s="2">
-        <v>1.1428571428571428</v>
+        <v>1</v>
       </c>
       <c r="R31" s="2" t="str">
-        <v>80%</v>
+        <v>30%</v>
       </c>
       <c r="S31" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3683,13 +3703,13 @@
         <v>None</v>
       </c>
       <c r="U31" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-23</v>
       </c>
       <c r="V31" s="2" t="str">
         <v>2026-06-24</v>
       </c>
       <c r="W31" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
       </c>
     </row>
     <row r="32">
@@ -3706,25 +3726,25 @@
         <v>Sprint 4</v>
       </c>
       <c r="E32" s="2" t="str">
-        <v>Dashboard &amp; Navbar</v>
+        <v>N/A</v>
       </c>
       <c r="F32" s="2" t="str">
-        <v>Role Dashboards &amp; Analytics</v>
+        <v>Microsoft Teams Integration</v>
       </c>
       <c r="G32" s="2" t="str">
-        <v>Performance Tuning</v>
+        <v>Teams Webhook Alerts</v>
       </c>
       <c r="H32" s="2" t="str">
-        <v>TSK-PERF-001</v>
+        <v>TSK-TEAMS-001</v>
       </c>
       <c r="I32" s="2" t="str">
-        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
       </c>
       <c r="J32" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="K32" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="L32" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3736,16 +3756,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O32" s="2" t="str">
-        <v>HIGH</v>
+        <v>MEDIUM</v>
       </c>
       <c r="P32" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q32" s="2">
-        <v>1.1428571428571428</v>
+        <v>1</v>
       </c>
       <c r="R32" s="2" t="str">
-        <v>50%</v>
+        <v>80%</v>
       </c>
       <c r="S32" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3760,12 +3780,83 @@
         <v>2026-06-24</v>
       </c>
       <c r="W32" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B33" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C33" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D33" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E33" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F33" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G33" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H33" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I33" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J33" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K33" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L33" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M33" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N33" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O33" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P33" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q33" s="2">
+        <v>1</v>
+      </c>
+      <c r="R33" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S33" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T33" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U33" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V33" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W33" s="2" t="str">
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W33"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(attendance): implement paid overtime pre-approval workflow and project tracking sync
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1205,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1475,16 +1475,36 @@
         <v>* [COMPLETED] TSK-ATT-008 (Fix Web Break Session AWAY Status Telemetry): Resolved a major telemetry tracking issue where checked-in employees on active web-initiated breaks remained stuck as ACTIVE. Modified the /live-status backend query to select BreakSession records where endTime is null, setting user status to AWAY if an active break session is present. Implemented a break-updated global event listener in the frontend AppProvider to instantly synchronize and refresh local status dots in the Navbar and Sidebar upon starting or ending breaks.</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B14" s="2" t="str">
+        <v>TSK-ATT-009</v>
+      </c>
+      <c r="C14" s="2" t="str">
+        <v>Implement Paid Overtime Pre-Approval Workflow and Paid Tags</v>
+      </c>
+      <c r="D14" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E14" s="2" t="str">
+        <v>Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days (with full calendar-exception check) by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+      </c>
+      <c r="F14" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-009 (Implement Paid Overtime Pre-Approval Workflow and Paid Tags): Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days (with full calendar-exception check) by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W33"/>
+  <dimension ref="A1:W34"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -1492,7 +1512,7 @@
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="39.83203125" customWidth="1"/>
     <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="35.83203125" customWidth="1"/>
+    <col min="7" max="7" width="38.83203125" customWidth="1"/>
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
     <col min="9" max="9" width="65.83203125" customWidth="1"/>
     <col min="10" max="10" width="18.83203125" customWidth="1"/>
@@ -3336,7 +3356,7 @@
         <v>2</v>
       </c>
       <c r="Q26" s="2">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="R26" s="2" t="str">
         <v>100%</v>
@@ -3354,7 +3374,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W26" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
       </c>
     </row>
     <row r="27">
@@ -3407,7 +3427,7 @@
         <v>8</v>
       </c>
       <c r="Q27" s="2">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="R27" s="2" t="str">
         <v>100%</v>
@@ -3425,7 +3445,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W27" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
       </c>
     </row>
     <row r="28">
@@ -3478,7 +3498,7 @@
         <v>4</v>
       </c>
       <c r="Q28" s="2">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="R28" s="2" t="str">
         <v>100%</v>
@@ -3496,7 +3516,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W28" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
       </c>
     </row>
     <row r="29">
@@ -3549,7 +3569,7 @@
         <v>6</v>
       </c>
       <c r="Q29" s="2">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="R29" s="2" t="str">
         <v>100%</v>
@@ -3567,7 +3587,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W29" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
       </c>
     </row>
     <row r="30">
@@ -3620,7 +3640,7 @@
         <v>4</v>
       </c>
       <c r="Q30" s="2">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="R30" s="2" t="str">
         <v>100%</v>
@@ -3638,7 +3658,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W30" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
       </c>
     </row>
     <row r="31">
@@ -3655,61 +3675,61 @@
         <v>Sprint 4</v>
       </c>
       <c r="E31" s="2" t="str">
-        <v>Payroll Page</v>
+        <v>Attendance Page</v>
       </c>
       <c r="F31" s="2" t="str">
-        <v>Payroll</v>
+        <v>Attendance</v>
       </c>
       <c r="G31" s="2" t="str">
-        <v>Finalize Payroll</v>
+        <v>Paid Overtime Pre-Approval Workflow</v>
       </c>
       <c r="H31" s="2" t="str">
-        <v>TSK-PAY-004</v>
+        <v>TSK-ATT-009</v>
       </c>
       <c r="I31" s="2" t="str">
-        <v>Implement Payroll finalization and publishing controls</v>
+        <v>Implement Paid Overtime Pre-Approval Workflow and Paid Tags</v>
       </c>
       <c r="J31" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="K31" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="L31" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="M31" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="N31" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O31" s="2" t="str">
         <v>HIGH</v>
       </c>
       <c r="P31" s="2">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="Q31" s="2">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="R31" s="2" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="S31" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T31" s="2" t="str">
         <v>None</v>
       </c>
       <c r="U31" s="2" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-26</v>
       </c>
       <c r="V31" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-26</v>
       </c>
       <c r="W31" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
       </c>
     </row>
     <row r="32">
@@ -3726,22 +3746,22 @@
         <v>Sprint 4</v>
       </c>
       <c r="E32" s="2" t="str">
-        <v>N/A</v>
+        <v>Payroll Page</v>
       </c>
       <c r="F32" s="2" t="str">
-        <v>Microsoft Teams Integration</v>
+        <v>Payroll</v>
       </c>
       <c r="G32" s="2" t="str">
-        <v>Teams Webhook Alerts</v>
+        <v>Finalize Payroll</v>
       </c>
       <c r="H32" s="2" t="str">
-        <v>TSK-TEAMS-001</v>
+        <v>TSK-PAY-004</v>
       </c>
       <c r="I32" s="2" t="str">
-        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+        <v>Implement Payroll finalization and publishing controls</v>
       </c>
       <c r="J32" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="K32" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3756,16 +3776,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O32" s="2" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="P32" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q32" s="2">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="R32" s="2" t="str">
-        <v>80%</v>
+        <v>30%</v>
       </c>
       <c r="S32" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3774,13 +3794,13 @@
         <v>None</v>
       </c>
       <c r="U32" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-23</v>
       </c>
       <c r="V32" s="2" t="str">
         <v>2026-06-24</v>
       </c>
       <c r="W32" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
       </c>
     </row>
     <row r="33">
@@ -3797,25 +3817,25 @@
         <v>Sprint 4</v>
       </c>
       <c r="E33" s="2" t="str">
-        <v>Dashboard &amp; Navbar</v>
+        <v>N/A</v>
       </c>
       <c r="F33" s="2" t="str">
-        <v>Role Dashboards &amp; Analytics</v>
+        <v>Microsoft Teams Integration</v>
       </c>
       <c r="G33" s="2" t="str">
-        <v>Performance Tuning</v>
+        <v>Teams Webhook Alerts</v>
       </c>
       <c r="H33" s="2" t="str">
-        <v>TSK-PERF-001</v>
+        <v>TSK-TEAMS-001</v>
       </c>
       <c r="I33" s="2" t="str">
-        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
       </c>
       <c r="J33" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="K33" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="L33" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3827,16 +3847,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O33" s="2" t="str">
-        <v>HIGH</v>
+        <v>MEDIUM</v>
       </c>
       <c r="P33" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q33" s="2">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="R33" s="2" t="str">
-        <v>50%</v>
+        <v>80%</v>
       </c>
       <c r="S33" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3851,12 +3871,83 @@
         <v>2026-06-24</v>
       </c>
       <c r="W33" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B34" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C34" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D34" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E34" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F34" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G34" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H34" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I34" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J34" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K34" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L34" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M34" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N34" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O34" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P34" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q34" s="2">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="R34" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S34" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T34" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U34" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V34" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W34" s="2" t="str">
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W34"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(attendance): add early checkout and app logout shift concluding warnings
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1205,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1495,16 +1495,36 @@
         <v>* [COMPLETED] TSK-ATT-009 (Implement Paid Overtime Pre-Approval Workflow and Paid Tags): Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days (with full calendar-exception check) by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B15" s="2" t="str">
+        <v>TSK-ATT-010</v>
+      </c>
+      <c r="C15" s="2" t="str">
+        <v>Implement Incomplete Shift Hours Warning on Checkout and Logout</v>
+      </c>
+      <c r="D15" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E15" s="2" t="str">
+        <v>Designed and implemented proactive warnings for employees who attempt to check out of their shift or log out of the application before completing their required working hours (9 hours + late penalties). Rendered a prominent, high-visibility red warning banner at the top of the Checkout Modal detailing their shift requirements and remaining time. Integrated a similar warning into the browser confirmation alert when clicking the application logout button in the topbar, ensuring zero gaps in compliance and attendance tracking.</v>
+      </c>
+      <c r="F15" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-010 (Implement Incomplete Shift Hours Warning on Checkout and Logout): Designed and implemented proactive warnings for employees who attempt to check out of their shift or log out of the application before completing their required working hours (9 hours + late penalties). Rendered a prominent, high-visibility red warning banner at the top of the Checkout Modal detailing their shift requirements and remaining time. Integrated a similar warning into the browser confirmation alert when clicking the application logout button in the topbar, ensuring zero gaps in compliance and attendance tracking.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W34"/>
+  <dimension ref="A1:W35"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -3356,7 +3376,7 @@
         <v>2</v>
       </c>
       <c r="Q26" s="2">
-        <v>0.8888888888888888</v>
+        <v>0.8</v>
       </c>
       <c r="R26" s="2" t="str">
         <v>100%</v>
@@ -3374,7 +3394,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W26" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
       </c>
     </row>
     <row r="27">
@@ -3427,7 +3447,7 @@
         <v>8</v>
       </c>
       <c r="Q27" s="2">
-        <v>0.8888888888888888</v>
+        <v>0.8</v>
       </c>
       <c r="R27" s="2" t="str">
         <v>100%</v>
@@ -3445,7 +3465,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W27" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
       </c>
     </row>
     <row r="28">
@@ -3498,7 +3518,7 @@
         <v>4</v>
       </c>
       <c r="Q28" s="2">
-        <v>0.8888888888888888</v>
+        <v>0.8</v>
       </c>
       <c r="R28" s="2" t="str">
         <v>100%</v>
@@ -3516,7 +3536,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W28" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
       </c>
     </row>
     <row r="29">
@@ -3569,7 +3589,7 @@
         <v>6</v>
       </c>
       <c r="Q29" s="2">
-        <v>0.8888888888888888</v>
+        <v>0.8</v>
       </c>
       <c r="R29" s="2" t="str">
         <v>100%</v>
@@ -3587,7 +3607,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W29" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
       </c>
     </row>
     <row r="30">
@@ -3640,7 +3660,7 @@
         <v>4</v>
       </c>
       <c r="Q30" s="2">
-        <v>0.8888888888888888</v>
+        <v>0.8</v>
       </c>
       <c r="R30" s="2" t="str">
         <v>100%</v>
@@ -3658,7 +3678,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W30" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
       </c>
     </row>
     <row r="31">
@@ -3711,7 +3731,7 @@
         <v>8</v>
       </c>
       <c r="Q31" s="2">
-        <v>0.8888888888888888</v>
+        <v>0.8</v>
       </c>
       <c r="R31" s="2" t="str">
         <v>100%</v>
@@ -3729,7 +3749,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W31" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
       </c>
     </row>
     <row r="32">
@@ -3746,61 +3766,61 @@
         <v>Sprint 4</v>
       </c>
       <c r="E32" s="2" t="str">
-        <v>Payroll Page</v>
+        <v>Navbar &amp; Attendance Quick Action</v>
       </c>
       <c r="F32" s="2" t="str">
-        <v>Payroll</v>
+        <v>Attendance</v>
       </c>
       <c r="G32" s="2" t="str">
-        <v>Finalize Payroll</v>
+        <v>Shift Concluding Warning</v>
       </c>
       <c r="H32" s="2" t="str">
-        <v>TSK-PAY-004</v>
+        <v>TSK-ATT-010</v>
       </c>
       <c r="I32" s="2" t="str">
-        <v>Implement Payroll finalization and publishing controls</v>
+        <v>Implement Incomplete Shift Hours Warning on Checkout and Logout</v>
       </c>
       <c r="J32" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="K32" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="L32" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="M32" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="N32" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O32" s="2" t="str">
         <v>HIGH</v>
       </c>
       <c r="P32" s="2">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="Q32" s="2">
-        <v>0.8888888888888888</v>
+        <v>0.8</v>
       </c>
       <c r="R32" s="2" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="S32" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T32" s="2" t="str">
         <v>None</v>
       </c>
       <c r="U32" s="2" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-26</v>
       </c>
       <c r="V32" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-26</v>
       </c>
       <c r="W32" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
       </c>
     </row>
     <row r="33">
@@ -3817,22 +3837,22 @@
         <v>Sprint 4</v>
       </c>
       <c r="E33" s="2" t="str">
-        <v>N/A</v>
+        <v>Payroll Page</v>
       </c>
       <c r="F33" s="2" t="str">
-        <v>Microsoft Teams Integration</v>
+        <v>Payroll</v>
       </c>
       <c r="G33" s="2" t="str">
-        <v>Teams Webhook Alerts</v>
+        <v>Finalize Payroll</v>
       </c>
       <c r="H33" s="2" t="str">
-        <v>TSK-TEAMS-001</v>
+        <v>TSK-PAY-004</v>
       </c>
       <c r="I33" s="2" t="str">
-        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+        <v>Implement Payroll finalization and publishing controls</v>
       </c>
       <c r="J33" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="K33" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3847,16 +3867,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O33" s="2" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="P33" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q33" s="2">
-        <v>0.8888888888888888</v>
+        <v>0.8</v>
       </c>
       <c r="R33" s="2" t="str">
-        <v>80%</v>
+        <v>30%</v>
       </c>
       <c r="S33" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3865,13 +3885,13 @@
         <v>None</v>
       </c>
       <c r="U33" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-23</v>
       </c>
       <c r="V33" s="2" t="str">
         <v>2026-06-24</v>
       </c>
       <c r="W33" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
       </c>
     </row>
     <row r="34">
@@ -3888,25 +3908,25 @@
         <v>Sprint 4</v>
       </c>
       <c r="E34" s="2" t="str">
-        <v>Dashboard &amp; Navbar</v>
+        <v>N/A</v>
       </c>
       <c r="F34" s="2" t="str">
-        <v>Role Dashboards &amp; Analytics</v>
+        <v>Microsoft Teams Integration</v>
       </c>
       <c r="G34" s="2" t="str">
-        <v>Performance Tuning</v>
+        <v>Teams Webhook Alerts</v>
       </c>
       <c r="H34" s="2" t="str">
-        <v>TSK-PERF-001</v>
+        <v>TSK-TEAMS-001</v>
       </c>
       <c r="I34" s="2" t="str">
-        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
       </c>
       <c r="J34" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="K34" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="L34" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3918,16 +3938,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O34" s="2" t="str">
-        <v>HIGH</v>
+        <v>MEDIUM</v>
       </c>
       <c r="P34" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q34" s="2">
-        <v>0.8888888888888888</v>
+        <v>0.8</v>
       </c>
       <c r="R34" s="2" t="str">
-        <v>50%</v>
+        <v>80%</v>
       </c>
       <c r="S34" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3942,12 +3962,83 @@
         <v>2026-06-24</v>
       </c>
       <c r="W34" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Finally, designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B35" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C35" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D35" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E35" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F35" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G35" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H35" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I35" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J35" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K35" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L35" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M35" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N35" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O35" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P35" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q35" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="R35" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S35" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T35" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U35" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V35" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W35" s="2" t="str">
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W35"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Implement Dynamic Shift Management System (Admin Only) and refactor attendance calculations to be shift-aware
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1205,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1515,16 +1515,36 @@
         <v>* [COMPLETED] TSK-ATT-010 (Implement Incomplete Shift Hours Warning on Checkout and Logout): Designed and implemented proactive warnings for employees who attempt to check out of their shift or log out of the application before completing their required working hours (9 hours + late penalties). Rendered a prominent, high-visibility red warning banner at the top of the Checkout Modal detailing their shift requirements and remaining time. Integrated a similar warning into the browser confirmation alert when clicking the application logout button in the topbar, ensuring zero gaps in compliance and attendance tracking.</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B16" s="2" t="str">
+        <v>TSK-ATT-011</v>
+      </c>
+      <c r="C16" s="2" t="str">
+        <v>Implement Dynamic Shift Management System</v>
+      </c>
+      <c r="D16" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E16" s="2" t="str">
+        <v>Designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+      </c>
+      <c r="F16" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-011 (Implement Dynamic Shift Management System): Designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W35"/>
+  <dimension ref="A1:W36"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -3376,7 +3396,7 @@
         <v>2</v>
       </c>
       <c r="Q26" s="2">
-        <v>0.8</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="R26" s="2" t="str">
         <v>100%</v>
@@ -3394,7 +3414,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W26" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
       </c>
     </row>
     <row r="27">
@@ -3447,7 +3467,7 @@
         <v>8</v>
       </c>
       <c r="Q27" s="2">
-        <v>0.8</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="R27" s="2" t="str">
         <v>100%</v>
@@ -3465,7 +3485,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W27" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
       </c>
     </row>
     <row r="28">
@@ -3518,7 +3538,7 @@
         <v>4</v>
       </c>
       <c r="Q28" s="2">
-        <v>0.8</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="R28" s="2" t="str">
         <v>100%</v>
@@ -3536,7 +3556,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W28" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
       </c>
     </row>
     <row r="29">
@@ -3589,7 +3609,7 @@
         <v>6</v>
       </c>
       <c r="Q29" s="2">
-        <v>0.8</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="R29" s="2" t="str">
         <v>100%</v>
@@ -3607,7 +3627,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W29" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
       </c>
     </row>
     <row r="30">
@@ -3660,7 +3680,7 @@
         <v>4</v>
       </c>
       <c r="Q30" s="2">
-        <v>0.8</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="R30" s="2" t="str">
         <v>100%</v>
@@ -3678,7 +3698,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W30" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
       </c>
     </row>
     <row r="31">
@@ -3731,7 +3751,7 @@
         <v>8</v>
       </c>
       <c r="Q31" s="2">
-        <v>0.8</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="R31" s="2" t="str">
         <v>100%</v>
@@ -3749,7 +3769,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W31" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
       </c>
     </row>
     <row r="32">
@@ -3802,7 +3822,7 @@
         <v>4</v>
       </c>
       <c r="Q32" s="2">
-        <v>0.8</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="R32" s="2" t="str">
         <v>100%</v>
@@ -3820,7 +3840,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W32" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
       </c>
     </row>
     <row r="33">
@@ -3837,61 +3857,61 @@
         <v>Sprint 4</v>
       </c>
       <c r="E33" s="2" t="str">
-        <v>Payroll Page</v>
+        <v>Shift Management Page</v>
       </c>
       <c r="F33" s="2" t="str">
-        <v>Payroll</v>
+        <v>Attendance</v>
       </c>
       <c r="G33" s="2" t="str">
-        <v>Finalize Payroll</v>
+        <v>Dynamic Shift Management</v>
       </c>
       <c r="H33" s="2" t="str">
-        <v>TSK-PAY-004</v>
+        <v>TSK-ATT-011</v>
       </c>
       <c r="I33" s="2" t="str">
-        <v>Implement Payroll finalization and publishing controls</v>
+        <v>Implement Dynamic Shift Management System</v>
       </c>
       <c r="J33" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="K33" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="L33" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="M33" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="N33" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O33" s="2" t="str">
         <v>HIGH</v>
       </c>
       <c r="P33" s="2">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="Q33" s="2">
-        <v>0.8</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="R33" s="2" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="S33" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T33" s="2" t="str">
         <v>None</v>
       </c>
       <c r="U33" s="2" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-26</v>
       </c>
       <c r="V33" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-26</v>
       </c>
       <c r="W33" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
       </c>
     </row>
     <row r="34">
@@ -3908,22 +3928,22 @@
         <v>Sprint 4</v>
       </c>
       <c r="E34" s="2" t="str">
-        <v>N/A</v>
+        <v>Payroll Page</v>
       </c>
       <c r="F34" s="2" t="str">
-        <v>Microsoft Teams Integration</v>
+        <v>Payroll</v>
       </c>
       <c r="G34" s="2" t="str">
-        <v>Teams Webhook Alerts</v>
+        <v>Finalize Payroll</v>
       </c>
       <c r="H34" s="2" t="str">
-        <v>TSK-TEAMS-001</v>
+        <v>TSK-PAY-004</v>
       </c>
       <c r="I34" s="2" t="str">
-        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+        <v>Implement Payroll finalization and publishing controls</v>
       </c>
       <c r="J34" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="K34" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3938,16 +3958,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O34" s="2" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="P34" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q34" s="2">
-        <v>0.8</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="R34" s="2" t="str">
-        <v>80%</v>
+        <v>30%</v>
       </c>
       <c r="S34" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -3956,13 +3976,13 @@
         <v>None</v>
       </c>
       <c r="U34" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-23</v>
       </c>
       <c r="V34" s="2" t="str">
         <v>2026-06-24</v>
       </c>
       <c r="W34" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
       </c>
     </row>
     <row r="35">
@@ -3979,25 +3999,25 @@
         <v>Sprint 4</v>
       </c>
       <c r="E35" s="2" t="str">
-        <v>Dashboard &amp; Navbar</v>
+        <v>N/A</v>
       </c>
       <c r="F35" s="2" t="str">
-        <v>Role Dashboards &amp; Analytics</v>
+        <v>Microsoft Teams Integration</v>
       </c>
       <c r="G35" s="2" t="str">
-        <v>Performance Tuning</v>
+        <v>Teams Webhook Alerts</v>
       </c>
       <c r="H35" s="2" t="str">
-        <v>TSK-PERF-001</v>
+        <v>TSK-TEAMS-001</v>
       </c>
       <c r="I35" s="2" t="str">
-        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
       </c>
       <c r="J35" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="K35" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="L35" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -4009,16 +4029,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O35" s="2" t="str">
-        <v>HIGH</v>
+        <v>MEDIUM</v>
       </c>
       <c r="P35" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q35" s="2">
-        <v>0.8</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="R35" s="2" t="str">
-        <v>50%</v>
+        <v>80%</v>
       </c>
       <c r="S35" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -4033,12 +4053,83 @@
         <v>2026-06-24</v>
       </c>
       <c r="W35" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B36" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C36" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D36" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E36" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F36" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G36" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H36" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I36" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J36" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K36" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L36" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M36" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N36" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O36" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P36" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q36" s="2">
+        <v>0.7272727272727273</v>
+      </c>
+      <c r="R36" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S36" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T36" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U36" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V36" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W36" s="2" t="str">
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W36"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(shifts): implement dynamic shift management, customizable break timings, and style alignment fixes
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -1205,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1535,16 +1535,36 @@
         <v>* [COMPLETED] TSK-ATT-011 (Implement Dynamic Shift Management System): Designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B17" s="2" t="str">
+        <v>TSK-ATT-012</v>
+      </c>
+      <c r="C17" s="2" t="str">
+        <v>Implement Shift Break Configurations &amp; Customizable Timing Windows</v>
+      </c>
+      <c r="D17" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E17" s="2" t="str">
+        <v>Designed and implemented a comprehensive Shift Break Configuration system and customizable timing windows. Added five break toggles and eight break start/end timing columns to the Shift model in the database schema, pushed it via Prisma, and regenerated the client. Refactored backend break start and end routes to enforce shift-specific break configurations and dynamically parse/evaluate break start times against custom shift timing windows rather than hardcoded ranges. Also introduced a brand new 40-minute Dinner Break. Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI, enforcing this via Zod and route intercepts. Overhauled the frontend Shift Management modal to add customizable inline start/end timing inputs (HH:MM) that dynamically render when a break is enabled, and configured a useEffect hook to automatically sync Lunch/Dinner toggles based on the shift start time. Finally, designed and integrated allowed break badges on the active shift cards displaying their custom time ranges.</v>
+      </c>
+      <c r="F17" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-012 (Implement Shift Break Configurations &amp; Customizable Timing Windows): Designed and implemented a comprehensive Shift Break Configuration system and customizable timing windows. Added five break toggles and eight break start/end timing columns to the Shift model in the database schema, pushed it via Prisma, and regenerated the client. Refactored backend break start and end routes to enforce shift-specific break configurations and dynamically parse/evaluate break start times against custom shift timing windows rather than hardcoded ranges. Also introduced a brand new 40-minute Dinner Break. Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI, enforcing this via Zod and route intercepts. Overhauled the frontend Shift Management modal to add customizable inline start/end timing inputs (HH:MM) that dynamically render when a break is enabled, and configured a useEffect hook to automatically sync Lunch/Dinner toggles based on the shift start time. Finally, designed and integrated allowed break badges on the active shift cards displaying their custom time ranges.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W36"/>
+  <dimension ref="A1:W37"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -3396,7 +3416,7 @@
         <v>2</v>
       </c>
       <c r="Q26" s="2">
-        <v>0.7272727272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R26" s="2" t="str">
         <v>100%</v>
@@ -3414,7 +3434,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W26" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
     <row r="27">
@@ -3467,7 +3487,7 @@
         <v>8</v>
       </c>
       <c r="Q27" s="2">
-        <v>0.7272727272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R27" s="2" t="str">
         <v>100%</v>
@@ -3485,7 +3505,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W27" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
     <row r="28">
@@ -3538,7 +3558,7 @@
         <v>4</v>
       </c>
       <c r="Q28" s="2">
-        <v>0.7272727272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R28" s="2" t="str">
         <v>100%</v>
@@ -3556,7 +3576,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W28" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
     <row r="29">
@@ -3609,7 +3629,7 @@
         <v>6</v>
       </c>
       <c r="Q29" s="2">
-        <v>0.7272727272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R29" s="2" t="str">
         <v>100%</v>
@@ -3627,7 +3647,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W29" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
     <row r="30">
@@ -3680,7 +3700,7 @@
         <v>4</v>
       </c>
       <c r="Q30" s="2">
-        <v>0.7272727272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R30" s="2" t="str">
         <v>100%</v>
@@ -3698,7 +3718,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W30" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
     <row r="31">
@@ -3751,7 +3771,7 @@
         <v>8</v>
       </c>
       <c r="Q31" s="2">
-        <v>0.7272727272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R31" s="2" t="str">
         <v>100%</v>
@@ -3769,7 +3789,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W31" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
     <row r="32">
@@ -3822,7 +3842,7 @@
         <v>4</v>
       </c>
       <c r="Q32" s="2">
-        <v>0.7272727272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R32" s="2" t="str">
         <v>100%</v>
@@ -3840,7 +3860,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W32" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
     <row r="33">
@@ -3893,7 +3913,7 @@
         <v>12</v>
       </c>
       <c r="Q33" s="2">
-        <v>0.7272727272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R33" s="2" t="str">
         <v>100%</v>
@@ -3911,7 +3931,7 @@
         <v>2026-06-26</v>
       </c>
       <c r="W33" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
     <row r="34">
@@ -3928,61 +3948,61 @@
         <v>Sprint 4</v>
       </c>
       <c r="E34" s="2" t="str">
-        <v>Payroll Page</v>
+        <v>Shift Management Page</v>
       </c>
       <c r="F34" s="2" t="str">
-        <v>Payroll</v>
+        <v>Attendance</v>
       </c>
       <c r="G34" s="2" t="str">
-        <v>Finalize Payroll</v>
+        <v>Shift Break Configurations</v>
       </c>
       <c r="H34" s="2" t="str">
-        <v>TSK-PAY-004</v>
+        <v>TSK-ATT-012</v>
       </c>
       <c r="I34" s="2" t="str">
-        <v>Implement Payroll finalization and publishing controls</v>
+        <v>Implement Shift-Specific Break Configurations &amp; Customizable Timing Windows</v>
       </c>
       <c r="J34" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="K34" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="L34" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="M34" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="N34" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O34" s="2" t="str">
         <v>HIGH</v>
       </c>
       <c r="P34" s="2">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="Q34" s="2">
-        <v>0.7272727272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R34" s="2" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="S34" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="T34" s="2" t="str">
         <v>None</v>
       </c>
       <c r="U34" s="2" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-26</v>
       </c>
       <c r="V34" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-26</v>
       </c>
       <c r="W34" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
     <row r="35">
@@ -3999,22 +4019,22 @@
         <v>Sprint 4</v>
       </c>
       <c r="E35" s="2" t="str">
-        <v>N/A</v>
+        <v>Payroll Page</v>
       </c>
       <c r="F35" s="2" t="str">
-        <v>Microsoft Teams Integration</v>
+        <v>Payroll</v>
       </c>
       <c r="G35" s="2" t="str">
-        <v>Teams Webhook Alerts</v>
+        <v>Finalize Payroll</v>
       </c>
       <c r="H35" s="2" t="str">
-        <v>TSK-TEAMS-001</v>
+        <v>TSK-PAY-004</v>
       </c>
       <c r="I35" s="2" t="str">
-        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
+        <v>Implement Payroll finalization and publishing controls</v>
       </c>
       <c r="J35" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="K35" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -4029,16 +4049,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O35" s="2" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="P35" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q35" s="2">
-        <v>0.7272727272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R35" s="2" t="str">
-        <v>80%</v>
+        <v>30%</v>
       </c>
       <c r="S35" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -4047,13 +4067,13 @@
         <v>None</v>
       </c>
       <c r="U35" s="2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-23</v>
       </c>
       <c r="V35" s="2" t="str">
         <v>2026-06-24</v>
       </c>
       <c r="W35" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
     <row r="36">
@@ -4070,25 +4090,25 @@
         <v>Sprint 4</v>
       </c>
       <c r="E36" s="2" t="str">
-        <v>Dashboard &amp; Navbar</v>
+        <v>N/A</v>
       </c>
       <c r="F36" s="2" t="str">
-        <v>Role Dashboards &amp; Analytics</v>
+        <v>Microsoft Teams Integration</v>
       </c>
       <c r="G36" s="2" t="str">
-        <v>Performance Tuning</v>
+        <v>Teams Webhook Alerts</v>
       </c>
       <c r="H36" s="2" t="str">
-        <v>TSK-PERF-001</v>
+        <v>TSK-TEAMS-001</v>
       </c>
       <c r="I36" s="2" t="str">
-        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+        <v>Implement Microsoft Teams Alerts for Leave submissions and Friday updates</v>
       </c>
       <c r="J36" s="2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>N/A</v>
       </c>
       <c r="K36" s="2" t="str">
-        <v>N/A</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="L36" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -4100,16 +4120,16 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="O36" s="2" t="str">
-        <v>HIGH</v>
+        <v>MEDIUM</v>
       </c>
       <c r="P36" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q36" s="2">
-        <v>0.7272727272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R36" s="2" t="str">
-        <v>50%</v>
+        <v>80%</v>
       </c>
       <c r="S36" s="2" t="str">
         <v>IN_PROGRESS</v>
@@ -4124,12 +4144,83 @@
         <v>2026-06-24</v>
       </c>
       <c r="W36" s="2" t="str">
-        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Productive Time (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B37" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C37" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D37" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E37" s="2" t="str">
+        <v>Dashboard &amp; Navbar</v>
+      </c>
+      <c r="F37" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G37" s="2" t="str">
+        <v>Performance Tuning</v>
+      </c>
+      <c r="H37" s="2" t="str">
+        <v>TSK-PERF-001</v>
+      </c>
+      <c r="I37" s="2" t="str">
+        <v>Lift Employee Summary data to global context to avoid redundant fetches</v>
+      </c>
+      <c r="J37" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="K37" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L37" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="M37" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="N37" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="O37" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P37" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q37" s="2">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="R37" s="2" t="str">
+        <v>50%</v>
+      </c>
+      <c r="S37" s="2" t="str">
+        <v>IN_PROGRESS</v>
+      </c>
+      <c r="T37" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U37" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="V37" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="W37" s="2" t="str">
+        <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W37"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: Saturday absent records cleanup, timezone mismatch issues, and desktop agent startup registry config
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -3,22 +3,22 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Projects_Master" sheetId="1" r:id="rId1"/>
-    <sheet name="Daily_Updates" sheetId="2" r:id="rId2"/>
-    <sheet name="Daily_Task_Planner" sheetId="3" r:id="rId3"/>
-    <sheet name="Weekly_Roadmap" sheetId="4" r:id="rId4"/>
-    <sheet name="Sprint_Tracker" sheetId="5" r:id="rId5"/>
-    <sheet name="Feature_Tracker" sheetId="6" r:id="rId6"/>
-    <sheet name="Frontend_Tracker" sheetId="7" r:id="rId7"/>
-    <sheet name="Backend_Tracker" sheetId="8" r:id="rId8"/>
-    <sheet name="Database_Tracker" sheetId="9" r:id="rId9"/>
-    <sheet name="API_Tracker" sheetId="10" r:id="rId10"/>
-    <sheet name="Bug_Tracker" sheetId="11" r:id="rId11"/>
-    <sheet name="Testing_Tracker" sheetId="12" r:id="rId12"/>
-    <sheet name="Deployment_Tracker" sheetId="13" r:id="rId13"/>
-    <sheet name="Risks_And_Blockers" sheetId="14" r:id="rId14"/>
-    <sheet name="Team_Productivity" sheetId="15" r:id="rId15"/>
-    <sheet name="Standup_Feed" sheetId="16" r:id="rId16"/>
+    <sheet name="Standup_Feed" sheetId="1" r:id="rId1"/>
+    <sheet name="Projects_Master" sheetId="2" r:id="rId2"/>
+    <sheet name="Daily_Updates" sheetId="3" r:id="rId3"/>
+    <sheet name="Daily_Task_Planner" sheetId="4" r:id="rId4"/>
+    <sheet name="Weekly_Roadmap" sheetId="5" r:id="rId5"/>
+    <sheet name="Sprint_Tracker" sheetId="6" r:id="rId6"/>
+    <sheet name="Feature_Tracker" sheetId="7" r:id="rId7"/>
+    <sheet name="Frontend_Tracker" sheetId="8" r:id="rId8"/>
+    <sheet name="Backend_Tracker" sheetId="9" r:id="rId9"/>
+    <sheet name="Database_Tracker" sheetId="10" r:id="rId10"/>
+    <sheet name="API_Tracker" sheetId="11" r:id="rId11"/>
+    <sheet name="Bug_Tracker" sheetId="12" r:id="rId12"/>
+    <sheet name="Testing_Tracker" sheetId="13" r:id="rId13"/>
+    <sheet name="Deployment_Tracker" sheetId="14" r:id="rId14"/>
+    <sheet name="Risks_And_Blockers" sheetId="15" r:id="rId15"/>
+    <sheet name="Team_Productivity" sheetId="16" r:id="rId16"/>
   </sheets>
 </workbook>
 </file>
@@ -439,6 +439,1235 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F20"/>
+  <cols>
+    <col min="1" max="1" width="13.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="65.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="65.83203125" customWidth="1"/>
+    <col min="6" max="6" width="65.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>Task ID</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>Feature Title</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>Status</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>Development Narrative</v>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v>Standup Copy-Paste Text</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>TSK-DESK-001</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>Build IntelliHrHub Desktop Agent</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>Developed native Windows C# desktop tray application to track locks, wakes, sleep, and user idleness, forwarding events to POST /api/attendance/desktop-event to automate break sessions and checkouts. Tested and verified locally with active Express dev server and remote Hostinger DB.</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>* [COMPLETED] TSK-DESK-001 (Build IntelliHrHub Desktop Agent): Developed native Windows C# desktop tray application to track locks, wakes, sleep, and user idleness, forwarding events to POST /api/attendance/desktop-event to automate break sessions and checkouts. Tested and verified locally with active Express dev server and remote Hostinger DB.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>TSK-ATT-003</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>Implement Live Status Badges &amp; Workday Timeline</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>Implemented live status telemetry indicators (Active, Away, Offline) on Navbar, Sidebar, and Employee Table. Created Live Status Tracker panel in AttendancePage and integrated visual workday timelines, enabling users and HR to click on past dates in history to view worked/break block intervals.</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-003 (Implement Live Status Badges &amp; Workday Timeline): Implemented live status telemetry indicators (Active, Away, Offline) on Navbar, Sidebar, and Employee Table. Created Live Status Tracker panel in AttendancePage and integrated visual workday timelines, enabling users and HR to click on past dates in history to view worked/break block intervals.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>TSK-ATT-004</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>Redesign Workday Timeline with Desktop Telemetry Logs</v>
+      </c>
+      <c r="D4" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>Overhauled the Workday Timeline to show rich activity segments (Active, Idle, Locked), a sleek collapsed state, and a split expanded view with chronological Event Log and Day Summary. Polished card margins and padding, aligned title and panel typography to match cards design system, centered Event Log timeline vertical line, corrected undefined CSS variables, completely removed the block containers around Day Summary items for a cleaner, boundaryless list look, and added a direct 'Download Agent' link at the bottom of the sidebar.</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-004 (Redesign Workday Timeline with Desktop Telemetry Logs): Overhauled the Workday Timeline to show rich activity segments (Active, Idle, Locked), a sleek collapsed state, and a split expanded view with chronological Event Log and Day Summary. Polished card margins and padding, aligned title and panel typography to match cards design system, centered Event Log timeline vertical line, corrected undefined CSS variables, completely removed the block containers around Day Summary items for a cleaner, boundaryless list look, and added a direct 'Download Agent' link at the bottom of the sidebar.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>TSK-DESK-002</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>Integrate Attendance Reminders &amp; Logging in Desktop Agent</v>
+      </c>
+      <c r="D5" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>Successfully integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin ritesh branch.</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <v>* [COMPLETED] TSK-DESK-002 (Integrate Attendance Reminders &amp; Logging in Desktop Agent): Successfully integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin ritesh branch.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>TSK-DESK-003</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>Implement Visible Desktop Dashboard Mini-App Window</v>
+      </c>
+      <c r="D6" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent. Added specific, context-aware confirmation dialogs for starting and ending breaks across the Dashboard, System Tray menu, and slide-up reminders to prevent accidental break markings. Resolved the Hour 14 (2:00 PM to 2:59 PM) classification bug, ensuring afternoon breaks correctly display as Evening Tea Break / End Tea instead of incorrectly mapping to Lunch Break. Refactored the tea break button to dynamically display 'Morning Tea' in the morning hours (before 12 PM) and 'Evening Tea' in the afternoon/evening. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Overhauled the UI spacing, padding, and alignments: increased the header titlebar height, added a 25px symmetrical margin/padding to all internal controls (such as titles, lists, and buttons), and perfectly aligned window control buttons to prevent any edge-clipping or crowding in both normal and maximized window states. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations.</v>
+      </c>
+      <c r="F6" s="2" t="str">
+        <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent. Added specific, context-aware confirmation dialogs for starting and ending breaks across the Dashboard, System Tray menu, and slide-up reminders to prevent accidental break markings. Resolved the Hour 14 (2:00 PM to 2:59 PM) classification bug, ensuring afternoon breaks correctly display as Evening Tea Break / End Tea instead of incorrectly mapping to Lunch Break. Refactored the tea break button to dynamically display 'Morning Tea' in the morning hours (before 12 PM) and 'Evening Tea' in the afternoon/evening. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Overhauled the UI spacing, padding, and alignments: increased the header titlebar height, added a 25px symmetrical margin/padding to all internal controls (such as titles, lists, and buttons), and perfectly aligned window control buttons to prevent any edge-clipping or crowding in both normal and maximized window states. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>TSK-EMP-004</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>Implement Points Dispute Tickets workflow</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>Added PointsDisputeTicket database model and status enum to the Prisma schema, and pushed it to remote database. Created the Express API endpoints (post dispute, fetch, resolve dispute with transaction-safe points reversal and compensating history entries in DB). Overhauled the Leaderboard Page frontend, adding an inline dispute raising form to the Points History Modal, showing status badges, and building a dedicated HR Disputes Queue tab to review, approve, and reject tickets.</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>* [COMPLETED] TSK-EMP-004 (Implement Points Dispute Tickets workflow): Added PointsDisputeTicket database model and status enum to the Prisma schema, and pushed it to remote database. Created the Express API endpoints (post dispute, fetch, resolve dispute with transaction-safe points reversal and compensating history entries in DB). Overhauled the Leaderboard Page frontend, adding an inline dispute raising form to the Points History Modal, showing status badges, and building a dedicated HR Disputes Queue tab to review, approve, and reject tickets.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>TSK-ATT-005</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v>Fix Workday Timeline Calculations &amp; Overhaul UI Popup</v>
+      </c>
+      <c r="D8" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v>Corrected Workday Timeline calculations to prevent calculating worked duration up to 23:59:59 PM for past dates with missing checkouts, aligning it with database workedMinutes. Used zoned time parsing for check-in/out and break times to eliminate UTC-to-local timezone conversion offsets. Overhauled modal UI, increasing width to 760px, resolving overlaps, and stripping double card styles when displayed inside popups.</v>
+      </c>
+      <c r="F8" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-005 (Fix Workday Timeline Calculations &amp; Overhaul UI Popup): Corrected Workday Timeline calculations to prevent calculating worked duration up to 23:59:59 PM for past dates with missing checkouts, aligning it with database workedMinutes. Used zoned time parsing for check-in/out and break times to eliminate UTC-to-local timezone conversion offsets. Overhauled modal UI, increasing width to 760px, resolving overlaps, and stripping double card styles when displayed inside popups.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B9" s="2" t="str">
+        <v>TSK-ATT-006</v>
+      </c>
+      <c r="C9" s="2" t="str">
+        <v>Fix Overtime Calculation in Attendance History Table</v>
+      </c>
+      <c r="D9" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E9" s="2" t="str">
+        <v>Resolved a discrepancy where the attendance history table displayed incorrect overtime durations for employees with late check-ins. Refactored the renderOvertime function in AttendancePage.tsx to dynamically factor in late check-in penalty minutes, ensuring the table matches the employee dashboard Workday Timeline exactly.</v>
+      </c>
+      <c r="F9" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-006 (Fix Overtime Calculation in Attendance History Table): Resolved a discrepancy where the attendance history table displayed incorrect overtime durations for employees with late check-ins. Refactored the renderOvertime function in AttendancePage.tsx to dynamically factor in late check-in penalty minutes, ensuring the table matches the employee dashboard Workday Timeline exactly.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B10" s="2" t="str">
+        <v>TSK-ATT-007</v>
+      </c>
+      <c r="C10" s="2" t="str">
+        <v>Implement Net Worked Minutes and Crash-Aware Concluding Scheduler</v>
+      </c>
+      <c r="D10" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E10" s="2" t="str">
+        <v>Successfully implemented Net Worked Minutes (Option B) by deducting completed break durations from gross checked-in minutes across web checkout, regularization approval, and daily finalization. Rescheduled daily finalization cron job to 7:00 AM IST and implemented a crash-aware classification algorithm: it uses desktop agent activity logs to distinguish between clean OS shutdown without checkout (marked HALF_DAY as neglect penalty) and unexpected power cuts/system crashes (marked PRESENT without penalty). Replaced Events Logged in the frontend Day Summary panel with premium Uptime (since last break/away) and Active Penalties cards.</v>
+      </c>
+      <c r="F10" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-007 (Implement Net Worked Minutes and Crash-Aware Concluding Scheduler): Successfully implemented Net Worked Minutes (Option B) by deducting completed break durations from gross checked-in minutes across web checkout, regularization approval, and daily finalization. Rescheduled daily finalization cron job to 7:00 AM IST and implemented a crash-aware classification algorithm: it uses desktop agent activity logs to distinguish between clean OS shutdown without checkout (marked HALF_DAY as neglect penalty) and unexpected power cuts/system crashes (marked PRESENT without penalty). Replaced Events Logged in the frontend Day Summary panel with premium Uptime (since last break/away) and Active Penalties cards.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B11" s="2" t="str">
+        <v>TSK-TEAM-001</v>
+      </c>
+      <c r="C11" s="2" t="str">
+        <v>Unify Projects under The Star Prime (TSP)</v>
+      </c>
+      <c r="D11" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E11" s="2" t="str">
+        <v>Migrated all 48 Outlook email identities to 'The Star Prime' (TSP) client in the database, preserving all existing assignments. Cleaned up the old TUT and TEC client records. Consolidated the hardcoded magazines and industries into single TSP-owned lists in the Team workspace UI. Removed the client-switcher buttons and integrated inline delete (✕) controls with verification dialogs next to every project card, enabling dynamic addition and removal of projects for managers and team leads.</v>
+      </c>
+      <c r="F11" s="2" t="str">
+        <v>* [COMPLETED] TSK-TEAM-001 (Unify Projects under The Star Prime (TSP)): Migrated all 48 Outlook email identities to 'The Star Prime' (TSP) client in the database, preserving all existing assignments. Cleaned up the old TUT and TEC client records. Consolidated the hardcoded magazines and industries into single TSP-owned lists in the Team workspace UI. Removed the client-switcher buttons and integrated inline delete (✕) controls with verification dialogs next to every project card, enabling dynamic addition and removal of projects for managers and team leads.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B12" s="2" t="str">
+        <v>TSK-TASK-001</v>
+      </c>
+      <c r="C12" s="2" t="str">
+        <v>Implement Dual-View Task Console for Managers and Team Leads</v>
+      </c>
+      <c r="D12" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E12" s="2" t="str">
+        <v>Developed a unified Dual-View Task Console for managers, team leads, admin, and HR. Fetches both personal assigned tasks and manager assigned tasks concurrently. Integrated a premium tab switcher ('Tasks Assigned to Me' vs 'Tasks Assigned to Others') with custom icons and stats, and overhauled the card layout to display creator/assigner metadata (e.g. 'Assigned by: Swapnil Deshmukh (Manager)') for received tasks.</v>
+      </c>
+      <c r="F12" s="2" t="str">
+        <v>* [COMPLETED] TSK-TASK-001 (Implement Dual-View Task Console for Managers and Team Leads): Developed a unified Dual-View Task Console for managers, team leads, admin, and HR. Fetches both personal assigned tasks and manager assigned tasks concurrently. Integrated a premium tab switcher ('Tasks Assigned to Me' vs 'Tasks Assigned to Others') with custom icons and stats, and overhauled the card layout to display creator/assigner metadata (e.g. 'Assigned by: Swapnil Deshmukh (Manager)') for received tasks.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B13" s="2" t="str">
+        <v>TSK-ATT-008</v>
+      </c>
+      <c r="C13" s="2" t="str">
+        <v>Fix Web Break Session AWAY Status Telemetry</v>
+      </c>
+      <c r="D13" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E13" s="2" t="str">
+        <v>Resolved a major telemetry tracking issue where checked-in employees on active web-initiated breaks remained stuck as ACTIVE. Modified the /live-status backend query to select BreakSession records where endTime is null, setting user status to AWAY if an active break session is present. Implemented a break-updated global event listener in the frontend AppProvider to instantly synchronize and refresh local status dots in the Navbar and Sidebar upon starting or ending breaks.</v>
+      </c>
+      <c r="F13" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-008 (Fix Web Break Session AWAY Status Telemetry): Resolved a major telemetry tracking issue where checked-in employees on active web-initiated breaks remained stuck as ACTIVE. Modified the /live-status backend query to select BreakSession records where endTime is null, setting user status to AWAY if an active break session is present. Implemented a break-updated global event listener in the frontend AppProvider to instantly synchronize and refresh local status dots in the Navbar and Sidebar upon starting or ending breaks.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B14" s="2" t="str">
+        <v>TSK-ATT-009</v>
+      </c>
+      <c r="C14" s="2" t="str">
+        <v>Implement Paid Overtime Pre-Approval Workflow and Paid Tags</v>
+      </c>
+      <c r="D14" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E14" s="2" t="str">
+        <v>Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days (with full calendar-exception check) by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+      </c>
+      <c r="F14" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-009 (Implement Paid Overtime Pre-Approval Workflow and Paid Tags): Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days (with full calendar-exception check) by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B15" s="2" t="str">
+        <v>TSK-ATT-010</v>
+      </c>
+      <c r="C15" s="2" t="str">
+        <v>Implement Incomplete Shift Hours Warning on Checkout and Logout</v>
+      </c>
+      <c r="D15" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E15" s="2" t="str">
+        <v>Designed and implemented proactive warnings for employees who attempt to check out of their shift or log out of the application before completing their required working hours (9 hours + late penalties). Rendered a prominent, high-visibility red warning banner at the top of the Checkout Modal detailing their shift requirements and remaining time. Integrated a similar warning into the browser confirmation alert when clicking the application logout button in the topbar, ensuring zero gaps in compliance and attendance tracking.</v>
+      </c>
+      <c r="F15" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-010 (Implement Incomplete Shift Hours Warning on Checkout and Logout): Designed and implemented proactive warnings for employees who attempt to check out of their shift or log out of the application before completing their required working hours (9 hours + late penalties). Rendered a prominent, high-visibility red warning banner at the top of the Checkout Modal detailing their shift requirements and remaining time. Integrated a similar warning into the browser confirmation alert when clicking the application logout button in the topbar, ensuring zero gaps in compliance and attendance tracking.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B16" s="2" t="str">
+        <v>TSK-ATT-011</v>
+      </c>
+      <c r="C16" s="2" t="str">
+        <v>Implement Dynamic Shift Management System</v>
+      </c>
+      <c r="D16" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E16" s="2" t="str">
+        <v>Designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+      </c>
+      <c r="F16" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-011 (Implement Dynamic Shift Management System): Designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B17" s="2" t="str">
+        <v>TSK-ATT-012</v>
+      </c>
+      <c r="C17" s="2" t="str">
+        <v>Implement Shift Break Configurations &amp; Customizable Timing Windows</v>
+      </c>
+      <c r="D17" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E17" s="2" t="str">
+        <v>Designed and implemented a comprehensive Shift Break Configuration system and customizable timing windows. Added five break toggles and eight break start/end timing columns to the Shift model in the database schema, pushed it via Prisma, and regenerated the client. Refactored backend break start and end routes to enforce shift-specific break configurations and dynamically parse/evaluate break start times against custom shift timing windows rather than hardcoded ranges. Also introduced a brand new 40-minute Dinner Break. Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI, enforcing this via Zod and route intercepts. Overhauled the frontend Shift Management modal to add customizable inline start/end timing inputs (HH:MM) that dynamically render when a break is enabled, and configured a useEffect hook to automatically sync Lunch/Dinner toggles based on the shift start time. Finally, designed and integrated allowed break badges on the active shift cards displaying their custom time ranges.</v>
+      </c>
+      <c r="F17" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-012 (Implement Shift Break Configurations &amp; Customizable Timing Windows): Designed and implemented a comprehensive Shift Break Configuration system and customizable timing windows. Added five break toggles and eight break start/end timing columns to the Shift model in the database schema, pushed it via Prisma, and regenerated the client. Refactored backend break start and end routes to enforce shift-specific break configurations and dynamically parse/evaluate break start times against custom shift timing windows rather than hardcoded ranges. Also introduced a brand new 40-minute Dinner Break. Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI, enforcing this via Zod and route intercepts. Overhauled the frontend Shift Management modal to add customizable inline start/end timing inputs (HH:MM) that dynamically render when a break is enabled, and configured a useEffect hook to automatically sync Lunch/Dinner toggles based on the shift start time. Finally, designed and integrated allowed break badges on the active shift cards displaying their custom time ranges.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="B18" s="2" t="str">
+        <v>TSK-ATT-013</v>
+      </c>
+      <c r="C18" s="2" t="str">
+        <v>Fix Weekend Attendance Accuracy: DB Cleanup, Status Priority &amp; Dynamic Exceptions Fetching</v>
+      </c>
+      <c r="D18" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E18" s="2" t="str">
+        <v>Conducted a full audit of the employee profile attendance history and identified three root-cause bugs causing Saturdays to incorrectly appear as Absent. (1) The pre-June-26 daily finalization cron had no working-day guard, which created 87 rogue ABSENT records on Saturdays from May 23 to June 20. A one-time cleanup script was written and executed to bulk-delete all 87 records. (2) The frontend finalStatus resolution logic in EmployeeAttendanceTab was refactored to enforce a strict priority hierarchy: PRESENT/HALF_DAY &gt; LEAVE &gt; HOLIDAY/OFF &gt; ABSENT. This prevents any rogue ABSENT database record from overriding a correctly-calculated Off Day or Leave status. (3) Calendar exceptions (Working Saturdays, Holidays) were previously fetched once at page load using today's date. Switching the month/year in the Attendance History dropdown did not re-fetch. The selectedMonth and selectedYear state was lifted to EmployeeProfilePage, added as dependencies to the reloadProfile callback, and the /calendar API call was updated to use the selected month/year dynamically. TypeScript compilation passed with 0 errors.</v>
+      </c>
+      <c r="F18" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-013 (Fix Weekend Attendance Accuracy: DB Cleanup, Status Priority &amp; Dynamic Exceptions Fetching): Conducted a full audit of the employee profile attendance history and identified three root-cause bugs causing Saturdays to incorrectly appear as Absent. (1) The pre-June-26 daily finalization cron had no working-day guard, which created 87 rogue ABSENT records on Saturdays from May 23 to June 20. A one-time cleanup script was written and executed to bulk-delete all 87 records. (2) The frontend finalStatus resolution logic in EmployeeAttendanceTab was refactored to enforce a strict priority hierarchy: PRESENT/HALF_DAY &gt; LEAVE &gt; HOLIDAY/OFF &gt; ABSENT. This prevents any rogue ABSENT database record from overriding a correctly-calculated Off Day or Leave status. (3) Calendar exceptions (Working Saturdays, Holidays) were previously fetched once at page load using today's date. Switching the month/year in the Attendance History dropdown did not re-fetch. The selectedMonth and selectedYear state was lifted to EmployeeProfilePage, added as dependencies to the reloadProfile callback, and the /calendar API call was updated to use the selected month/year dynamically. TypeScript compilation passed with 0 errors.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="B19" s="2" t="str">
+        <v>TSK-ATT-014</v>
+      </c>
+      <c r="C19" s="2" t="str">
+        <v>Fix Timezone Mismatches in Attendance Timeline &amp; Progress Bars</v>
+      </c>
+      <c r="D19" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E19" s="2" t="str">
+        <v>Identified and fixed a timezone shift bug where UTC attendanceDate strings returned by the backend shifted by one day when parsed locally in the browser. This offset caused today's active check-in record to match the previous day (yesterday) in the Employee Profile page list, while correctly displaying under today in the Live status telemetry page. The mismatch also broke the Workday Timeline progress bar for that record because it mapped a check-in time of today onto yesterday's schedule grid. Fixed by refactoring EmployeeAttendanceTab.tsx and AttendancePage.tsx to use formatInTimeZone and toZonedTime with Asia/Kolkata timezone mapping instead of raw local Date parts. Also resolved the date.toISOString() local-to-ISO date serialization shift inside the unifiedHistory map which shifted dates back by one day for selected profile timeline popups. Resolved a bug where several instantiations of the WorkdayTimeline component across the web app were missing the employeeId and token props, which prevented it from authenticating and fetching desktop logs. Resolved a bug where the timeline defaulted to a 9:00 AM - 6:00 PM shift, which caused night shift employee check-ins (e.g. checked in at 9:07 AM for an 18:00 night shift) to be incorrectly flagged as LATE while displaying an empty Active Penalties card (since the database correctly stores 0 penalties for night shift check-ins). Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Included shift relation in employee GET by ID and auth me endpoints. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Finally, overhauled the Day Summary grid list style in WorkdayTimeline.css, making the rows borderless, compact, and matched to the Break Schedule's typography and font size. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments, and added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Updated monthlySummaryRows to group historical rows by zoned month/year, preventing date boundaries from spilling into adjacent months.</v>
+      </c>
+      <c r="F19" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-014 (Fix Timezone Mismatches in Attendance Timeline &amp; Progress Bars): Identified and fixed a timezone shift bug where UTC attendanceDate strings returned by the backend shifted by one day when parsed locally in the browser. This offset caused today's active check-in record to match the previous day (yesterday) in the Employee Profile page list, while correctly displaying under today in the Live status telemetry page. The mismatch also broke the Workday Timeline progress bar for that record because it mapped a check-in time of today onto yesterday's schedule grid. Fixed by refactoring EmployeeAttendanceTab.tsx and AttendancePage.tsx to use formatInTimeZone and toZonedTime with Asia/Kolkata timezone mapping instead of raw local Date parts. Also resolved the date.toISOString() local-to-ISO date serialization shift inside the unifiedHistory map which shifted dates back by one day for selected profile timeline popups. Resolved a bug where several instantiations of the WorkdayTimeline component across the web app were missing the employeeId and token props, which prevented it from authenticating and fetching desktop logs. Resolved a bug where the timeline defaulted to a 9:00 AM - 6:00 PM shift, which caused night shift employee check-ins (e.g. checked in at 9:07 AM for an 18:00 night shift) to be incorrectly flagged as LATE while displaying an empty Active Penalties card (since the database correctly stores 0 penalties for night shift check-ins). Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Included shift relation in employee GET by ID and auth me endpoints. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Finally, overhauled the Day Summary grid list style in WorkdayTimeline.css, making the rows borderless, compact, and matched to the Break Schedule's typography and font size. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments, and added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Updated monthlySummaryRows to group historical rows by zoned month/year, preventing date boundaries from spilling into adjacent months.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="B20" s="2" t="str">
+        <v>TSK-ATT-015</v>
+      </c>
+      <c r="C20" s="2" t="str">
+        <v>Enforce Desktop Client Continuous Tracking</v>
+      </c>
+      <c r="D20" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E20" s="2" t="str">
+        <v>Enforced desktop client telemetry tracking to prevent users from bypassing tracking or disconnecting manually. Removed the Disconnect button from the Dashboard UI and the Exit context menu from the system tray icon to ensure the app cannot be manually closed or logged out of. Implemented a registry key injection on application start to automatically register the client as a Windows startup application (HKCU\SOFTWARE\Microsoft\Windows\CurrentVersion\Run).</v>
+      </c>
+      <c r="F20" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-015 (Enforce Desktop Client Continuous Tracking): Enforced desktop client telemetry tracking to prevent users from bypassing tracking or disconnecting manually. Removed the Disconnect button from the Dashboard UI and the Exit context menu from the system tray icon to ensure the app cannot be manually closed or logged out of. Implemented a registry key injection on application start to automatically register the client as a Windows startup application (HKCU\SOFTWARE\Microsoft\Windows\CurrentVersion\Run).</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F20"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F7"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="29.83203125" customWidth="1"/>
+    <col min="3" max="3" width="58.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="str">
+        <v>Table</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>Relationships</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>Indexes</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>Migration</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>Seed Data</v>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v>Completion %</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>User / Role</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>Role 1:N User</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>users.email (unique), users.roleId</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>Seeded</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>Employee</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>User 1:1 Employee</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>employees.employeeCode (unique), employees.departmentId</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>Seeded</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>Employee 1:N Attendance</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>(employeeId, attendanceDate) unique</v>
+      </c>
+      <c r="D4" s="2" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>Seeded</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="str">
+        <v>LeaveRequest</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>Employee 1:N LeaveRequest</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>leave_requests.employeeId, leave_requests.status</v>
+      </c>
+      <c r="D5" s="2" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>Seeded</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v>PayrollRecord</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>Employee 1:N PayrollRecord</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>(employeeId, month, year) unique</v>
+      </c>
+      <c r="D6" s="2" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>Seeded</v>
+      </c>
+      <c r="F6" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="str">
+        <v>RefreshTokens</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>User 1:N RefreshTokens</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>refresh_tokens.userId</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F8"/>
+  <cols>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="str">
+        <v>API Name</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>Endpoint</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>Method</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>Integrated</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>Testing Status</v>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v>Completion %</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>User Login</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>/api/auth/login</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>POST</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>PASSED</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>Token Refresh</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>/api/auth/refresh</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>POST</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>PASSED</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>Clock In</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>/api/attendance/check-in</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>POST</v>
+      </c>
+      <c r="D4" s="2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>PASSED</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="str">
+        <v>Apply Leave</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>/api/leaves</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>POST</v>
+      </c>
+      <c r="D5" s="2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>PASSED</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v>Generate Payroll</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>/api/payroll/generate</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>POST</v>
+      </c>
+      <c r="D6" s="2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>PASSED</v>
+      </c>
+      <c r="F6" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="str">
+        <v>Lock Payroll</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>/api/payroll/:id/publish</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>PUT</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v>NO</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>30%</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>Quick Meet</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>/api/google/quick-meet</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v>POST</v>
+      </c>
+      <c r="D8" s="2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v>PASSED</v>
+      </c>
+      <c r="F8" s="2" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.83203125" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="str">
+        <v>Bug ID</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>Module</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>Severity</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>Assigned To</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>ETA</v>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>BUG-PAY-001</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>MOD-PAYROLL</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>LOW</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v>Amit (Backend)</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>2026-06-22</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>FIXED</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>BUG-LV-002</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>MOD-LEAVE</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>Priya (QA)</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>FIXED</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F7"/>
+  <cols>
+    <col min="1" max="1" width="17.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>Unit Test</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>Integration Test</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>Manual Test</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>Auth / RBAC</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>Vitest (Passed)</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>Supertest (Passed)</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>Signed Off</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>Employee CRUD</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>Vitest (Passed)</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>Supertest (Passed)</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>Signed Off</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>Time Clocking</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>Vitest (Passed)</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>Supertest (Passed)</v>
+      </c>
+      <c r="D4" s="2" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>Signed Off</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="str">
+        <v>Leave Workflow</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>Vitest (Passed)</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>Supertest (Passed)</v>
+      </c>
+      <c r="D5" s="2" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>Signed Off</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v>Payroll Drafts</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>Vitest (Passed)</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>Supertest (Passed)</v>
+      </c>
+      <c r="D6" s="2" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>Signed Off</v>
+      </c>
+      <c r="F6" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="str">
+        <v>Google Sync</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>Vitest (Passed)</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>Mock Sync (Passed)</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>Signed Off</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <cols>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="2" max="2" width="19.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="19.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="str">
+        <v>Environment</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>Frontend Version</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>Backend Version</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>Database Version</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>Staging (Render/Neon)</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>2.0.0-rc1</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>2.0.0-rc1</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v>v2.0-migration-8</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>HEALTHY</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>Production (VPS Target)</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>Pending Release</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>Pending Release</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>Pending Release</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>PLANNED</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="65.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.83203125" customWidth="1"/>
+    <col min="5" max="5" width="65.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="str">
+        <v>Risk Type</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>Description</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>Severity</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>Owner</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>Mitigation Plan</v>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>Third-Party OAuth</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>Requires corporate Google Cloud Project with OAuth consent verification for all employees.</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v>Lead Architect</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>Provide structured instructions for client credential creation and allow staging environment testing.</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>ACTIVE</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>Teams Webhook Delivery</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>Microsoft Teams incoming webhook configuration requires organizational admin privilege.</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>DevOps</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>Provide clear documentation for managers to generate incoming webhook URLs for their channels.</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>ACTIVE</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <cols>
+    <col min="1" max="1" width="13.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="21.83203125" customWidth="1"/>
+    <col min="5" max="5" width="58.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>Tasks Completed</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>Hours Worked</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>Productivity Score</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>Remarks</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>Rahul (FE)</v>
+      </c>
+      <c r="B2" s="2">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2">
+        <v>72</v>
+      </c>
+      <c r="D2" s="2">
+        <v>9.5</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>High quality CSS styling and responsive UI pages</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>Amit (BE)</v>
+      </c>
+      <c r="B3" s="2">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2">
+        <v>80</v>
+      </c>
+      <c r="D3" s="2">
+        <v>9.8</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>Extremely robust controllers, schemas and Prisma models</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>Priya (QA)</v>
+      </c>
+      <c r="B4" s="2">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2">
+        <v>48</v>
+      </c>
+      <c r="D4" s="2">
+        <v>9.2</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>Thorough test suites and Playwright setup</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N2"/>
   <cols>
     <col min="1" max="1" width="36.83203125" customWidth="1"/>
@@ -552,1025 +1781,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
-  <cols>
-    <col min="1" max="1" width="19.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
-    <col min="5" max="5" width="17.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="3" t="str">
-        <v>API Name</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Endpoint</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>Method</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>Integrated</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>Testing Status</v>
-      </c>
-      <c r="F1" s="3" t="str">
-        <v>Completion %</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="str">
-        <v>User Login</v>
-      </c>
-      <c r="B2" s="2" t="str">
-        <v>/api/auth/login</v>
-      </c>
-      <c r="C2" s="2" t="str">
-        <v>POST</v>
-      </c>
-      <c r="D2" s="2" t="str">
-        <v>YES</v>
-      </c>
-      <c r="E2" s="2" t="str">
-        <v>PASSED</v>
-      </c>
-      <c r="F2" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v>Token Refresh</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>/api/auth/refresh</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>POST</v>
-      </c>
-      <c r="D3" s="2" t="str">
-        <v>YES</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v>PASSED</v>
-      </c>
-      <c r="F3" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="str">
-        <v>Clock In</v>
-      </c>
-      <c r="B4" s="2" t="str">
-        <v>/api/attendance/check-in</v>
-      </c>
-      <c r="C4" s="2" t="str">
-        <v>POST</v>
-      </c>
-      <c r="D4" s="2" t="str">
-        <v>YES</v>
-      </c>
-      <c r="E4" s="2" t="str">
-        <v>PASSED</v>
-      </c>
-      <c r="F4" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="str">
-        <v>Apply Leave</v>
-      </c>
-      <c r="B5" s="2" t="str">
-        <v>/api/leaves</v>
-      </c>
-      <c r="C5" s="2" t="str">
-        <v>POST</v>
-      </c>
-      <c r="D5" s="2" t="str">
-        <v>YES</v>
-      </c>
-      <c r="E5" s="2" t="str">
-        <v>PASSED</v>
-      </c>
-      <c r="F5" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="str">
-        <v>Generate Payroll</v>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v>/api/payroll/generate</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v>POST</v>
-      </c>
-      <c r="D6" s="2" t="str">
-        <v>YES</v>
-      </c>
-      <c r="E6" s="2" t="str">
-        <v>PASSED</v>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="str">
-        <v>Lock Payroll</v>
-      </c>
-      <c r="B7" s="2" t="str">
-        <v>/api/payroll/:id/publish</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v>PUT</v>
-      </c>
-      <c r="D7" s="2" t="str">
-        <v>NO</v>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v>PENDING</v>
-      </c>
-      <c r="F7" s="2" t="str">
-        <v>30%</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="str">
-        <v>Quick Meet</v>
-      </c>
-      <c r="B8" s="2" t="str">
-        <v>/api/google/quick-meet</v>
-      </c>
-      <c r="C8" s="2" t="str">
-        <v>POST</v>
-      </c>
-      <c r="D8" s="2" t="str">
-        <v>YES</v>
-      </c>
-      <c r="E8" s="2" t="str">
-        <v>PASSED</v>
-      </c>
-      <c r="F8" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="17.83203125" customWidth="1"/>
-    <col min="5" max="5" width="13.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="3" t="str">
-        <v>Bug ID</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Module</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>Severity</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>Assigned To</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>ETA</v>
-      </c>
-      <c r="F1" s="3" t="str">
-        <v>Status</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="str">
-        <v>BUG-PAY-001</v>
-      </c>
-      <c r="B2" s="2" t="str">
-        <v>MOD-PAYROLL</v>
-      </c>
-      <c r="C2" s="2" t="str">
-        <v>LOW</v>
-      </c>
-      <c r="D2" s="2" t="str">
-        <v>Amit (Backend)</v>
-      </c>
-      <c r="E2" s="2" t="str">
-        <v>2026-06-22</v>
-      </c>
-      <c r="F2" s="2" t="str">
-        <v>FIXED</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v>BUG-LV-002</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>MOD-LEAVE</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>MEDIUM</v>
-      </c>
-      <c r="D3" s="2" t="str">
-        <v>Priya (QA)</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v>2026-06-24</v>
-      </c>
-      <c r="F3" s="2" t="str">
-        <v>FIXED</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
-  <cols>
-    <col min="1" max="1" width="17.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="21.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="13.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="3" t="str">
-        <v>Feature</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Unit Test</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>Integration Test</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>Manual Test</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>UAT</v>
-      </c>
-      <c r="F1" s="3" t="str">
-        <v>Status</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="str">
-        <v>Auth / RBAC</v>
-      </c>
-      <c r="B2" s="2" t="str">
-        <v>Vitest (Passed)</v>
-      </c>
-      <c r="C2" s="2" t="str">
-        <v>Supertest (Passed)</v>
-      </c>
-      <c r="D2" s="2" t="str">
-        <v>Verified</v>
-      </c>
-      <c r="E2" s="2" t="str">
-        <v>Signed Off</v>
-      </c>
-      <c r="F2" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v>Employee CRUD</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>Vitest (Passed)</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>Supertest (Passed)</v>
-      </c>
-      <c r="D3" s="2" t="str">
-        <v>Verified</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v>Signed Off</v>
-      </c>
-      <c r="F3" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="str">
-        <v>Time Clocking</v>
-      </c>
-      <c r="B4" s="2" t="str">
-        <v>Vitest (Passed)</v>
-      </c>
-      <c r="C4" s="2" t="str">
-        <v>Supertest (Passed)</v>
-      </c>
-      <c r="D4" s="2" t="str">
-        <v>Verified</v>
-      </c>
-      <c r="E4" s="2" t="str">
-        <v>Signed Off</v>
-      </c>
-      <c r="F4" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="str">
-        <v>Leave Workflow</v>
-      </c>
-      <c r="B5" s="2" t="str">
-        <v>Vitest (Passed)</v>
-      </c>
-      <c r="C5" s="2" t="str">
-        <v>Supertest (Passed)</v>
-      </c>
-      <c r="D5" s="2" t="str">
-        <v>Verified</v>
-      </c>
-      <c r="E5" s="2" t="str">
-        <v>Signed Off</v>
-      </c>
-      <c r="F5" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="str">
-        <v>Payroll Drafts</v>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v>Vitest (Passed)</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v>Supertest (Passed)</v>
-      </c>
-      <c r="D6" s="2" t="str">
-        <v>Verified</v>
-      </c>
-      <c r="E6" s="2" t="str">
-        <v>Signed Off</v>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="str">
-        <v>Google Sync</v>
-      </c>
-      <c r="B7" s="2" t="str">
-        <v>Vitest (Passed)</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v>Mock Sync (Passed)</v>
-      </c>
-      <c r="D7" s="2" t="str">
-        <v>Verified</v>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v>Signed Off</v>
-      </c>
-      <c r="F7" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="19.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="3" t="str">
-        <v>Environment</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Frontend Version</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>Backend Version</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>Database Version</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>Status</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="str">
-        <v>Staging (Render/Neon)</v>
-      </c>
-      <c r="B2" s="2" t="str">
-        <v>2.0.0-rc1</v>
-      </c>
-      <c r="C2" s="2" t="str">
-        <v>2.0.0-rc1</v>
-      </c>
-      <c r="D2" s="2" t="str">
-        <v>v2.0-migration-8</v>
-      </c>
-      <c r="E2" s="2" t="str">
-        <v>HEALTHY</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v>Production (VPS Target)</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>Pending Release</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>Pending Release</v>
-      </c>
-      <c r="D3" s="2" t="str">
-        <v>Pending Release</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v>PLANNED</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="65.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="17.83203125" customWidth="1"/>
-    <col min="5" max="5" width="65.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="3" t="str">
-        <v>Risk Type</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Description</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>Severity</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>Mitigation Plan</v>
-      </c>
-      <c r="F1" s="3" t="str">
-        <v>Status</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="str">
-        <v>Third-Party OAuth</v>
-      </c>
-      <c r="B2" s="2" t="str">
-        <v>Requires corporate Google Cloud Project with OAuth consent verification for all employees.</v>
-      </c>
-      <c r="C2" s="2" t="str">
-        <v>MEDIUM</v>
-      </c>
-      <c r="D2" s="2" t="str">
-        <v>Lead Architect</v>
-      </c>
-      <c r="E2" s="2" t="str">
-        <v>Provide structured instructions for client credential creation and allow staging environment testing.</v>
-      </c>
-      <c r="F2" s="2" t="str">
-        <v>ACTIVE</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v>Teams Webhook Delivery</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>Microsoft Teams incoming webhook configuration requires organizational admin privilege.</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>MEDIUM</v>
-      </c>
-      <c r="D3" s="2" t="str">
-        <v>DevOps</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v>Provide clear documentation for managers to generate incoming webhook URLs for their channels.</v>
-      </c>
-      <c r="F3" s="2" t="str">
-        <v>ACTIVE</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
-  <cols>
-    <col min="1" max="1" width="13.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="21.83203125" customWidth="1"/>
-    <col min="5" max="5" width="58.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="3" t="str">
-        <v>Developer</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Tasks Completed</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>Hours Worked</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>Productivity Score</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>Remarks</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="str">
-        <v>Rahul (FE)</v>
-      </c>
-      <c r="B2" s="2">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2">
-        <v>72</v>
-      </c>
-      <c r="D2" s="2">
-        <v>9.5</v>
-      </c>
-      <c r="E2" s="2" t="str">
-        <v>High quality CSS styling and responsive UI pages</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v>Amit (BE)</v>
-      </c>
-      <c r="B3" s="2">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2">
-        <v>80</v>
-      </c>
-      <c r="D3" s="2">
-        <v>9.8</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v>Extremely robust controllers, schemas and Prisma models</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="str">
-        <v>Priya (QA)</v>
-      </c>
-      <c r="B4" s="2">
-        <v>6</v>
-      </c>
-      <c r="C4" s="2">
-        <v>48</v>
-      </c>
-      <c r="D4" s="2">
-        <v>9.2</v>
-      </c>
-      <c r="E4" s="2" t="str">
-        <v>Thorough test suites and Playwright setup</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F17"/>
-  <cols>
-    <col min="1" max="1" width="13.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="65.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="65.83203125" customWidth="1"/>
-    <col min="6" max="6" width="65.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="3" t="str">
-        <v>Date</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Task ID</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>Feature Title</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>Status</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>Development Narrative</v>
-      </c>
-      <c r="F1" s="3" t="str">
-        <v>Standup Copy-Paste Text</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="str">
-        <v>2026-06-24</v>
-      </c>
-      <c r="B2" s="2" t="str">
-        <v>TSK-DESK-001</v>
-      </c>
-      <c r="C2" s="2" t="str">
-        <v>Build IntelliHrHub Desktop Agent</v>
-      </c>
-      <c r="D2" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E2" s="2" t="str">
-        <v>Developed native Windows C# desktop tray application to track locks, wakes, sleep, and user idleness, forwarding events to POST /api/attendance/desktop-event to automate break sessions and checkouts. Tested and verified locally with active Express dev server and remote Hostinger DB.</v>
-      </c>
-      <c r="F2" s="2" t="str">
-        <v>* [COMPLETED] TSK-DESK-001 (Build IntelliHrHub Desktop Agent): Developed native Windows C# desktop tray application to track locks, wakes, sleep, and user idleness, forwarding events to POST /api/attendance/desktop-event to automate break sessions and checkouts. Tested and verified locally with active Express dev server and remote Hostinger DB.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v>2026-06-24</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>TSK-ATT-003</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>Implement Live Status Badges &amp; Workday Timeline</v>
-      </c>
-      <c r="D3" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v>Implemented live status telemetry indicators (Active, Away, Offline) on Navbar, Sidebar, and Employee Table. Created Live Status Tracker panel in AttendancePage and integrated visual workday timelines, enabling users and HR to click on past dates in history to view worked/break block intervals.</v>
-      </c>
-      <c r="F3" s="2" t="str">
-        <v>* [COMPLETED] TSK-ATT-003 (Implement Live Status Badges &amp; Workday Timeline): Implemented live status telemetry indicators (Active, Away, Offline) on Navbar, Sidebar, and Employee Table. Created Live Status Tracker panel in AttendancePage and integrated visual workday timelines, enabling users and HR to click on past dates in history to view worked/break block intervals.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="str">
-        <v>2026-06-24</v>
-      </c>
-      <c r="B4" s="2" t="str">
-        <v>TSK-ATT-004</v>
-      </c>
-      <c r="C4" s="2" t="str">
-        <v>Redesign Workday Timeline with Desktop Telemetry Logs</v>
-      </c>
-      <c r="D4" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E4" s="2" t="str">
-        <v>Overhauled the Workday Timeline to show rich activity segments (Active, Idle, Locked), a sleek collapsed state, and a split expanded view with chronological Event Log and Day Summary. Polished card margins and padding, aligned title and panel typography to match cards design system, centered Event Log timeline vertical line, corrected undefined CSS variables, completely removed the block containers around Day Summary items for a cleaner, boundaryless list look, and added a direct 'Download Agent' link at the bottom of the sidebar.</v>
-      </c>
-      <c r="F4" s="2" t="str">
-        <v>* [COMPLETED] TSK-ATT-004 (Redesign Workday Timeline with Desktop Telemetry Logs): Overhauled the Workday Timeline to show rich activity segments (Active, Idle, Locked), a sleek collapsed state, and a split expanded view with chronological Event Log and Day Summary. Polished card margins and padding, aligned title and panel typography to match cards design system, centered Event Log timeline vertical line, corrected undefined CSS variables, completely removed the block containers around Day Summary items for a cleaner, boundaryless list look, and added a direct 'Download Agent' link at the bottom of the sidebar.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="str">
-        <v>2026-06-25</v>
-      </c>
-      <c r="B5" s="2" t="str">
-        <v>TSK-DESK-002</v>
-      </c>
-      <c r="C5" s="2" t="str">
-        <v>Integrate Attendance Reminders &amp; Logging in Desktop Agent</v>
-      </c>
-      <c r="D5" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E5" s="2" t="str">
-        <v>Successfully integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin ritesh branch.</v>
-      </c>
-      <c r="F5" s="2" t="str">
-        <v>* [COMPLETED] TSK-DESK-002 (Integrate Attendance Reminders &amp; Logging in Desktop Agent): Successfully integrated check-in/out and break reminders, dynamic state-aware context menus, and custom slide-up notification alert cards in the native Windows C# Desktop Agent. Pushed all changes to origin ritesh branch.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="str">
-        <v>2026-06-25</v>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v>TSK-DESK-003</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v>Implement Visible Desktop Dashboard Mini-App Window</v>
-      </c>
-      <c r="D6" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E6" s="2" t="str">
-        <v>Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent. Added specific, context-aware confirmation dialogs for starting and ending breaks across the Dashboard, System Tray menu, and slide-up reminders to prevent accidental break markings. Resolved the Hour 14 (2:00 PM to 2:59 PM) classification bug, ensuring afternoon breaks correctly display as Evening Tea Break / End Tea instead of incorrectly mapping to Lunch Break. Refactored the tea break button to dynamically display 'Morning Tea' in the morning hours (before 12 PM) and 'Evening Tea' in the afternoon/evening. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Overhauled the UI spacing, padding, and alignments: increased the header titlebar height, added a 25px symmetrical margin/padding to all internal controls (such as titles, lists, and buttons), and perfectly aligned window control buttons to prevent any edge-clipping or crowding in both normal and maximized window states. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations.</v>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v>* [COMPLETED] TSK-DESK-003 (Implement Visible Desktop Dashboard Mini-App Window): Developed an interactive, visible C# Windows Forms Dashboard window in the Desktop Agent. Added specific, context-aware confirmation dialogs for starting and ending breaks across the Dashboard, System Tray menu, and slide-up reminders to prevent accidental break markings. Resolved the Hour 14 (2:00 PM to 2:59 PM) classification bug, ensuring afternoon breaks correctly display as Evening Tea Break / End Tea instead of incorrectly mapping to Lunch Break. Refactored the tea break button to dynamically display 'Morning Tea' in the morning hours (before 12 PM) and 'Evening Tea' in the afternoon/evening. Resolved a timezone mismatch bug where the active shift and break timers showed incorrect negative durations on the C# desktop agent. Overhauled the UI spacing, padding, and alignments: increased the header titlebar height, added a 25px symmetrical margin/padding to all internal controls (such as titles, lists, and buttons), and perfectly aligned window control buttons to prevent any edge-clipping or crowding in both normal and maximized window states. Resolved the telemetry activity log signature mismatch to fetch, sort, and display daily telemetry activity events chronologically in the desktop agent list box, and enhanced the web app's progress bar with interactive hover tooltips detailing activity log events and durations.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="str">
-        <v>2026-06-25</v>
-      </c>
-      <c r="B7" s="2" t="str">
-        <v>TSK-EMP-004</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v>Implement Points Dispute Tickets workflow</v>
-      </c>
-      <c r="D7" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v>Added PointsDisputeTicket database model and status enum to the Prisma schema, and pushed it to remote database. Created the Express API endpoints (post dispute, fetch, resolve dispute with transaction-safe points reversal and compensating history entries in DB). Overhauled the Leaderboard Page frontend, adding an inline dispute raising form to the Points History Modal, showing status badges, and building a dedicated HR Disputes Queue tab to review, approve, and reject tickets.</v>
-      </c>
-      <c r="F7" s="2" t="str">
-        <v>* [COMPLETED] TSK-EMP-004 (Implement Points Dispute Tickets workflow): Added PointsDisputeTicket database model and status enum to the Prisma schema, and pushed it to remote database. Created the Express API endpoints (post dispute, fetch, resolve dispute with transaction-safe points reversal and compensating history entries in DB). Overhauled the Leaderboard Page frontend, adding an inline dispute raising form to the Points History Modal, showing status badges, and building a dedicated HR Disputes Queue tab to review, approve, and reject tickets.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="str">
-        <v>2026-06-25</v>
-      </c>
-      <c r="B8" s="2" t="str">
-        <v>TSK-ATT-005</v>
-      </c>
-      <c r="C8" s="2" t="str">
-        <v>Fix Workday Timeline Calculations &amp; Overhaul UI Popup</v>
-      </c>
-      <c r="D8" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E8" s="2" t="str">
-        <v>Corrected Workday Timeline calculations to prevent calculating worked duration up to 23:59:59 PM for past dates with missing checkouts, aligning it with database workedMinutes. Used zoned time parsing for check-in/out and break times to eliminate UTC-to-local timezone conversion offsets. Overhauled modal UI, increasing width to 760px, resolving overlaps, and stripping double card styles when displayed inside popups.</v>
-      </c>
-      <c r="F8" s="2" t="str">
-        <v>* [COMPLETED] TSK-ATT-005 (Fix Workday Timeline Calculations &amp; Overhaul UI Popup): Corrected Workday Timeline calculations to prevent calculating worked duration up to 23:59:59 PM for past dates with missing checkouts, aligning it with database workedMinutes. Used zoned time parsing for check-in/out and break times to eliminate UTC-to-local timezone conversion offsets. Overhauled modal UI, increasing width to 760px, resolving overlaps, and stripping double card styles when displayed inside popups.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="str">
-        <v>2026-06-26</v>
-      </c>
-      <c r="B9" s="2" t="str">
-        <v>TSK-ATT-006</v>
-      </c>
-      <c r="C9" s="2" t="str">
-        <v>Fix Overtime Calculation in Attendance History Table</v>
-      </c>
-      <c r="D9" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E9" s="2" t="str">
-        <v>Resolved a discrepancy where the attendance history table displayed incorrect overtime durations for employees with late check-ins. Refactored the renderOvertime function in AttendancePage.tsx to dynamically factor in late check-in penalty minutes, ensuring the table matches the employee dashboard Workday Timeline exactly.</v>
-      </c>
-      <c r="F9" s="2" t="str">
-        <v>* [COMPLETED] TSK-ATT-006 (Fix Overtime Calculation in Attendance History Table): Resolved a discrepancy where the attendance history table displayed incorrect overtime durations for employees with late check-ins. Refactored the renderOvertime function in AttendancePage.tsx to dynamically factor in late check-in penalty minutes, ensuring the table matches the employee dashboard Workday Timeline exactly.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="str">
-        <v>2026-06-26</v>
-      </c>
-      <c r="B10" s="2" t="str">
-        <v>TSK-ATT-007</v>
-      </c>
-      <c r="C10" s="2" t="str">
-        <v>Implement Net Worked Minutes and Crash-Aware Concluding Scheduler</v>
-      </c>
-      <c r="D10" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E10" s="2" t="str">
-        <v>Successfully implemented Net Worked Minutes (Option B) by deducting completed break durations from gross checked-in minutes across web checkout, regularization approval, and daily finalization. Rescheduled daily finalization cron job to 7:00 AM IST and implemented a crash-aware classification algorithm: it uses desktop agent activity logs to distinguish between clean OS shutdown without checkout (marked HALF_DAY as neglect penalty) and unexpected power cuts/system crashes (marked PRESENT without penalty). Replaced Events Logged in the frontend Day Summary panel with premium Uptime (since last break/away) and Active Penalties cards.</v>
-      </c>
-      <c r="F10" s="2" t="str">
-        <v>* [COMPLETED] TSK-ATT-007 (Implement Net Worked Minutes and Crash-Aware Concluding Scheduler): Successfully implemented Net Worked Minutes (Option B) by deducting completed break durations from gross checked-in minutes across web checkout, regularization approval, and daily finalization. Rescheduled daily finalization cron job to 7:00 AM IST and implemented a crash-aware classification algorithm: it uses desktop agent activity logs to distinguish between clean OS shutdown without checkout (marked HALF_DAY as neglect penalty) and unexpected power cuts/system crashes (marked PRESENT without penalty). Replaced Events Logged in the frontend Day Summary panel with premium Uptime (since last break/away) and Active Penalties cards.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="str">
-        <v>2026-06-26</v>
-      </c>
-      <c r="B11" s="2" t="str">
-        <v>TSK-TEAM-001</v>
-      </c>
-      <c r="C11" s="2" t="str">
-        <v>Unify Projects under The Star Prime (TSP)</v>
-      </c>
-      <c r="D11" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E11" s="2" t="str">
-        <v>Migrated all 48 Outlook email identities to 'The Star Prime' (TSP) client in the database, preserving all existing assignments. Cleaned up the old TUT and TEC client records. Consolidated the hardcoded magazines and industries into single TSP-owned lists in the Team workspace UI. Removed the client-switcher buttons and integrated inline delete (✕) controls with verification dialogs next to every project card, enabling dynamic addition and removal of projects for managers and team leads.</v>
-      </c>
-      <c r="F11" s="2" t="str">
-        <v>* [COMPLETED] TSK-TEAM-001 (Unify Projects under The Star Prime (TSP)): Migrated all 48 Outlook email identities to 'The Star Prime' (TSP) client in the database, preserving all existing assignments. Cleaned up the old TUT and TEC client records. Consolidated the hardcoded magazines and industries into single TSP-owned lists in the Team workspace UI. Removed the client-switcher buttons and integrated inline delete (✕) controls with verification dialogs next to every project card, enabling dynamic addition and removal of projects for managers and team leads.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="str">
-        <v>2026-06-26</v>
-      </c>
-      <c r="B12" s="2" t="str">
-        <v>TSK-TASK-001</v>
-      </c>
-      <c r="C12" s="2" t="str">
-        <v>Implement Dual-View Task Console for Managers and Team Leads</v>
-      </c>
-      <c r="D12" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E12" s="2" t="str">
-        <v>Developed a unified Dual-View Task Console for managers, team leads, admin, and HR. Fetches both personal assigned tasks and manager assigned tasks concurrently. Integrated a premium tab switcher ('Tasks Assigned to Me' vs 'Tasks Assigned to Others') with custom icons and stats, and overhauled the card layout to display creator/assigner metadata (e.g. 'Assigned by: Swapnil Deshmukh (Manager)') for received tasks.</v>
-      </c>
-      <c r="F12" s="2" t="str">
-        <v>* [COMPLETED] TSK-TASK-001 (Implement Dual-View Task Console for Managers and Team Leads): Developed a unified Dual-View Task Console for managers, team leads, admin, and HR. Fetches both personal assigned tasks and manager assigned tasks concurrently. Integrated a premium tab switcher ('Tasks Assigned to Me' vs 'Tasks Assigned to Others') with custom icons and stats, and overhauled the card layout to display creator/assigner metadata (e.g. 'Assigned by: Swapnil Deshmukh (Manager)') for received tasks.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="str">
-        <v>2026-06-26</v>
-      </c>
-      <c r="B13" s="2" t="str">
-        <v>TSK-ATT-008</v>
-      </c>
-      <c r="C13" s="2" t="str">
-        <v>Fix Web Break Session AWAY Status Telemetry</v>
-      </c>
-      <c r="D13" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E13" s="2" t="str">
-        <v>Resolved a major telemetry tracking issue where checked-in employees on active web-initiated breaks remained stuck as ACTIVE. Modified the /live-status backend query to select BreakSession records where endTime is null, setting user status to AWAY if an active break session is present. Implemented a break-updated global event listener in the frontend AppProvider to instantly synchronize and refresh local status dots in the Navbar and Sidebar upon starting or ending breaks.</v>
-      </c>
-      <c r="F13" s="2" t="str">
-        <v>* [COMPLETED] TSK-ATT-008 (Fix Web Break Session AWAY Status Telemetry): Resolved a major telemetry tracking issue where checked-in employees on active web-initiated breaks remained stuck as ACTIVE. Modified the /live-status backend query to select BreakSession records where endTime is null, setting user status to AWAY if an active break session is present. Implemented a break-updated global event listener in the frontend AppProvider to instantly synchronize and refresh local status dots in the Navbar and Sidebar upon starting or ending breaks.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="str">
-        <v>2026-06-26</v>
-      </c>
-      <c r="B14" s="2" t="str">
-        <v>TSK-ATT-009</v>
-      </c>
-      <c r="C14" s="2" t="str">
-        <v>Implement Paid Overtime Pre-Approval Workflow and Paid Tags</v>
-      </c>
-      <c r="D14" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E14" s="2" t="str">
-        <v>Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days (with full calendar-exception check) by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
-      </c>
-      <c r="F14" s="2" t="str">
-        <v>* [COMPLETED] TSK-ATT-009 (Implement Paid Overtime Pre-Approval Workflow and Paid Tags): Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days (with full calendar-exception check) by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency.</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="str">
-        <v>2026-06-26</v>
-      </c>
-      <c r="B15" s="2" t="str">
-        <v>TSK-ATT-010</v>
-      </c>
-      <c r="C15" s="2" t="str">
-        <v>Implement Incomplete Shift Hours Warning on Checkout and Logout</v>
-      </c>
-      <c r="D15" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E15" s="2" t="str">
-        <v>Designed and implemented proactive warnings for employees who attempt to check out of their shift or log out of the application before completing their required working hours (9 hours + late penalties). Rendered a prominent, high-visibility red warning banner at the top of the Checkout Modal detailing their shift requirements and remaining time. Integrated a similar warning into the browser confirmation alert when clicking the application logout button in the topbar, ensuring zero gaps in compliance and attendance tracking.</v>
-      </c>
-      <c r="F15" s="2" t="str">
-        <v>* [COMPLETED] TSK-ATT-010 (Implement Incomplete Shift Hours Warning on Checkout and Logout): Designed and implemented proactive warnings for employees who attempt to check out of their shift or log out of the application before completing their required working hours (9 hours + late penalties). Rendered a prominent, high-visibility red warning banner at the top of the Checkout Modal detailing their shift requirements and remaining time. Integrated a similar warning into the browser confirmation alert when clicking the application logout button in the topbar, ensuring zero gaps in compliance and attendance tracking.</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="str">
-        <v>2026-06-26</v>
-      </c>
-      <c r="B16" s="2" t="str">
-        <v>TSK-ATT-011</v>
-      </c>
-      <c r="C16" s="2" t="str">
-        <v>Implement Dynamic Shift Management System</v>
-      </c>
-      <c r="D16" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E16" s="2" t="str">
-        <v>Designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
-      </c>
-      <c r="F16" s="2" t="str">
-        <v>* [COMPLETED] TSK-ATT-011 (Implement Dynamic Shift Management System): Designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift.</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="str">
-        <v>2026-06-26</v>
-      </c>
-      <c r="B17" s="2" t="str">
-        <v>TSK-ATT-012</v>
-      </c>
-      <c r="C17" s="2" t="str">
-        <v>Implement Shift Break Configurations &amp; Customizable Timing Windows</v>
-      </c>
-      <c r="D17" s="2" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="E17" s="2" t="str">
-        <v>Designed and implemented a comprehensive Shift Break Configuration system and customizable timing windows. Added five break toggles and eight break start/end timing columns to the Shift model in the database schema, pushed it via Prisma, and regenerated the client. Refactored backend break start and end routes to enforce shift-specific break configurations and dynamically parse/evaluate break start times against custom shift timing windows rather than hardcoded ranges. Also introduced a brand new 40-minute Dinner Break. Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI, enforcing this via Zod and route intercepts. Overhauled the frontend Shift Management modal to add customizable inline start/end timing inputs (HH:MM) that dynamically render when a break is enabled, and configured a useEffect hook to automatically sync Lunch/Dinner toggles based on the shift start time. Finally, designed and integrated allowed break badges on the active shift cards displaying their custom time ranges.</v>
-      </c>
-      <c r="F17" s="2" t="str">
-        <v>* [COMPLETED] TSK-ATT-012 (Implement Shift Break Configurations &amp; Customizable Timing Windows): Designed and implemented a comprehensive Shift Break Configuration system and customizable timing windows. Added five break toggles and eight break start/end timing columns to the Shift model in the database schema, pushed it via Prisma, and regenerated the client. Refactored backend break start and end routes to enforce shift-specific break configurations and dynamically parse/evaluate break start times against custom shift timing windows rather than hardcoded ranges. Also introduced a brand new 40-minute Dinner Break. Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI, enforcing this via Zod and route intercepts. Overhauled the frontend Shift Management modal to add customizable inline start/end timing inputs (HH:MM) that dynamically render when a break is enabled, and configured a useEffect hook to automatically sync Lunch/Dinner toggles based on the shift start time. Finally, designed and integrated allowed break badges on the active shift cards displaying their custom time ranges.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W37"/>
+  <dimension ref="A1:W40"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="39.83203125" customWidth="1"/>
+    <col min="5" max="5" width="41.83203125" customWidth="1"/>
     <col min="6" max="6" width="30.83203125" customWidth="1"/>
     <col min="7" max="7" width="38.83203125" customWidth="1"/>
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
@@ -4218,14 +4437,227 @@
         <v>Resolved a major overtime calculation bug in the attendance history table by incorporating late check-in penalty minutes. Additionally, implemented Net Worked Minutes (Option B) by subtracting completed break session durations from workedMinutes during checkout, regularization approval, and daily finalization. Refactored the daily finalization scheduler, moving it to 7:00 AM IST and implementing intelligent crash detection: using desktop activity logs, the scheduler marks clean shutdowns without web checkout as HALF_DAY (neglect penalty), but automatically checks out and marks sudden hardware crashes or power cuts as PRESENT (no penalty). Overhauled the frontend WorkdayTimeline summary cards, replacing Events Logged with premium Uptime (since last break/away) and Active Penalties cards. Unified all project contexts under 'The Star Prime' (TSP). Migrated all 48 outlook email identities to the new TSP client inside the PostgreSQL database, successfully preserving all employee email mappings. Cleaned up the obsolete TUT and TEC database client records. Completely redesigned the frontend Team workspace Ongoing Projects and Outlook Emails tabs by removing the obsolete TUT/TEC switcher tabs and showing all lists under TSP. Added dynamic project (magazine and industry) add and delete functionalities directly into the UI with instant state updates and double confirmation boxes. Implemented the Dual-View Task Console for Managers and Team Leads, allowing them to both assign tasks to their team members and receive/complete tasks assigned to them by their superiors. Enabled concurrent dual-fetching of tasks assigned to me and tasks assigned to others, integrated a premium tab switcher globally consistent with the design system, and customized the task cards to dynamically render Assigned by metadata for received tasks. Resolved the AWAY status bug by updating the live-status route to query active break sessions (endTime: null) and correctly classify checked-in employees on break as AWAY. Registered a break-updated global event listener in the frontend AppProvider context to instantly refresh status dots in the Navbar and Sidebar without waiting for the 30-second polling interval. Designed and implemented a comprehensive pre-approval workflow for Paid Overtime. Employees can submit pre-approval requests before 5:00 PM IST on working days by stating their reason in a premium purple-styled modal. Managers, HR, or Admins can approve these requests, transitioning their status to APPROVED. Starting overtime transitions approved sessions to ACTIVE (isPaid: true) while rejected pre-approvals fallback to regular overtime (isPaid: false). Refactored the Attendance History table to render a purple 'Paid' tag next to the overtime hours for all verified paid overtime sessions, ensuring premium visual consistency. Finally, designed and implemented proactive shift-completion warning systems. If an employee attempts to check out of their shift before completing their required working hours (9 hours + any late penalties), they receive a high-visibility, bold red warning card inside the Checkout Modal detailing their shift goals and exact remaining duration. Similarly, if they try to log out of the application session from the topbar, the logout click triggers an alert warning detailing the remaining hours to guarantee compliance. Lastly, designed and implemented a comprehensive dynamic Shift Management system restricted strictly to the ADMIN role. Built a premium React dashboard featuring shift profile cards with timing and grace period metrics, a shift creation/editing form, and a search-and-filter Employee Shift Switcher directory supporting bulk shift assignments. Secured the app layout by rendering the sidebar link only for administrators, and updated backend employee queries to return their active shift. All check-in delays, grace penalties, and overtime required hours automatically recalculate in real-time according to the employee's dynamically assigned shift. In addition, designed and implemented a comprehensive Shift Break Configuration system and Dinner Break provision. Added five database-synced break toggles (hasBreaks, allowMorningTea, allowLunch, allowEveningTea, allowDinner) to the Shift model. Refactored backend break start and end routes to enforce shift-specific break configurations. Toggling breaks off globally blocks employees from starting breaks. When breaks are enabled, starting or ending a break dynamically enforces allowed durations per shift. Also introduced a new 40-minute Dinner Break window (20:00 - 22:00 IST). Restricted Lunch breaks exclusively to morning shifts (start time before 12 PM) and Dinner breaks exclusively to night shifts (start time 12 PM or later) in both the backend APIs and frontend UI. Updated the frontend Shift Management modal with a main toggle and a dynamic sub-checkbox grid that automatically syncs and conditionally renders Lunch or Dinner based on the shift start time. Finally, designed and integrated premium allowed break badges onto the active shift cards. Furthermore, designed and implemented customizable break start and end timings per shift profile. Added 8 break-timing columns (start and end times for all 4 break types) with defaults to the database schema, successfully ran db push, and regenerated the Prisma Client. Updated the backend Zod validator and Express routes to check timing inputs, and refactored the break end handler to parse and evaluate employee breaks dynamically against these custom shift-level windows. Lastly, updated the frontend Shift Management page modal to render inline start/end timing inputs when a break is enabled, and updated the shift cards to display these custom ranges alongside the break badges.</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="B38" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C38" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D38" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E38" s="2" t="str">
+        <v>Employee Profile Page — Attendance Tab</v>
+      </c>
+      <c r="F38" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G38" s="2" t="str">
+        <v>Profile Attendance Accuracy</v>
+      </c>
+      <c r="H38" s="2" t="str">
+        <v>TSK-ATT-013</v>
+      </c>
+      <c r="I38" s="2" t="str">
+        <v>Fix Weekend Attendance Accuracy: DB Cleanup, Status Priority &amp; Dynamic Exceptions Fetching</v>
+      </c>
+      <c r="J38" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K38" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L38" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="M38" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="N38" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O38" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P38" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>5.333333333333333</v>
+      </c>
+      <c r="R38" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S38" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T38" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U38" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="V38" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="W38" s="2" t="str">
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends.</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="B39" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C39" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D39" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E39" s="2" t="str">
+        <v>Attendance Page &amp; Employee Directory</v>
+      </c>
+      <c r="F39" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G39" s="2" t="str">
+        <v>Real-time Telemetry &amp; Timeline</v>
+      </c>
+      <c r="H39" s="2" t="str">
+        <v>TSK-ATT-014</v>
+      </c>
+      <c r="I39" s="2" t="str">
+        <v>Fix Timezone Mismatches in Attendance Timeline &amp; Progress Bars</v>
+      </c>
+      <c r="J39" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K39" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L39" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="M39" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N39" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O39" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P39" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q39" s="2">
+        <v>5.333333333333333</v>
+      </c>
+      <c r="R39" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S39" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T39" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U39" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="V39" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="W39" s="2" t="str">
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends.</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="B40" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C40" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D40" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E40" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F40" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G40" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H40" s="2" t="str">
+        <v>TSK-ATT-015</v>
+      </c>
+      <c r="I40" s="2" t="str">
+        <v>Work on task</v>
+      </c>
+      <c r="J40" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K40" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L40" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M40" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N40" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="O40" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P40" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="2">
+        <v>5.333333333333333</v>
+      </c>
+      <c r="R40" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S40" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T40" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U40" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="V40" s="2" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="W40" s="2" t="str">
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W40"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H6"/>
   <cols>
@@ -4402,7 +4834,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L4"/>
   <cols>
@@ -4579,7 +5011,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I5"/>
   <cols>
@@ -4746,7 +5178,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I13"/>
   <cols>
@@ -5145,7 +5577,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F7"/>
   <cols>
@@ -5304,7 +5736,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G7"/>
   <cols>
@@ -5483,163 +5915,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="29.83203125" customWidth="1"/>
-    <col min="3" max="3" width="58.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="3" t="str">
-        <v>Table</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Relationships</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>Indexes</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>Migration</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>Seed Data</v>
-      </c>
-      <c r="F1" s="3" t="str">
-        <v>Completion %</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="str">
-        <v>User / Role</v>
-      </c>
-      <c r="B2" s="2" t="str">
-        <v>Role 1:N User</v>
-      </c>
-      <c r="C2" s="2" t="str">
-        <v>users.email (unique), users.roleId</v>
-      </c>
-      <c r="D2" s="2" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="E2" s="2" t="str">
-        <v>Seeded</v>
-      </c>
-      <c r="F2" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v>Employee</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>User 1:1 Employee</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>employees.employeeCode (unique), employees.departmentId</v>
-      </c>
-      <c r="D3" s="2" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v>Seeded</v>
-      </c>
-      <c r="F3" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="str">
-        <v>Attendance</v>
-      </c>
-      <c r="B4" s="2" t="str">
-        <v>Employee 1:N Attendance</v>
-      </c>
-      <c r="C4" s="2" t="str">
-        <v>(employeeId, attendanceDate) unique</v>
-      </c>
-      <c r="D4" s="2" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="E4" s="2" t="str">
-        <v>Seeded</v>
-      </c>
-      <c r="F4" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="str">
-        <v>LeaveRequest</v>
-      </c>
-      <c r="B5" s="2" t="str">
-        <v>Employee 1:N LeaveRequest</v>
-      </c>
-      <c r="C5" s="2" t="str">
-        <v>leave_requests.employeeId, leave_requests.status</v>
-      </c>
-      <c r="D5" s="2" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="E5" s="2" t="str">
-        <v>Seeded</v>
-      </c>
-      <c r="F5" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="str">
-        <v>PayrollRecord</v>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v>Employee 1:N PayrollRecord</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v>(employeeId, month, year) unique</v>
-      </c>
-      <c r="D6" s="2" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="E6" s="2" t="str">
-        <v>Seeded</v>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="str">
-        <v>RefreshTokens</v>
-      </c>
-      <c r="B7" s="2" t="str">
-        <v>User 1:N RefreshTokens</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v>refresh_tokens.userId</v>
-      </c>
-      <c r="D7" s="2" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="F7" s="2" t="str">
-        <v>100%</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: shift management create shift popup inputs and AM/PM toggle vertical alignment centering
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -4487,7 +4487,7 @@
         <v>3</v>
       </c>
       <c r="Q38" s="2">
-        <v>5.333333333333333</v>
+        <v>5.666666666666667</v>
       </c>
       <c r="R38" s="2" t="str">
         <v>100%</v>
@@ -4505,7 +4505,7 @@
         <v>2026-06-29</v>
       </c>
       <c r="W38" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Finally, fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1.</v>
       </c>
     </row>
     <row r="39">
@@ -4558,7 +4558,7 @@
         <v>2</v>
       </c>
       <c r="Q39" s="2">
-        <v>5.333333333333333</v>
+        <v>5.666666666666667</v>
       </c>
       <c r="R39" s="2" t="str">
         <v>100%</v>
@@ -4576,7 +4576,7 @@
         <v>2026-06-29</v>
       </c>
       <c r="W39" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Finally, fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1.</v>
       </c>
     </row>
     <row r="40">
@@ -4629,7 +4629,7 @@
         <v>0</v>
       </c>
       <c r="Q40" s="2">
-        <v>5.333333333333333</v>
+        <v>5.666666666666667</v>
       </c>
       <c r="R40" s="2" t="str">
         <v>100%</v>
@@ -4647,7 +4647,7 @@
         <v>2026-06-29</v>
       </c>
       <c r="W40" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Finally, fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: enforce 1-5 minutes points-only penalty for check-ins and breaks
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -4487,7 +4487,7 @@
         <v>3</v>
       </c>
       <c r="Q38" s="2">
-        <v>5.666666666666667</v>
+        <v>6</v>
       </c>
       <c r="R38" s="2" t="str">
         <v>100%</v>
@@ -4505,7 +4505,7 @@
         <v>2026-06-29</v>
       </c>
       <c r="W38" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Finally, fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Finally, updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes.</v>
       </c>
     </row>
     <row r="39">
@@ -4558,7 +4558,7 @@
         <v>2</v>
       </c>
       <c r="Q39" s="2">
-        <v>5.666666666666667</v>
+        <v>6</v>
       </c>
       <c r="R39" s="2" t="str">
         <v>100%</v>
@@ -4576,7 +4576,7 @@
         <v>2026-06-29</v>
       </c>
       <c r="W39" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Finally, fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Finally, updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes.</v>
       </c>
     </row>
     <row r="40">
@@ -4629,7 +4629,7 @@
         <v>0</v>
       </c>
       <c r="Q40" s="2">
-        <v>5.666666666666667</v>
+        <v>6</v>
       </c>
       <c r="R40" s="2" t="str">
         <v>100%</v>
@@ -4647,7 +4647,7 @@
         <v>2026-06-29</v>
       </c>
       <c r="W40" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Finally, fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Finally, updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(topbar): swap navbar button states, remove shadows, and update workday timeline progress bounds
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -4505,7 +4505,7 @@
         <v>2026-06-29</v>
       </c>
       <c r="W38" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Finally, updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes. Additionally, restyled the topbar elements in Navbar.css to a monochrome theme with 12px container font size, round buttons, and darker required duration label. Added dynamic click-to-view points history log list in Navbar.tsx. Prevented background scrolling while any modal popup is open in Modal.tsx. Aligned points history modal font sizes to 12px. Combined the Previous Winner and Current Leaderboard panels into a single, cohesive parent hero card on the Leaderboard page with a nested card layout styling. Updated the leaderboard ranking row avatars to display the employee's uploaded profile image matching the profile page, or render initials using a dynamic Android-like background color uniquely mapped to each employee id. Implemented a prominent purple highlight line and 'You' pill badge on the logged-in employee's ranking row. Added a gamified 'Your Standing' summary bar above each of the three ranking lists, displaying the user's current rank standing, relative percentile tier, and the distance in points or hours required to overtake the rank directly above them. Implemented Yesterday and View by Month shortcuts (ordered: Date Picker, Yesterday button, Month dropdown styled with a custom Chevron Down arrow) on the Attendance page filters, with corresponding backend query-builder updates to support filtering employee history by monthly ranges. Updated the Workday Timeline modal header title to dynamically print the name of the target employee being viewed. Resolved a major telemetry date linkage bug where selecting a previous date in the Attendance History section caused the Workforce Live Status timeline button to fetch and display that historical date's logs; fixed by refactoring the timeline click handler to asynchronously fetch the target employee's actual today's record directly from the backend, and decoupled the timeline button disabled state from the historical attendance list. Updated the WorkdayTimeline progress bar footer labels to show the employee's actual check-in time on the left, and the final shift end time (adding any late penalty minutes to the standard shift end time) on the right. Finally, swapped the normal and hover CSS state properties of the topbar buttons (notifications, profile, and logout) in Navbar.css so they are raised by default and become flat on hover.</v>
       </c>
     </row>
     <row r="39">
@@ -4576,7 +4576,7 @@
         <v>2026-06-29</v>
       </c>
       <c r="W39" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Finally, updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes. Additionally, restyled the topbar elements in Navbar.css to a monochrome theme with 12px container font size, round buttons, and darker required duration label. Added dynamic click-to-view points history log list in Navbar.tsx. Prevented background scrolling while any modal popup is open in Modal.tsx. Aligned points history modal font sizes to 12px. Combined the Previous Winner and Current Leaderboard panels into a single, cohesive parent hero card on the Leaderboard page with a nested card layout styling. Updated the leaderboard ranking row avatars to display the employee's uploaded profile image matching the profile page, or render initials using a dynamic Android-like background color uniquely mapped to each employee id. Implemented a prominent purple highlight line and 'You' pill badge on the logged-in employee's ranking row. Added a gamified 'Your Standing' summary bar above each of the three ranking lists, displaying the user's current rank standing, relative percentile tier, and the distance in points or hours required to overtake the rank directly above them. Implemented Yesterday and View by Month shortcuts (ordered: Date Picker, Yesterday button, Month dropdown styled with a custom Chevron Down arrow) on the Attendance page filters, with corresponding backend query-builder updates to support filtering employee history by monthly ranges. Updated the Workday Timeline modal header title to dynamically print the name of the target employee being viewed. Resolved a major telemetry date linkage bug where selecting a previous date in the Attendance History section caused the Workforce Live Status timeline button to fetch and display that historical date's logs; fixed by refactoring the timeline click handler to asynchronously fetch the target employee's actual today's record directly from the backend, and decoupled the timeline button disabled state from the historical attendance list. Updated the WorkdayTimeline progress bar footer labels to show the employee's actual check-in time on the left, and the final shift end time (adding any late penalty minutes to the standard shift end time) on the right. Finally, swapped the normal and hover CSS state properties of the topbar buttons (notifications, profile, and logout) in Navbar.css so they are raised by default and become flat on hover.</v>
       </c>
     </row>
     <row r="40">
@@ -4647,7 +4647,7 @@
         <v>2026-06-29</v>
       </c>
       <c r="W40" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Finally, updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes. Additionally, restyled the topbar elements in Navbar.css to a monochrome theme with 12px container font size, round buttons, and darker required duration label. Added dynamic click-to-view points history log list in Navbar.tsx. Prevented background scrolling while any modal popup is open in Modal.tsx. Aligned points history modal font sizes to 12px. Combined the Previous Winner and Current Leaderboard panels into a single, cohesive parent hero card on the Leaderboard page with a nested card layout styling. Updated the leaderboard ranking row avatars to display the employee's uploaded profile image matching the profile page, or render initials using a dynamic Android-like background color uniquely mapped to each employee id. Implemented a prominent purple highlight line and 'You' pill badge on the logged-in employee's ranking row. Added a gamified 'Your Standing' summary bar above each of the three ranking lists, displaying the user's current rank standing, relative percentile tier, and the distance in points or hours required to overtake the rank directly above them. Implemented Yesterday and View by Month shortcuts (ordered: Date Picker, Yesterday button, Month dropdown styled with a custom Chevron Down arrow) on the Attendance page filters, with corresponding backend query-builder updates to support filtering employee history by monthly ranges. Updated the Workday Timeline modal header title to dynamically print the name of the target employee being viewed. Resolved a major telemetry date linkage bug where selecting a previous date in the Attendance History section caused the Workforce Live Status timeline button to fetch and display that historical date's logs; fixed by refactoring the timeline click handler to asynchronously fetch the target employee's actual today's record directly from the backend, and decoupled the timeline button disabled state from the historical attendance list. Updated the WorkdayTimeline progress bar footer labels to show the employee's actual check-in time on the left, and the final shift end time (adding any late penalty minutes to the standard shift end time) on the right. Finally, swapped the normal and hover CSS state properties of the topbar buttons (notifications, profile, and logout) in Navbar.css so they are raised by default and become flat on hover.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: update daily logs, task lists, and synchronize HRMS_Project_Management.xlsx
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F22"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -849,9 +849,49 @@
         <v>* [COMPLETED] TSK-ATT-015 (Enforce Desktop Client Continuous Tracking): Enforced desktop client telemetry tracking to prevent users from bypassing tracking or disconnecting manually. Removed the Disconnect button from the Dashboard UI and the Exit context menu from the system tray icon to ensure the app cannot be manually closed or logged out of. Implemented a registry key injection on application start to automatically register the client as a Windows startup application (HKCU\SOFTWARE\Microsoft\Windows\CurrentVersion\Run).</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B21" s="2" t="str">
+        <v>TSK-DEPT-001</v>
+      </c>
+      <c r="C21" s="2" t="str">
+        <v>Redesign Departments Page with Box Structure and Employee Counts</v>
+      </c>
+      <c r="D21" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E21" s="2" t="str">
+        <v>Redesigned the Departments page to display a grid of premium cards instead of a table list. Updated the backend /departments API to include the active employee count via Prisma relations. The frontend cards render modern linear-gradient avatars, pill-shaped code badges, and hover lift effects.</v>
+      </c>
+      <c r="F21" s="2" t="str">
+        <v>* [COMPLETED] TSK-DEPT-001 (Redesign Departments Page with Box Structure and Employee Counts): Redesigned the Departments page to display a grid of premium cards instead of a table list. Updated the backend /departments API to include the active employee count via Prisma relations. The frontend cards render modern linear-gradient avatars, pill-shaped code badges, and hover lift effects.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B22" s="2" t="str">
+        <v>TSK-LDB-002</v>
+      </c>
+      <c r="C22" s="2" t="str">
+        <v>Refine Leaderboard Previous Winner Card, Avatars, and Button Themes</v>
+      </c>
+      <c r="D22" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E22" s="2" t="str">
+        <v>Refined the Previous Winner card on the Leaderboard page to be a square block taking exactly half the parent height on desktop, with responsive overrides for mobile. Replaced the trophy emoji with a party popper emoji featuring a custom scale-and-sway animation. Updated the employee ranking list avatars to use the same 6 premium linear gradients. Finally, unified the button design across the app by updating the Add Department and Add Employee buttons to use the dark blue accent gradient, 16px border-radius, and custom glow shadows.</v>
+      </c>
+      <c r="F22" s="2" t="str">
+        <v>* [COMPLETED] TSK-LDB-002 (Refine Leaderboard Previous Winner Card, Avatars, and Button Themes): Refined the Previous Winner card on the Leaderboard page to be a square block taking exactly half the parent height on desktop, with responsive overrides for mobile. Replaced the trophy emoji with a party popper emoji featuring a custom scale-and-sway animation. Updated the employee ranking list avatars to use the same 6 premium linear gradients. Finally, unified the button design across the app by updating the Add Department and Add Employee buttons to use the dark blue accent gradient, 16px border-radius, and custom glow shadows.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F22"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1783,7 +1823,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W40"/>
+  <dimension ref="A1:W42"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -4505,7 +4545,7 @@
         <v>2026-06-29</v>
       </c>
       <c r="W38" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes. Additionally, restyled the topbar elements in Navbar.css to a monochrome theme with 12px container font size, round buttons, and darker required duration label. Added dynamic click-to-view points history log list in Navbar.tsx. Prevented background scrolling while any modal popup is open in Modal.tsx. Aligned points history modal font sizes to 12px. Combined the Previous Winner and Current Leaderboard panels into a single, cohesive parent hero card on the Leaderboard page with a nested card layout styling. Updated the leaderboard ranking row avatars to display the employee's uploaded profile image matching the profile page, or render initials using a dynamic Android-like background color uniquely mapped to each employee id. Implemented a prominent purple highlight line and 'You' pill badge on the logged-in employee's ranking row. Added a gamified 'Your Standing' summary bar above each of the three ranking lists, displaying the user's current rank standing, relative percentile tier, and the distance in points or hours required to overtake the rank directly above them. Implemented Yesterday and View by Month shortcuts (ordered: Date Picker, Yesterday button, Month dropdown styled with a custom Chevron Down arrow) on the Attendance page filters, with corresponding backend query-builder updates to support filtering employee history by monthly ranges. Updated the Workday Timeline modal header title to dynamically print the name of the target employee being viewed. Resolved a major telemetry date linkage bug where selecting a previous date in the Attendance History section caused the Workforce Live Status timeline button to fetch and display that historical date's logs; fixed by refactoring the timeline click handler to asynchronously fetch the target employee's actual today's record directly from the backend, and decoupled the timeline button disabled state from the historical attendance list. Updated the WorkdayTimeline progress bar footer labels to show the employee's actual check-in time on the left, and the final shift end time (adding any late penalty minutes to the standard shift end time) on the right. Finally, swapped the normal and hover CSS state properties of the topbar buttons (notifications, profile, and logout) in Navbar.css so they are raised by default and become flat on hover.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings returned by the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes. Additionally, restyled the topbar elements in Navbar.css to a monochrome theme with 12px container font size, round buttons, and darker required duration label. Added dynamic click-to-view points history log list in Navbar.tsx. Prevented background scrolling while any modal popup is open in Modal.tsx. Aligned points history modal font sizes to 12px. Combined the Previous Winner and Current Leaderboard panels into a single, cohesive parent hero card on the Leaderboard page with a nested card layout styling. Updated the leaderboard ranking row avatars to display the employee's uploaded profile image matching the profile page, or render initials using a dynamic Android-like background color uniquely mapped to each employee id. Implemented a prominent purple highlight line and 'You' pill badge on the logged-in employee's ranking row. Added a gamified 'Your Standing' summary bar above each of the three ranking lists, displaying the user's current rank standing, relative percentile tier, and the distance in points or hours required to overtake the rank directly above them. Implemented Yesterday and View by Month shortcuts (ordered: Date Picker, Yesterday button, Month dropdown styled with a custom Chevron Down arrow) on the Attendance page filters, with corresponding backend query-builder updates to support filtering employee history by monthly ranges. Updated the Workday Timeline modal header title to dynamically print the name of the target employee being viewed. Resolved a major telemetry date linkage bug where selecting a previous date in the Attendance History section caused the Workforce Live Status timeline button to fetch and display that historical date's logs; fixed by refactoring the timeline click handler to asynchronously fetch the target employee's actual today's record directly from the backend, and decoupled the timeline button disabled state from the historical attendance list. Updated the WorkdayTimeline progress bar footer labels to show the employee's actual check-in time on the left, and the final shift end time (adding any late penalty minutes to the standard shift end time) on the right. Finally, swapped the normal and hover CSS state properties of the topbar buttons (notifications, profile, and logout) in Navbar.css so they are raised by default and become flat on hover.</v>
       </c>
     </row>
     <row r="39">
@@ -4576,7 +4616,7 @@
         <v>2026-06-29</v>
       </c>
       <c r="W39" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes. Additionally, restyled the topbar elements in Navbar.css to a monochrome theme with 12px container font size, round buttons, and darker required duration label. Added dynamic click-to-view points history log list in Navbar.tsx. Prevented background scrolling while any modal popup is open in Modal.tsx. Aligned points history modal font sizes to 12px. Combined the Previous Winner and Current Leaderboard panels into a single, cohesive parent hero card on the Leaderboard page with a nested card layout styling. Updated the leaderboard ranking row avatars to display the employee's uploaded profile image matching the profile page, or render initials using a dynamic Android-like background color uniquely mapped to each employee id. Implemented a prominent purple highlight line and 'You' pill badge on the logged-in employee's ranking row. Added a gamified 'Your Standing' summary bar above each of the three ranking lists, displaying the user's current rank standing, relative percentile tier, and the distance in points or hours required to overtake the rank directly above them. Implemented Yesterday and View by Month shortcuts (ordered: Date Picker, Yesterday button, Month dropdown styled with a custom Chevron Down arrow) on the Attendance page filters, with corresponding backend query-builder updates to support filtering employee history by monthly ranges. Updated the Workday Timeline modal header title to dynamically print the name of the target employee being viewed. Resolved a major telemetry date linkage bug where selecting a previous date in the Attendance History section caused the Workforce Live Status timeline button to fetch and display that historical date's logs; fixed by refactoring the timeline click handler to asynchronously fetch the target employee's actual today's record directly from the backend, and decoupled the timeline button disabled state from the historical attendance list. Updated the WorkdayTimeline progress bar footer labels to show the employee's actual check-in time on the left, and the final shift end time (adding any late penalty minutes to the standard shift end time) on the right. Finally, swapped the normal and hover CSS state properties of the topbar buttons (notifications, profile, and logout) in Navbar.css so they are raised by default and become flat on hover.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings returned by the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes. Additionally, restyled the topbar elements in Navbar.css to a monochrome theme with 12px container font size, round buttons, and darker required duration label. Added dynamic click-to-view points history log list in Navbar.tsx. Prevented background scrolling while any modal popup is open in Modal.tsx. Aligned points history modal font sizes to 12px. Combined the Previous Winner and Current Leaderboard panels into a single, cohesive parent hero card on the Leaderboard page with a nested card layout styling. Updated the leaderboard ranking row avatars to display the employee's uploaded profile image matching the profile page, or render initials using a dynamic Android-like background color uniquely mapped to each employee id. Implemented a prominent purple highlight line and 'You' pill badge on the logged-in employee's ranking row. Added a gamified 'Your Standing' summary bar above each of the three ranking lists, displaying the user's current rank standing, relative percentile tier, and the distance in points or hours required to overtake the rank directly above them. Implemented Yesterday and View by Month shortcuts (ordered: Date Picker, Yesterday button, Month dropdown styled with a custom Chevron Down arrow) on the Attendance page filters, with corresponding backend query-builder updates to support filtering employee history by monthly ranges. Updated the Workday Timeline modal header title to dynamically print the name of the target employee being viewed. Resolved a major telemetry date linkage bug where selecting a previous date in the Attendance History section caused the Workforce Live Status timeline button to fetch and display that historical date's logs; fixed by refactoring the timeline click handler to asynchronously fetch the target employee's actual today's record directly from the backend, and decoupled the timeline button disabled state from the historical attendance list. Updated the WorkdayTimeline progress bar footer labels to show the employee's actual check-in time on the left, and the final shift end time (adding any late penalty minutes to the standard shift end time) on the right. Finally, swapped the normal and hover CSS state properties of the topbar buttons (notifications, profile, and logout) in Navbar.css so they are raised by default and become flat on hover.</v>
       </c>
     </row>
     <row r="40">
@@ -4647,12 +4687,154 @@
         <v>2026-06-29</v>
       </c>
       <c r="W40" s="2" t="str">
-        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings from the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes. Additionally, restyled the topbar elements in Navbar.css to a monochrome theme with 12px container font size, round buttons, and darker required duration label. Added dynamic click-to-view points history log list in Navbar.tsx. Prevented background scrolling while any modal popup is open in Modal.tsx. Aligned points history modal font sizes to 12px. Combined the Previous Winner and Current Leaderboard panels into a single, cohesive parent hero card on the Leaderboard page with a nested card layout styling. Updated the leaderboard ranking row avatars to display the employee's uploaded profile image matching the profile page, or render initials using a dynamic Android-like background color uniquely mapped to each employee id. Implemented a prominent purple highlight line and 'You' pill badge on the logged-in employee's ranking row. Added a gamified 'Your Standing' summary bar above each of the three ranking lists, displaying the user's current rank standing, relative percentile tier, and the distance in points or hours required to overtake the rank directly above them. Implemented Yesterday and View by Month shortcuts (ordered: Date Picker, Yesterday button, Month dropdown styled with a custom Chevron Down arrow) on the Attendance page filters, with corresponding backend query-builder updates to support filtering employee history by monthly ranges. Updated the Workday Timeline modal header title to dynamically print the name of the target employee being viewed. Resolved a major telemetry date linkage bug where selecting a previous date in the Attendance History section caused the Workforce Live Status timeline button to fetch and display that historical date's logs; fixed by refactoring the timeline click handler to asynchronously fetch the target employee's actual today's record directly from the backend, and decoupled the timeline button disabled state from the historical attendance list. Updated the WorkdayTimeline progress bar footer labels to show the employee's actual check-in time on the left, and the final shift end time (adding any late penalty minutes to the standard shift end time) on the right. Finally, swapped the normal and hover CSS state properties of the topbar buttons (notifications, profile, and logout) in Navbar.css so they are raised by default and become flat on hover.</v>
+        <v>Investigated and fixed the root cause of Saturdays showing as Absent on the employee profile attendance history page. Refactored the frontend status resolution hierarchy in EmployeeAttendanceTab to ensure OFF days and LEAVE always override rogue ABSENT records. Lifted the selectedMonth and selectedYear state to EmployeeProfilePage so that calendar exceptions are re-fetched dynamically on month/year change. Resolved a timezone shift bug where UTC attendanceDate strings returned by the backend shifted by one day when parsed locally in the browser, causing today's check-in to display on yesterday's profile row. Also fixed date.toISOString() serialization inside unifiedHistory mapping which converted the local midnight date to UTC (shifting it back by one day). Resolved a bug where several instantiations of the WorkdayTimeline component were missing the employeeId and token props, which prevented it from fetching desktop logs. Resolved a bug where the timeline defaulted to 9:00 AM - 6:00 PM shift settings for all users. Fixed by including the shift relation in the backend API query and passing down shift timings/grace period props to correctly calculate bounds and late thresholds. Set all 33 employees to the Day Shift in the database and recalculated late status and penalties for all today's records. Updated the Day Summary grid list style in WorkdayTimeline.css. Refactored worked minutes to dynamically calculate true productive minutes by subtracting breaks and idle/locked segments. Added an elapsed time counter next to the worked label in the timeline header. Resolved check-in/checkout tag arrow alignment issues when tooltips are horizontally shifted due to viewport constraints by introducing dynamic CSS custom properties. Implemented Windows registry injection to ensure the desktop telemetry client runs silently on system boot, while retaining manual disconnect/exit options per user preference and verifying that the authentication token correctly persists locally so the application does not automatically log out upon restart. Also resolved the sleep event tracking bug where PC suspend interrupted the network call by refactoring the desktop logger to write sleep/wake events to disk synchronously first before attempting background uploads, ensuring offline safety during suspends. Fixed layout alignment bugs inside the Create/Edit Shift Profile modal where custom and standard time inputs were not vertically centered by refactoring the time input container to use flex vertical centering and setting input heights to auto and line-heights to 1. Updated both shift check-in and break end routes to enforce no grace period (any lateness is tracked), applying only a points deduction (-1 point) and zero extended shift time (0 penalty minutes) for lateness up to 5 minutes, with full time penalties starting at 6+ minutes. Additionally, restyled the topbar elements in Navbar.css to a monochrome theme with 12px container font size, round buttons, and darker required duration label. Added dynamic click-to-view points history log list in Navbar.tsx. Prevented background scrolling while any modal popup is open in Modal.tsx. Aligned points history modal font sizes to 12px. Combined the Previous Winner and Current Leaderboard panels into a single, cohesive parent hero card on the Leaderboard page with a nested card layout styling. Updated the leaderboard ranking row avatars to display the employee's uploaded profile image matching the profile page, or render initials using a dynamic Android-like background color uniquely mapped to each employee id. Implemented a prominent purple highlight line and 'You' pill badge on the logged-in employee's ranking row. Added a gamified 'Your Standing' summary bar above each of the three ranking lists, displaying the user's current rank standing, relative percentile tier, and the distance in points or hours required to overtake the rank directly above them. Implemented Yesterday and View by Month shortcuts (ordered: Date Picker, Yesterday button, Month dropdown styled with a custom Chevron Down arrow) on the Attendance page filters, with corresponding backend query-builder updates to support filtering employee history by monthly ranges. Updated the Workday Timeline modal header title to dynamically print the name of the target employee being viewed. Resolved a major telemetry date linkage bug where selecting a previous date in the Attendance History section caused the Workforce Live Status timeline button to fetch and display that historical date's logs; fixed by refactoring the timeline click handler to asynchronously fetch the target employee's actual today's record directly from the backend, and decoupled the timeline button disabled state from the historical attendance list. Updated the WorkdayTimeline progress bar footer labels to show the employee's actual check-in time on the left, and the final shift end time (adding any late penalty minutes to the standard shift end time) on the right. Finally, swapped the normal and hover CSS state properties of the topbar buttons (notifications, profile, and logout) in Navbar.css so they are raised by default and become flat on hover.</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B41" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C41" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D41" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E41" s="2" t="str">
+        <v>Departments Page</v>
+      </c>
+      <c r="F41" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G41" s="2" t="str">
+        <v>Departments Redesign</v>
+      </c>
+      <c r="H41" s="2" t="str">
+        <v>TSK-DEPT-001</v>
+      </c>
+      <c r="I41" s="2" t="str">
+        <v>Redesign Departments Page with Box Structure and Employee Counts</v>
+      </c>
+      <c r="J41" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K41" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L41" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M41" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="N41" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O41" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P41" s="2">
+        <v>6</v>
+      </c>
+      <c r="Q41" s="2">
+        <v>4</v>
+      </c>
+      <c r="R41" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S41" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T41" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U41" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="V41" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="W41" s="2" t="str">
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department and Add Employee buttons to use the dark blue accent gradient, 16px border-radius, and custom glow shadows.</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B42" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C42" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D42" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E42" s="2" t="str">
+        <v>Leaderboard Page</v>
+      </c>
+      <c r="F42" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G42" s="2" t="str">
+        <v>Leaderboard Refinements</v>
+      </c>
+      <c r="H42" s="2" t="str">
+        <v>TSK-LDB-002</v>
+      </c>
+      <c r="I42" s="2" t="str">
+        <v>Refine Leaderboard Previous Winner Card, Avatars, and Button Themes</v>
+      </c>
+      <c r="J42" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K42" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L42" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M42" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N42" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O42" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P42" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q42" s="2">
+        <v>4</v>
+      </c>
+      <c r="R42" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S42" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T42" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U42" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="V42" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="W42" s="2" t="str">
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department and Add Employee buttons to use the dark blue accent gradient, 16px border-radius, and custom glow shadows.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W42"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: refine workday header, premium button styles, shift-employee assignment, test account seeding, and mobile menu clickability
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F24"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -889,9 +889,49 @@
         <v>* [COMPLETED] TSK-LDB-002 (Refine Leaderboard Previous Winner Card, Avatars, and Button Themes): Refined the Previous Winner card on the Leaderboard page to be a square block taking exactly half the parent height on desktop, with responsive overrides for mobile. Replaced the trophy emoji with a party popper emoji featuring a custom scale-and-sway animation. Updated the employee ranking list avatars to use the same 6 premium linear gradients. Finally, unified the button design across the app by updating the Add Department and Add Employee buttons to use the dark blue accent gradient, 16px border-radius, and custom glow shadows.</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B23" s="2" t="str">
+        <v>TSK-ATT-016</v>
+      </c>
+      <c r="C23" s="2" t="str">
+        <v>Refine Workday Progress Header Layout and Handle Not-Checked-In State</v>
+      </c>
+      <c r="D23" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E23" s="2" t="str">
+        <v>Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail.</v>
+      </c>
+      <c r="F23" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-016 (Refine Workday Progress Header Layout and Handle Not-Checked-In State): Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B24" s="2" t="str">
+        <v>TSK-EMP-005</v>
+      </c>
+      <c r="C24" s="2" t="str">
+        <v>Align Button Themes on Payroll/Leaves Pages and Seed Test Accounts</v>
+      </c>
+      <c r="D24" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E24" s="2" t="str">
+        <v>Unified the button styling across the app by transforming the Create Record, View Team Calendar, View Leave Balances, and Apply for Leave buttons to use the dark blue accent gradient and outline themes with high contrast. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances.</v>
+      </c>
+      <c r="F24" s="2" t="str">
+        <v>* [COMPLETED] TSK-EMP-005 (Align Button Themes on Payroll/Leaves Pages and Seed Test Accounts): Unified the button styling across the app by transforming the Create Record, View Team Calendar, View Leave Balances, and Apply for Leave buttons to use the dark blue accent gradient and outline themes with high contrast. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1823,7 +1863,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W42"/>
+  <dimension ref="A1:W44"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -1831,7 +1871,7 @@
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="41.83203125" customWidth="1"/>
     <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="38.83203125" customWidth="1"/>
+    <col min="7" max="7" width="61.83203125" customWidth="1"/>
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
     <col min="9" max="9" width="65.83203125" customWidth="1"/>
     <col min="10" max="10" width="18.83203125" customWidth="1"/>
@@ -4740,7 +4780,7 @@
         <v>6</v>
       </c>
       <c r="Q41" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R41" s="2" t="str">
         <v>100%</v>
@@ -4758,7 +4798,7 @@
         <v>2026-06-30</v>
       </c>
       <c r="W41" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department and Add Employee buttons to use the dark blue accent gradient, 16px border-radius, and custom glow shadows.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, and Apply for Leave buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances.</v>
       </c>
     </row>
     <row r="42">
@@ -4811,7 +4851,7 @@
         <v>4</v>
       </c>
       <c r="Q42" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R42" s="2" t="str">
         <v>100%</v>
@@ -4829,12 +4869,154 @@
         <v>2026-06-30</v>
       </c>
       <c r="W42" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department and Add Employee buttons to use the dark blue accent gradient, 16px border-radius, and custom glow shadows.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, and Apply for Leave buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances.</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B43" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C43" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D43" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E43" s="2" t="str">
+        <v>Dashboard Page &amp; Live Status Tracking</v>
+      </c>
+      <c r="F43" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G43" s="2" t="str">
+        <v>Workday Progress Header Alignment and Not-Checked-In State</v>
+      </c>
+      <c r="H43" s="2" t="str">
+        <v>TSK-ATT-016</v>
+      </c>
+      <c r="I43" s="2" t="str">
+        <v>Refine Workday Progress Header Layout and Handle Not-Checked-In State</v>
+      </c>
+      <c r="J43" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K43" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L43" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M43" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N43" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O43" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P43" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q43" s="2">
+        <v>3</v>
+      </c>
+      <c r="R43" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S43" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T43" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U43" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="V43" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="W43" s="2" t="str">
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, and Apply for Leave buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances.</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B44" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C44" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D44" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E44" s="2" t="str">
+        <v>Payroll &amp; Leaves Pages &amp; Seeding</v>
+      </c>
+      <c r="F44" s="2" t="str">
+        <v>Employee Management</v>
+      </c>
+      <c r="G44" s="2" t="str">
+        <v>Button Theme Alignments &amp; Test Account Seeding</v>
+      </c>
+      <c r="H44" s="2" t="str">
+        <v>TSK-EMP-005</v>
+      </c>
+      <c r="I44" s="2" t="str">
+        <v>Align Button Themes on Payroll/Leaves Pages and Seed Test Accounts</v>
+      </c>
+      <c r="J44" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K44" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L44" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="M44" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N44" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O44" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P44" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q44" s="2">
+        <v>3</v>
+      </c>
+      <c r="R44" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S44" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T44" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U44" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="V44" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="W44" s="2" t="str">
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, and Apply for Leave buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W44"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: update project tracking and sync Excel sheet for z-index, download confirmation, and calendar back button
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F26"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -929,9 +929,49 @@
         <v>* [COMPLETED] TSK-EMP-005 (Align Button Themes on Payroll/Leaves Pages and Seed Test Accounts): Unified the button styling across the app by transforming the Create Record, View Team Calendar, View Leave Balances, and Apply for Leave buttons to use the dark blue accent gradient and outline themes with high contrast. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances.</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B25" s="2" t="str">
+        <v>TSK-NAV-004</v>
+      </c>
+      <c r="C25" s="2" t="str">
+        <v>Refine Navigation Layouts: Mobile Z-Index, Download Confirmation, and Conditional Back Button</v>
+      </c>
+      <c r="D25" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E25" s="2" t="str">
+        <v>Refined mobile navigation layouts. Solved mobile sidebar menu clickability by increasing the sidebar's z-index to 1810 to place it in front of the backdrop overlay (1800). Added a download confirmation dialog to the 'Download Agent' sidebar button. Implemented a conditional 'Back to Leaves' button on the Calendar page that only displays when navigated to from the Leaves page.</v>
+      </c>
+      <c r="F25" s="2" t="str">
+        <v>* [COMPLETED] TSK-NAV-004 (Refine Navigation Layouts: Mobile Z-Index, Download Confirmation, and Conditional Back Button): Refined mobile navigation layouts. Solved mobile sidebar menu clickability by increasing the sidebar's z-index to 1810 to place it in front of the backdrop overlay (1800). Added a download confirmation dialog to the 'Download Agent' sidebar button. Implemented a conditional 'Back to Leaves' button on the Calendar page that only displays when navigated to from the Leaves page.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B26" s="2" t="str">
+        <v>TSK-INC-001</v>
+      </c>
+      <c r="C26" s="2" t="str">
+        <v>Align Incentives Page Button Themes to Premium Theme</v>
+      </c>
+      <c r="D26" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E26" s="2" t="str">
+        <v>Unified the button styling on the Incentives page by transforming the Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes.</v>
+      </c>
+      <c r="F26" s="2" t="str">
+        <v>* [COMPLETED] TSK-INC-001 (Align Incentives Page Button Themes to Premium Theme): Unified the button styling on the Incentives page by transforming the Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F26"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1863,7 +1903,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W44"/>
+  <dimension ref="A1:W46"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -4780,7 +4820,7 @@
         <v>6</v>
       </c>
       <c r="Q41" s="2">
-        <v>3</v>
+        <v>2.6666666666666665</v>
       </c>
       <c r="R41" s="2" t="str">
         <v>100%</v>
@@ -4798,7 +4838,7 @@
         <v>2026-06-30</v>
       </c>
       <c r="W41" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, and Apply for Leave buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
       </c>
     </row>
     <row r="42">
@@ -4851,7 +4891,7 @@
         <v>4</v>
       </c>
       <c r="Q42" s="2">
-        <v>3</v>
+        <v>2.6666666666666665</v>
       </c>
       <c r="R42" s="2" t="str">
         <v>100%</v>
@@ -4869,7 +4909,7 @@
         <v>2026-06-30</v>
       </c>
       <c r="W42" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, and Apply for Leave buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
       </c>
     </row>
     <row r="43">
@@ -4922,7 +4962,7 @@
         <v>4</v>
       </c>
       <c r="Q43" s="2">
-        <v>3</v>
+        <v>2.6666666666666665</v>
       </c>
       <c r="R43" s="2" t="str">
         <v>100%</v>
@@ -4940,7 +4980,7 @@
         <v>2026-06-30</v>
       </c>
       <c r="W43" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, and Apply for Leave buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
       </c>
     </row>
     <row r="44">
@@ -4993,7 +5033,7 @@
         <v>3</v>
       </c>
       <c r="Q44" s="2">
-        <v>3</v>
+        <v>2.6666666666666665</v>
       </c>
       <c r="R44" s="2" t="str">
         <v>100%</v>
@@ -5011,12 +5051,154 @@
         <v>2026-06-30</v>
       </c>
       <c r="W44" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, and Apply for Leave buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B45" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C45" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D45" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E45" s="2" t="str">
+        <v>Sidebar &amp; Calendar Pages</v>
+      </c>
+      <c r="F45" s="2" t="str">
+        <v>Navigation</v>
+      </c>
+      <c r="G45" s="2" t="str">
+        <v>Mobile Sidebar Overlay and Download Agent Dialog</v>
+      </c>
+      <c r="H45" s="2" t="str">
+        <v>TSK-NAV-004</v>
+      </c>
+      <c r="I45" s="2" t="str">
+        <v>Refine Navigation Layouts: Mobile Z-Index, Download Confirmation, and Conditional Back Button</v>
+      </c>
+      <c r="J45" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K45" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L45" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M45" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N45" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O45" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P45" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q45" s="2">
+        <v>2.6666666666666665</v>
+      </c>
+      <c r="R45" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S45" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T45" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U45" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="V45" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="W45" s="2" t="str">
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B46" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C46" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D46" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E46" s="2" t="str">
+        <v>Incentives Page</v>
+      </c>
+      <c r="F46" s="2" t="str">
+        <v>Payroll</v>
+      </c>
+      <c r="G46" s="2" t="str">
+        <v>Incentives Button Themes</v>
+      </c>
+      <c r="H46" s="2" t="str">
+        <v>TSK-INC-001</v>
+      </c>
+      <c r="I46" s="2" t="str">
+        <v>Align Incentives Page Button Themes to Premium Theme</v>
+      </c>
+      <c r="J46" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K46" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L46" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M46" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N46" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O46" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P46" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q46" s="2">
+        <v>2.6666666666666665</v>
+      </c>
+      <c r="R46" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S46" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T46" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U46" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="V46" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="W46" s="2" t="str">
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W46"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: sync project sheet and update tracking JSONs with desktop agent tasks
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F28"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -969,9 +969,49 @@
         <v>* [COMPLETED] TSK-INC-001 (Align Incentives Page Button Themes to Premium Theme): Unified the button styling on the Incentives page by transforming the Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes.</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B27" s="2" t="str">
+        <v>TSK-DSK-002</v>
+      </c>
+      <c r="C27" s="2" t="str">
+        <v>Implement Dynamic Reminders, Early Checkout Warnings, and Status Updates in Desktop Agent</v>
+      </c>
+      <c r="D27" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E27" s="2" t="str">
+        <v>Refactored the C# desktop agent to fetch employee shift details and late penalties dynamically from the backend, replacing all hardcoded reminder times. Implemented early checkout validation to warn users before checking out with incomplete hours. Designed and integrated a new dark-themed status update dialog to collect and save daily work summaries during checkout.</v>
+      </c>
+      <c r="F27" s="2" t="str">
+        <v>* [COMPLETED] TSK-DSK-002 (Implement Dynamic Reminders, Early Checkout Warnings, and Status Updates in Desktop Agent): Refactored the C# desktop agent to fetch employee shift details and late penalties dynamically from the backend, replacing all hardcoded reminder times. Implemented early checkout validation to warn users before checking out with incomplete hours. Designed and integrated a new dark-themed status update dialog to collect and save daily work summaries during checkout.</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B28" s="2" t="str">
+        <v>TSK-DSK-003</v>
+      </c>
+      <c r="C28" s="2" t="str">
+        <v>Redesign and Center Desktop Reminder Popup with Topmost Fade Animation</v>
+      </c>
+      <c r="D28" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E28" s="2" t="str">
+        <v>Redesigned the desktop reminder popup, doubling its size to 880x480 and scaling all controls. Positioned it in the center of the screen with a smooth opacity fade-in/fade-out animation, and forced topmost focus on load using BringToFront() and Activate() to ensure it displays above all running apps.</v>
+      </c>
+      <c r="F28" s="2" t="str">
+        <v>* [COMPLETED] TSK-DSK-003 (Redesign and Center Desktop Reminder Popup with Topmost Fade Animation): Redesigned the desktop reminder popup, doubling its size to 880x480 and scaling all controls. Positioned it in the center of the screen with a smooth opacity fade-in/fade-out animation, and forced topmost focus on load using BringToFront() and Activate() to ensure it displays above all running apps.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1903,7 +1943,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W46"/>
+  <dimension ref="A1:W48"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -4820,7 +4860,7 @@
         <v>6</v>
       </c>
       <c r="Q41" s="2">
-        <v>2.6666666666666665</v>
+        <v>2.875</v>
       </c>
       <c r="R41" s="2" t="str">
         <v>100%</v>
@@ -4838,7 +4878,7 @@
         <v>2026-06-30</v>
       </c>
       <c r="W41" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page. Integrated dynamic shift-based reminders, early checkout validation and warnings, and a checkout status update dialog in the C# desktop agent, and redesigned the reminder popup to be twice as large, centered on screen, and topmost with a fade-in animation.</v>
       </c>
     </row>
     <row r="42">
@@ -4891,7 +4931,7 @@
         <v>4</v>
       </c>
       <c r="Q42" s="2">
-        <v>2.6666666666666665</v>
+        <v>2.875</v>
       </c>
       <c r="R42" s="2" t="str">
         <v>100%</v>
@@ -4909,7 +4949,7 @@
         <v>2026-06-30</v>
       </c>
       <c r="W42" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page. Integrated dynamic shift-based reminders, early checkout validation and warnings, and a checkout status update dialog in the C# desktop agent, and redesigned the reminder popup to be twice as large, centered on screen, and topmost with a fade-in animation.</v>
       </c>
     </row>
     <row r="43">
@@ -4962,7 +5002,7 @@
         <v>4</v>
       </c>
       <c r="Q43" s="2">
-        <v>2.6666666666666665</v>
+        <v>2.875</v>
       </c>
       <c r="R43" s="2" t="str">
         <v>100%</v>
@@ -4980,7 +5020,7 @@
         <v>2026-06-30</v>
       </c>
       <c r="W43" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page. Integrated dynamic shift-based reminders, early checkout validation and warnings, and a checkout status update dialog in the C# desktop agent, and redesigned the reminder popup to be twice as large, centered on screen, and topmost with a fade-in animation.</v>
       </c>
     </row>
     <row r="44">
@@ -5033,7 +5073,7 @@
         <v>3</v>
       </c>
       <c r="Q44" s="2">
-        <v>2.6666666666666665</v>
+        <v>2.875</v>
       </c>
       <c r="R44" s="2" t="str">
         <v>100%</v>
@@ -5051,7 +5091,7 @@
         <v>2026-06-30</v>
       </c>
       <c r="W44" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page. Integrated dynamic shift-based reminders, early checkout validation and warnings, and a checkout status update dialog in the C# desktop agent, and redesigned the reminder popup to be twice as large, centered on screen, and topmost with a fade-in animation.</v>
       </c>
     </row>
     <row r="45">
@@ -5104,7 +5144,7 @@
         <v>3</v>
       </c>
       <c r="Q45" s="2">
-        <v>2.6666666666666665</v>
+        <v>2.875</v>
       </c>
       <c r="R45" s="2" t="str">
         <v>100%</v>
@@ -5122,7 +5162,7 @@
         <v>2026-06-30</v>
       </c>
       <c r="W45" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page. Integrated dynamic shift-based reminders, early checkout validation and warnings, and a checkout status update dialog in the C# desktop agent, and redesigned the reminder popup to be twice as large, centered on screen, and topmost with a fade-in animation.</v>
       </c>
     </row>
     <row r="46">
@@ -5175,7 +5215,7 @@
         <v>2</v>
       </c>
       <c r="Q46" s="2">
-        <v>2.6666666666666665</v>
+        <v>2.875</v>
       </c>
       <c r="R46" s="2" t="str">
         <v>100%</v>
@@ -5193,12 +5233,154 @@
         <v>2026-06-30</v>
       </c>
       <c r="W46" s="2" t="str">
-        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page.</v>
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page. Integrated dynamic shift-based reminders, early checkout validation and warnings, and a checkout status update dialog in the C# desktop agent, and redesigned the reminder popup to be twice as large, centered on screen, and topmost with a fade-in animation.</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B47" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C47" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D47" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E47" s="2" t="str">
+        <v>Desktop Agent App</v>
+      </c>
+      <c r="F47" s="2" t="str">
+        <v>Desktop Agent</v>
+      </c>
+      <c r="G47" s="2" t="str">
+        <v>Dynamic Reminders and Checkout Validation</v>
+      </c>
+      <c r="H47" s="2" t="str">
+        <v>TSK-DSK-002</v>
+      </c>
+      <c r="I47" s="2" t="str">
+        <v>Implement Dynamic Reminders, Early Checkout Warnings, and Status Updates in Desktop Agent</v>
+      </c>
+      <c r="J47" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K47" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L47" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M47" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="N47" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O47" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P47" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q47" s="2">
+        <v>2.875</v>
+      </c>
+      <c r="R47" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S47" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T47" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U47" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="V47" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="W47" s="2" t="str">
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page. Integrated dynamic shift-based reminders, early checkout validation and warnings, and a checkout status update dialog in the C# desktop agent, and redesigned the reminder popup to be twice as large, centered on screen, and topmost with a fade-in animation.</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B48" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C48" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D48" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E48" s="2" t="str">
+        <v>Desktop Agent App</v>
+      </c>
+      <c r="F48" s="2" t="str">
+        <v>Desktop Agent</v>
+      </c>
+      <c r="G48" s="2" t="str">
+        <v>Reminder Form Centering and Sizing</v>
+      </c>
+      <c r="H48" s="2" t="str">
+        <v>TSK-DSK-003</v>
+      </c>
+      <c r="I48" s="2" t="str">
+        <v>Redesign and Center Desktop Reminder Popup with Topmost Fade Animation</v>
+      </c>
+      <c r="J48" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K48" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L48" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M48" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N48" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O48" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P48" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q48" s="2">
+        <v>2.875</v>
+      </c>
+      <c r="R48" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S48" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T48" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U48" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="V48" s="2" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="W48" s="2" t="str">
+        <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page. Integrated dynamic shift-based reminders, early checkout validation and warnings, and a checkout status update dialog in the C# desktop agent, and redesigned the reminder popup to be twice as large, centered on screen, and topmost with a fade-in animation.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W48"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: restrict attendance history monthly filter to employee panel
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1009,9 +1009,29 @@
         <v>* [COMPLETED] TSK-DSK-003 (Redesign and Center Desktop Reminder Popup with Topmost Fade Animation): Redesigned the desktop reminder popup, doubling its size to 880x480 and scaling all controls. Positioned it in the center of the screen with a smooth opacity fade-in/fade-out animation, and forced topmost focus on load using BringToFront() and Activate() to ensure it displays above all running apps.</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B29" s="2" t="str">
+        <v>TSK-ATT-017</v>
+      </c>
+      <c r="C29" s="2" t="str">
+        <v>Restrict Attendance History Monthly Filter to Employee Panel</v>
+      </c>
+      <c r="D29" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E29" s="2" t="str">
+        <v>Modified the Attendance History page to conditionally hide the 'View by Month' dropdown filter from the Manager, HR, and Admin views. It is now only visible when the active user has the 'EMPLOYEE' role.</v>
+      </c>
+      <c r="F29" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-017 (Restrict Attendance History Monthly Filter to Employee Panel): Modified the Attendance History page to conditionally hide the 'View by Month' dropdown filter from the Manager, HR, and Admin views. It is now only visible when the active user has the 'EMPLOYEE' role.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1943,7 +1963,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W48"/>
+  <dimension ref="A1:W49"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -5378,9 +5398,80 @@
         <v>Successfully redesigned the Departments page to display a grid of premium cards. The backend query was updated to fetch the active employee count in each department via Prisma relations, and the frontend renders modern gradient avatars, pill-shaped code badges, and hover lift effects. Also refined the Leaderboard page: resized the Previous Winner card to be a square block taking half the parent's height, replaced the trophy emoji with an animated party popper, and changed the employee list ranking avatars to use the same 6 premium linear gradients. Lastly, unified the button styling across the app by transforming the Add Department, Add Employee, Create Record, View Team Calendar, View Leave Balances, Apply for Leave, Create Incentive, Apply Filters, and Cancel buttons to use the dark blue accent gradient and outline themes. Restructured the Workday Progress header to center the title horizontally while keeping the status dot and badge side-by-side on the left. Correctly handled the not-checked-in state by showing a Not Checked In status label, a gray dot, and a centered placeholder text overlay inside the progress bar rail. Created a seeding script to add test1@gmail.com and test2@gmail.com test employee accounts with default profiles and leave balances. Fixed mobile sidebar clickability, added a confirmation box before downloading the desktop agent, and added a conditional 'Back to Leaves' button on the Calendar page. Integrated dynamic shift-based reminders, early checkout validation and warnings, and a checkout status update dialog in the C# desktop agent, and redesigned the reminder popup to be twice as large, centered on screen, and topmost with a fade-in animation.</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B49" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C49" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D49" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E49" s="2" t="str">
+        <v>Attendance Page</v>
+      </c>
+      <c r="F49" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G49" s="2" t="str">
+        <v>Attendance History Filters</v>
+      </c>
+      <c r="H49" s="2" t="str">
+        <v>TSK-ATT-017</v>
+      </c>
+      <c r="I49" s="2" t="str">
+        <v>Restrict Attendance History Monthly Filter to Employee Panel</v>
+      </c>
+      <c r="J49" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K49" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L49" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M49" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N49" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O49" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P49" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q49" s="2">
+        <v>1</v>
+      </c>
+      <c r="R49" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S49" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T49" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U49" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V49" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W49" s="2" t="str">
+        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W49"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: show away/on break status tag and gold dot on workday timeline
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1029,9 +1029,29 @@
         <v>* [COMPLETED] TSK-ATT-017 (Restrict Attendance History Monthly Filter to Employee Panel): Modified the Attendance History page to conditionally hide the 'View by Month' dropdown filter from the Manager, HR, and Admin views. It is now only visible when the active user has the 'EMPLOYEE' role.</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B30" s="2" t="str">
+        <v>TSK-ATT-018</v>
+      </c>
+      <c r="C30" s="2" t="str">
+        <v>Refine Attendance Status Dot and Active Labels in Workday Timeline</v>
+      </c>
+      <c r="D30" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E30" s="2" t="str">
+        <v>Refactored the Workday Timeline header to set a green status dot (active class) for checked-in late employees, indicating their active presence in the shift. Renamed the fallback 'Present' label to 'Active' for on-time check-ins.</v>
+      </c>
+      <c r="F30" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-018 (Refine Attendance Status Dot and Active Labels in Workday Timeline): Refactored the Workday Timeline header to set a green status dot (active class) for checked-in late employees, indicating their active presence in the shift. Renamed the fallback 'Present' label to 'Active' for on-time check-ins.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F30"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1963,7 +1983,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W49"/>
+  <dimension ref="A1:W50"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -5466,12 +5486,83 @@
         <v>2026-07-01</v>
       </c>
       <c r="W49" s="2" t="str">
-        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels.</v>
+        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence.</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B50" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C50" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D50" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E50" s="2" t="str">
+        <v>Dashboard Page</v>
+      </c>
+      <c r="F50" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G50" s="2" t="str">
+        <v>Workday Timeline Header Indicators</v>
+      </c>
+      <c r="H50" s="2" t="str">
+        <v>TSK-ATT-018</v>
+      </c>
+      <c r="I50" s="2" t="str">
+        <v>Refine Attendance Status Dot and Active Labels in Workday Timeline</v>
+      </c>
+      <c r="J50" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K50" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L50" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M50" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N50" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O50" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P50" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q50" s="2">
+        <v>1</v>
+      </c>
+      <c r="R50" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S50" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T50" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U50" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V50" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W50" s="2" t="str">
+        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W50"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: implement live desktop agent connectivity tracking and solve sleep/shutdown tracking bugs
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F32"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1049,9 +1049,49 @@
         <v>* [COMPLETED] TSK-ATT-018 (Refine Attendance Status Dot and Active Labels in Workday Timeline): Refactored the Workday Timeline header to set a green status dot (active class) for checked-in late employees, indicating their active presence in the shift. Renamed the fallback 'Present' label to 'Active' for on-time check-ins.</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B31" s="2" t="str">
+        <v>TSK-DSK-004</v>
+      </c>
+      <c r="C31" s="2" t="str">
+        <v>Resolve Sleep, Wake, and Shutdown Telemetry Event Logging Bugs</v>
+      </c>
+      <c r="D31" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E31" s="2" t="str">
+        <v>Fixed asynchronous event truncation during system sleep and shutdown. Subscribed to native PowerModeChanged, blocked shutdown and suspend events synchronously using GetAwaiter().GetResult(), added a 3s timeout to HTTP requests, and auto-synced offline queues on network state changes.</v>
+      </c>
+      <c r="F31" s="2" t="str">
+        <v>* [COMPLETED] TSK-DSK-004 (Resolve Sleep, Wake, and Shutdown Telemetry Event Logging Bugs): Fixed asynchronous event truncation during system sleep and shutdown. Subscribed to native PowerModeChanged, blocked shutdown and suspend events synchronously using GetAwaiter().GetResult(), added a 3s timeout to HTTP requests, and auto-synced offline queues on network state changes.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B32" s="2" t="str">
+        <v>TSK-DSK-005</v>
+      </c>
+      <c r="C32" s="2" t="str">
+        <v>Implement Live Desktop Agent Connectivity Indicator in Telemetry Tracker</v>
+      </c>
+      <c r="D32" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E32" s="2" t="str">
+        <v>Tracked live connection status of desktop agent by updating a lastDesktopActive database column. Identified desktop requests via User-Agent and displayed a laptop emoji (💻) next to active user names in the Workforce Live Status tracker.</v>
+      </c>
+      <c r="F32" s="2" t="str">
+        <v>* [COMPLETED] TSK-DSK-005 (Implement Live Desktop Agent Connectivity Indicator in Telemetry Tracker): Tracked live connection status of desktop agent by updating a lastDesktopActive database column. Identified desktop requests via User-Agent and displayed a laptop emoji (💻) next to active user names in the Workforce Live Status tracker.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F32"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1983,7 +2023,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W50"/>
+  <dimension ref="A1:W52"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -5468,7 +5508,7 @@
         <v>1</v>
       </c>
       <c r="Q49" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R49" s="2" t="str">
         <v>100%</v>
@@ -5486,7 +5526,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W49" s="2" t="str">
-        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence.</v>
+        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page.</v>
       </c>
     </row>
     <row r="50">
@@ -5539,7 +5579,7 @@
         <v>1</v>
       </c>
       <c r="Q50" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R50" s="2" t="str">
         <v>100%</v>
@@ -5557,12 +5597,154 @@
         <v>2026-07-01</v>
       </c>
       <c r="W50" s="2" t="str">
-        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence.</v>
+        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page.</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B51" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C51" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D51" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E51" s="2" t="str">
+        <v>Desktop Agent App</v>
+      </c>
+      <c r="F51" s="2" t="str">
+        <v>Desktop Agent</v>
+      </c>
+      <c r="G51" s="2" t="str">
+        <v>Telemetry Event Reliability</v>
+      </c>
+      <c r="H51" s="2" t="str">
+        <v>TSK-DSK-004</v>
+      </c>
+      <c r="I51" s="2" t="str">
+        <v>Resolve Sleep, Wake, and Shutdown Telemetry Event Logging Bugs</v>
+      </c>
+      <c r="J51" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K51" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L51" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M51" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N51" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O51" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P51" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q51" s="2">
+        <v>2</v>
+      </c>
+      <c r="R51" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S51" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T51" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U51" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V51" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W51" s="2" t="str">
+        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page.</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B52" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C52" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D52" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E52" s="2" t="str">
+        <v>Attendance Page</v>
+      </c>
+      <c r="F52" s="2" t="str">
+        <v>Desktop Agent</v>
+      </c>
+      <c r="G52" s="2" t="str">
+        <v>Live Connectivity Indicator</v>
+      </c>
+      <c r="H52" s="2" t="str">
+        <v>TSK-DSK-005</v>
+      </c>
+      <c r="I52" s="2" t="str">
+        <v>Implement Live Desktop Agent Connectivity Indicator in Telemetry Tracker</v>
+      </c>
+      <c r="J52" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K52" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L52" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="M52" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="N52" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O52" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P52" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q52" s="2">
+        <v>2</v>
+      </c>
+      <c r="R52" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S52" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T52" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U52" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V52" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W52" s="2" t="str">
+        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W52"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: resolve casing capitalization mismatch in desktop activity log sync
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -5508,7 +5508,7 @@
         <v>1</v>
       </c>
       <c r="Q49" s="2">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="R49" s="2" t="str">
         <v>100%</v>
@@ -5526,7 +5526,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W49" s="2" t="str">
-        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page.</v>
+        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page. Resolved capitalization mismatch on event logs to support seamless, backwards-compatible local event sync.</v>
       </c>
     </row>
     <row r="50">
@@ -5579,7 +5579,7 @@
         <v>1</v>
       </c>
       <c r="Q50" s="2">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="R50" s="2" t="str">
         <v>100%</v>
@@ -5597,7 +5597,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W50" s="2" t="str">
-        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page.</v>
+        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page. Resolved capitalization mismatch on event logs to support seamless, backwards-compatible local event sync.</v>
       </c>
     </row>
     <row r="51">
@@ -5650,7 +5650,7 @@
         <v>3</v>
       </c>
       <c r="Q51" s="2">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="R51" s="2" t="str">
         <v>100%</v>
@@ -5668,7 +5668,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W51" s="2" t="str">
-        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page.</v>
+        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page. Resolved capitalization mismatch on event logs to support seamless, backwards-compatible local event sync.</v>
       </c>
     </row>
     <row r="52">
@@ -5721,7 +5721,7 @@
         <v>3</v>
       </c>
       <c r="Q52" s="2">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="R52" s="2" t="str">
         <v>100%</v>
@@ -5739,7 +5739,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W52" s="2" t="str">
-        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page.</v>
+        <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page. Resolved capitalization mismatch on event logs to support seamless, backwards-compatible local event sync.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement curated CEO business-growth thought pool for Rutik Bhosle
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F35"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1089,9 +1089,69 @@
         <v>* [COMPLETED] TSK-DSK-005 (Implement Live Desktop Agent Connectivity Indicator in Telemetry Tracker): Tracked live connection status of desktop agent by updating a lastDesktopActive database column. Identified desktop requests via User-Agent and displayed a laptop emoji (💻) next to active user names in the Workforce Live Status tracker.</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B33" s="2" t="str">
+        <v>TSK-ATT-019</v>
+      </c>
+      <c r="C33" s="2" t="str">
+        <v>Fix Silent 401 Failure Hiding Desktop Event Logs in Timeline Modal</v>
+      </c>
+      <c r="D33" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E33" s="2" t="str">
+        <v>Diagnosed and resolved a silent API failure in WorkdayTimeline.tsx where the loadDesktopLogs function was firing unauthenticated requests when the token was null (scenario: admin opens Timeline from the Live Telemetry Tracker tab). The backend returned 401, but the empty catch block swallowed it silently, leaving the Event Log section always blank. Added a one-line if (!token) return guard, mirroring the identical guard already present in the sibling loadBreaks function. Build verified clean. LOCK and UNLOCK events are now visible in the Event Log.</v>
+      </c>
+      <c r="F33" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-019 (Fix Silent 401 Failure Hiding Desktop Event Logs in Timeline Modal): Diagnosed and resolved a silent API failure in WorkdayTimeline.tsx where the loadDesktopLogs function was firing unauthenticated requests when the token was null (scenario: admin opens Timeline from the Live Telemetry Tracker tab). The backend returned 401, but the empty catch block swallowed it silently, leaving the Event Log section always blank. Added a one-line if (!token) return guard, mirroring the identical guard already present in the sibling loadBreaks function. Build verified clean. LOCK and UNLOCK events are now visible in the Event Log.</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B34" s="2" t="str">
+        <v>TSK-DSH-002</v>
+      </c>
+      <c r="C34" s="2" t="str">
+        <v>Eliminate Hero Section White Flash on Page Load and Scroll Re-entry</v>
+      </c>
+      <c r="D34" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E34" s="2" t="str">
+        <v>Traced a millisecond-long white strip flashing in the Dashboard hero section to a CSS cascade conflict: the .card base style (global.css) sets background: rgba(255,255,255,0.75), which the browser paints as a solid white layer before the background-image (bgh2.jpg) is composited. The fix was to split the .dashboard-hero background shorthand into a separate background-color: #0f172a (dark fallback, painted instantly in the first GPU frame) and background-image/position/size/repeat properties, eliminating the white flash on both initial load and scroll re-entry.</v>
+      </c>
+      <c r="F34" s="2" t="str">
+        <v>* [COMPLETED] TSK-DSH-002 (Eliminate Hero Section White Flash on Page Load and Scroll Re-entry): Traced a millisecond-long white strip flashing in the Dashboard hero section to a CSS cascade conflict: the .card base style (global.css) sets background: rgba(255,255,255,0.75), which the browser paints as a solid white layer before the background-image (bgh2.jpg) is composited. The fix was to split the .dashboard-hero background shorthand into a separate background-color: #0f172a (dark fallback, painted instantly in the first GPU frame) and background-image/position/size/repeat properties, eliminating the white flash on both initial load and scroll re-entry.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B35" s="2" t="str">
+        <v>TSK-DSH-003</v>
+      </c>
+      <c r="C35" s="2" t="str">
+        <v>Implement curated business-growth thought pool for CEO profile</v>
+      </c>
+      <c r="D35" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E35" s="2" t="str">
+        <v>Developed a dedicated motivational thought pool focusing on startup and corporate business growth, partner coordination, IT product scaling, and operational leadership. Configured the ThoughtOfTheDay component to accept employeeId, checking if the logged-in user is Rutik Bhosle (employeeId: 34). Regular employees continue to receive the default team motivation quotes, while Rutik receives the CEO thought list.</v>
+      </c>
+      <c r="F35" s="2" t="str">
+        <v>* [COMPLETED] TSK-DSH-003 (Implement curated business-growth thought pool for CEO profile): Developed a dedicated motivational thought pool focusing on startup and corporate business growth, partner coordination, IT product scaling, and operational leadership. Configured the ThoughtOfTheDay component to accept employeeId, checking if the logged-in user is Rutik Bhosle (employeeId: 34). Regular employees continue to receive the default team motivation quotes, while Rutik receives the CEO thought list.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F35"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2023,13 +2083,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W52"/>
+  <dimension ref="A1:W55"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="41.83203125" customWidth="1"/>
+    <col min="5" max="5" width="43.83203125" customWidth="1"/>
     <col min="6" max="6" width="30.83203125" customWidth="1"/>
     <col min="7" max="7" width="61.83203125" customWidth="1"/>
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
@@ -5742,9 +5802,222 @@
         <v>Restricted the View by Month dropdown select box on the Attendance History tab to the Employee panel, making it hidden in the other 3 administrative panels. Refined the Workday Progress header status tags: renamed the 'Present' tag to 'Active' for on-time checked-in employees, and ensured late check-ins use a green pulsing dot to indicate active shift presence. Fully resolved the C# desktop agent telemetry capture bugs for sleep, wake, and shutdown events using native OS power mode listeners, synchronous blocking handlers, and network state auto-sync. Built and integrated a live desktop connectivity indicator (💻) in the Workforce Live status table on the admin page. Resolved capitalization mismatch on event logs to support seamless, backwards-compatible local event sync.</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B53" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C53" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D53" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E53" s="2" t="str">
+        <v>Attendance Page — Live Telemetry Tracker</v>
+      </c>
+      <c r="F53" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G53" s="2" t="str">
+        <v>Workday Timeline Event Log Fix</v>
+      </c>
+      <c r="H53" s="2" t="str">
+        <v>TSK-ATT-019</v>
+      </c>
+      <c r="I53" s="2" t="str">
+        <v>Fix Silent 401 Failure Hiding Desktop Event Logs in Timeline Modal</v>
+      </c>
+      <c r="J53" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K53" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L53" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M53" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N53" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O53" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P53" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q53" s="2">
+        <v>1</v>
+      </c>
+      <c r="R53" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S53" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T53" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U53" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V53" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W53" s="2" t="str">
+        <v>Completed two critical bug fixes and implemented a custom feature: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated, business-growth-focused thought pool specifically for the CEO (Rutik Bhosle, employeeId 34) on the dashboard.</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B54" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C54" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D54" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E54" s="2" t="str">
+        <v>Dashboard — Hero Section</v>
+      </c>
+      <c r="F54" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G54" s="2" t="str">
+        <v>Hero Section White Flash Fix</v>
+      </c>
+      <c r="H54" s="2" t="str">
+        <v>TSK-DSH-002</v>
+      </c>
+      <c r="I54" s="2" t="str">
+        <v>Eliminate Hero Section White Flash on Page Load and Scroll Re-entry</v>
+      </c>
+      <c r="J54" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K54" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L54" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M54" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N54" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O54" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P54" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q54" s="2">
+        <v>1</v>
+      </c>
+      <c r="R54" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S54" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T54" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U54" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V54" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W54" s="2" t="str">
+        <v>Completed two critical bug fixes and implemented a custom feature: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated, business-growth-focused thought pool specifically for the CEO (Rutik Bhosle, employeeId 34) on the dashboard.</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B55" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C55" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D55" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E55" s="2" t="str">
+        <v>Dashboard Page</v>
+      </c>
+      <c r="F55" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G55" s="2" t="str">
+        <v>CEO Motivational Thought Pool</v>
+      </c>
+      <c r="H55" s="2" t="str">
+        <v>TSK-DSH-003</v>
+      </c>
+      <c r="I55" s="2" t="str">
+        <v>Implement curated business-growth thought pool for CEO profile</v>
+      </c>
+      <c r="J55" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K55" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L55" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M55" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N55" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O55" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P55" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q55" s="2">
+        <v>1</v>
+      </c>
+      <c r="R55" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S55" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T55" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U55" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V55" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W55" s="2" t="str">
+        <v>Completed two critical bug fixes and implemented a custom feature: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated, business-growth-focused thought pool specifically for the CEO (Rutik Bhosle, employeeId 34) on the dashboard.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W55"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
layout: refine management dashboard hero layout with left greeting/badge/context and right thoughts
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1149,9 +1149,29 @@
         <v>* [COMPLETED] TSK-DSH-003 (Implement curated business-growth thought pool for CEO profile): Developed a dedicated motivational thought pool focusing on startup and corporate business growth, partner coordination, IT product scaling, and operational leadership. Configured the ThoughtOfTheDay component to accept employeeId, checking if the logged-in user is Rutik Bhosle (employeeId: 34). Regular employees continue to receive the default team motivation quotes, while Rutik receives the CEO thought list.</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B36" s="2" t="str">
+        <v>TSK-DSH-004</v>
+      </c>
+      <c r="C36" s="2" t="str">
+        <v>Refine Management Hero layout: left-aligned greeting, designation badge, pill context and right-aligned thoughts</v>
+      </c>
+      <c r="D36" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E36" s="2" t="str">
+        <v>Swapped the layout of the dashboard hero section for managers/admins. Swapped the placement of the greeting and ThoughtOfTheDay components to put the greeting, name, and designation on the left and thoughts on the right. Styled the title group as a compact horizontal pill/card, and added CEO/Manager designation badges next to the name.</v>
+      </c>
+      <c r="F36" s="2" t="str">
+        <v>* [COMPLETED] TSK-DSH-004 (Refine Management Hero layout: left-aligned greeting, designation badge, pill context and right-aligned thoughts): Swapped the layout of the dashboard hero section for managers/admins. Swapped the placement of the greeting and ThoughtOfTheDay components to put the greeting, name, and designation on the left and thoughts on the right. Styled the title group as a compact horizontal pill/card, and added CEO/Manager designation badges next to the name.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2083,7 +2103,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W55"/>
+  <dimension ref="A1:W56"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -5870,7 +5890,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W53" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented a custom feature: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated, business-growth-focused thought pool specifically for the CEO (Rutik Bhosle, employeeId 34) on the dashboard.</v>
+        <v>Completed two critical bug fixes and implemented two dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated business thought pool for the CEO (Rutik Bhosle, employeeId 34). (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
     <row r="54">
@@ -5941,7 +5961,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W54" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented a custom feature: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated, business-growth-focused thought pool specifically for the CEO (Rutik Bhosle, employeeId 34) on the dashboard.</v>
+        <v>Completed two critical bug fixes and implemented two dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated business thought pool for the CEO (Rutik Bhosle, employeeId 34). (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
     <row r="55">
@@ -6012,12 +6032,83 @@
         <v>2026-07-01</v>
       </c>
       <c r="W55" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented a custom feature: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated, business-growth-focused thought pool specifically for the CEO (Rutik Bhosle, employeeId 34) on the dashboard.</v>
+        <v>Completed two critical bug fixes and implemented two dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated business thought pool for the CEO (Rutik Bhosle, employeeId 34). (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B56" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C56" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D56" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E56" s="2" t="str">
+        <v>Dashboard Page</v>
+      </c>
+      <c r="F56" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G56" s="2" t="str">
+        <v>Management Hero Layout Refinement</v>
+      </c>
+      <c r="H56" s="2" t="str">
+        <v>TSK-DSH-004</v>
+      </c>
+      <c r="I56" s="2" t="str">
+        <v>Refine Management Hero layout: left-aligned greeting, designation badge, pill context and right-aligned thoughts</v>
+      </c>
+      <c r="J56" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K56" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L56" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M56" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N56" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O56" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P56" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q56" s="2">
+        <v>1</v>
+      </c>
+      <c r="R56" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S56" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T56" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U56" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V56" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W56" s="2" t="str">
+        <v>Completed two critical bug fixes and implemented two dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated business thought pool for the CEO (Rutik Bhosle, employeeId 34). (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W56"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: implement dynamic thought pools for CEO, MD, HR, and general employees
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1169,9 +1169,29 @@
         <v>* [COMPLETED] TSK-DSH-004 (Refine Management Hero layout: left-aligned greeting, designation badge, pill context and right-aligned thoughts): Swapped the layout of the dashboard hero section for managers/admins. Swapped the placement of the greeting and ThoughtOfTheDay components to put the greeting, name, and designation on the left and thoughts on the right. Styled the title group as a compact horizontal pill/card, and added CEO/Manager designation badges next to the name.</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B37" s="2" t="str">
+        <v>TSK-DSH-005</v>
+      </c>
+      <c r="C37" s="2" t="str">
+        <v>Implement dynamic relatable thought pools for CEO, MD, HR, and regular employees</v>
+      </c>
+      <c r="D37" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E37" s="2" t="str">
+        <v>Expanded the role-specific thoughts feature. Created 4 distinct motivational quote pools: (1) CEO thoughts on startup and corporate growth, (2) MD thoughts on strategic operations and standard systems, (3) HR thoughts on culture, empathy, and employee mentoring, and (4) Employee thoughts on clean code, software craftsmanship, and problem solving. Refactored ThoughtOfTheDay to check jobTitle/role properties and dynamically select the pool, and updated dashboard invocations.</v>
+      </c>
+      <c r="F37" s="2" t="str">
+        <v>* [COMPLETED] TSK-DSH-005 (Implement dynamic relatable thought pools for CEO, MD, HR, and regular employees): Expanded the role-specific thoughts feature. Created 4 distinct motivational quote pools: (1) CEO thoughts on startup and corporate growth, (2) MD thoughts on strategic operations and standard systems, (3) HR thoughts on culture, empathy, and employee mentoring, and (4) Employee thoughts on clean code, software craftsmanship, and problem solving. Refactored ThoughtOfTheDay to check jobTitle/role properties and dynamically select the pool, and updated dashboard invocations.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2103,7 +2123,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W56"/>
+  <dimension ref="A1:W57"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -5890,7 +5910,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W53" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented two dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated business thought pool for the CEO (Rutik Bhosle, employeeId 34). (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed two critical bug fixes and implemented three dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
     <row r="54">
@@ -5961,7 +5981,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W54" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented two dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated business thought pool for the CEO (Rutik Bhosle, employeeId 34). (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed two critical bug fixes and implemented three dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
     <row r="55">
@@ -6032,7 +6052,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W55" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented two dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated business thought pool for the CEO (Rutik Bhosle, employeeId 34). (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed two critical bug fixes and implemented three dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
     <row r="56">
@@ -6103,12 +6123,83 @@
         <v>2026-07-01</v>
       </c>
       <c r="W56" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented two dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added a dedicated business thought pool for the CEO (Rutik Bhosle, employeeId 34). (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed two critical bug fixes and implemented three dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B57" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C57" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D57" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E57" s="2" t="str">
+        <v>Dashboard Page</v>
+      </c>
+      <c r="F57" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G57" s="2" t="str">
+        <v>Relatable Thought Pools by Role</v>
+      </c>
+      <c r="H57" s="2" t="str">
+        <v>TSK-DSH-005</v>
+      </c>
+      <c r="I57" s="2" t="str">
+        <v>Implement dynamic relatable thought pools for CEO, MD, HR, and regular employees</v>
+      </c>
+      <c r="J57" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K57" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L57" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M57" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N57" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O57" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P57" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q57" s="2">
+        <v>1</v>
+      </c>
+      <c r="R57" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S57" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T57" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U57" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V57" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W57" s="2" t="str">
+        <v>Completed two critical bug fixes and implemented three dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W57"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
layout: align employee dashboard hero layout with the management hero layout
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1189,9 +1189,29 @@
         <v>* [COMPLETED] TSK-DSH-005 (Implement dynamic relatable thought pools for CEO, MD, HR, and regular employees): Expanded the role-specific thoughts feature. Created 4 distinct motivational quote pools: (1) CEO thoughts on startup and corporate growth, (2) MD thoughts on strategic operations and standard systems, (3) HR thoughts on culture, empathy, and employee mentoring, and (4) Employee thoughts on clean code, software craftsmanship, and problem solving. Refactored ThoughtOfTheDay to check jobTitle/role properties and dynamically select the pool, and updated dashboard invocations.</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B38" s="2" t="str">
+        <v>TSK-DSH-006</v>
+      </c>
+      <c r="C38" s="2" t="str">
+        <v>Refine Employee Hero layout: left-aligned greeting, designation badge, pill context and right-aligned thoughts</v>
+      </c>
+      <c r="D38" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E38" s="2" t="str">
+        <v>Brought the Employee Dashboard hero section into full visual alignment with the refined Management Dashboard hero. Swapped components to place the user's name greeting, designation badge, and a new compact 'Personal Workspace | Employee Dashboard' pill context on the left, and right-aligned the ThoughtOfTheDay quotes on the right side.</v>
+      </c>
+      <c r="F38" s="2" t="str">
+        <v>* [COMPLETED] TSK-DSH-006 (Refine Employee Hero layout: left-aligned greeting, designation badge, pill context and right-aligned thoughts): Brought the Employee Dashboard hero section into full visual alignment with the refined Management Dashboard hero. Swapped components to place the user's name greeting, designation badge, and a new compact 'Personal Workspace | Employee Dashboard' pill context on the left, and right-aligned the ThoughtOfTheDay quotes on the right side.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2123,7 +2143,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W57"/>
+  <dimension ref="A1:W58"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -5910,7 +5930,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W53" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented three dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
     <row r="54">
@@ -5981,7 +6001,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W54" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented three dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
     <row r="55">
@@ -6052,7 +6072,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W55" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented three dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
     <row r="56">
@@ -6123,7 +6143,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W56" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented three dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
     <row r="57">
@@ -6194,12 +6214,83 @@
         <v>2026-07-01</v>
       </c>
       <c r="W57" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented three dashboard features: (1) Added token guard to WorkdayTimeline.tsx to prevent silent 401 failures loading event logs. (2) Eliminated hero section white flash by separating background-color from background-image on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Swapped the Management dashboard hero layout to place name greeting and designation badge on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B58" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C58" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D58" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E58" s="2" t="str">
+        <v>Dashboard Page</v>
+      </c>
+      <c r="F58" s="2" t="str">
+        <v>Role Dashboards &amp; Analytics</v>
+      </c>
+      <c r="G58" s="2" t="str">
+        <v>Employee Hero Layout Refinement</v>
+      </c>
+      <c r="H58" s="2" t="str">
+        <v>TSK-DSH-006</v>
+      </c>
+      <c r="I58" s="2" t="str">
+        <v>Refine Employee Hero layout: left-aligned greeting, designation badge, pill context and right-aligned thoughts</v>
+      </c>
+      <c r="J58" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K58" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L58" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M58" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N58" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O58" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P58" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q58" s="2">
+        <v>1</v>
+      </c>
+      <c r="R58" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S58" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T58" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U58" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V58" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W58" s="2" t="str">
+        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W58"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: parse correct attendance Date from desktop events and clean up old break sessions
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1209,9 +1209,29 @@
         <v>* [COMPLETED] TSK-DSH-006 (Refine Employee Hero layout: left-aligned greeting, designation badge, pill context and right-aligned thoughts): Brought the Employee Dashboard hero section into full visual alignment with the refined Management Dashboard hero. Swapped components to place the user's name greeting, designation badge, and a new compact 'Personal Workspace | Employee Dashboard' pill context on the left, and right-aligned the ThoughtOfTheDay quotes on the right side.</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B39" s="2" t="str">
+        <v>TSK-ATT-021</v>
+      </c>
+      <c r="C39" s="2" t="str">
+        <v>Fix desktop activity timeline data mapping and cleanup duplicate/offline synced breaks</v>
+      </c>
+      <c r="D39" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E39" s="2" t="str">
+        <v>Resolved a critical bug where offline queued events uploaded from the Windows C# desktop client replayed previous dates (e.g., June 25th or 29th) but linked their break session transitions to the current calendar date in the database. Refactored the backend /desktop-event endpoint in routes.ts to parse the attendanceDate parameter from the event's actual timestamp instead of hardcoding today's date. Wrote and ran a database cleanup script (cleanup_harshada_breaks.ts) to correctly re-map Harshada Nichit's duplicate previous days' breaks (June 25th and 29th) to their correct historical records, clearing today's (July 1st) timeline logs.</v>
+      </c>
+      <c r="F39" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-021 (Fix desktop activity timeline data mapping and cleanup duplicate/offline synced breaks): Resolved a critical bug where offline queued events uploaded from the Windows C# desktop client replayed previous dates (e.g., June 25th or 29th) but linked their break session transitions to the current calendar date in the database. Refactored the backend /desktop-event endpoint in routes.ts to parse the attendanceDate parameter from the event's actual timestamp instead of hardcoding today's date. Wrote and ran a database cleanup script (cleanup_harshada_breaks.ts) to correctly re-map Harshada Nichit's duplicate previous days' breaks (June 25th and 29th) to their correct historical records, clearing today's (July 1st) timeline logs.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F39"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2143,7 +2163,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W58"/>
+  <dimension ref="A1:W59"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -5930,7 +5950,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W53" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
       </c>
     </row>
     <row r="54">
@@ -6001,7 +6021,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W54" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
       </c>
     </row>
     <row r="55">
@@ -6072,7 +6092,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W55" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
       </c>
     </row>
     <row r="56">
@@ -6143,7 +6163,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W56" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
       </c>
     </row>
     <row r="57">
@@ -6214,7 +6234,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W57" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
       </c>
     </row>
     <row r="58">
@@ -6285,12 +6305,83 @@
         <v>2026-07-01</v>
       </c>
       <c r="W58" s="2" t="str">
-        <v>Completed two critical bug fixes and implemented dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both Employee and Management dashboards to place name greeting and designation badges on the left in a small style context pill, and quotes right-aligned on the right.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B59" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C59" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D59" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E59" s="2" t="str">
+        <v>Attendance Page &amp; Timeline Modal</v>
+      </c>
+      <c r="F59" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G59" s="2" t="str">
+        <v>Desktop Event Sync Fix</v>
+      </c>
+      <c r="H59" s="2" t="str">
+        <v>TSK-ATT-021</v>
+      </c>
+      <c r="I59" s="2" t="str">
+        <v>Fix desktop activity timeline data mapping and cleanup duplicate/offline synced breaks</v>
+      </c>
+      <c r="J59" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K59" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L59" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="M59" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="N59" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O59" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P59" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q59" s="2">
+        <v>1</v>
+      </c>
+      <c r="R59" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S59" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T59" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U59" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V59" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W59" s="2" t="str">
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W59"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: smart classification of scheduled breaks and fallback telemetry activity logs
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F41"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1229,9 +1229,49 @@
         <v>* [COMPLETED] TSK-ATT-021 (Fix desktop activity timeline data mapping and cleanup duplicate/offline synced breaks): Resolved a critical bug where offline queued events uploaded from the Windows C# desktop client replayed previous dates (e.g., June 25th or 29th) but linked their break session transitions to the current calendar date in the database. Refactored the backend /desktop-event endpoint in routes.ts to parse the attendanceDate parameter from the event's actual timestamp instead of hardcoding today's date. Wrote and ran a database cleanup script (cleanup_harshada_breaks.ts) to correctly re-map Harshada Nichit's duplicate previous days' breaks (June 25th and 29th) to their correct historical records, clearing today's (July 1st) timeline logs.</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B40" s="2" t="str">
+        <v>TSK-ATT-022</v>
+      </c>
+      <c r="C40" s="2" t="str">
+        <v>Clean up Workday Timeline Event Log redundancy and transient breaks</v>
+      </c>
+      <c r="D40" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E40" s="2" t="str">
+        <v>Resolved visual clutter in the Event Log where redundant desktop activity logs (e.g. Screen Locked, Went Idle) and their triggered break sessions (Lunch Break Started, etc.) were both listed at the exact same minute. Refactored WorkdayTimeline.tsx to: (1) filter out raw desktop activity logs if they correspond to a break session transition within 60 seconds; (2) hide transient break sessions that lasted less than 1 minute (e.g., brief 10-second screen locks) from the text log list, keeping the Event Log clean, structured, and easy to read.</v>
+      </c>
+      <c r="F40" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-022 (Clean up Workday Timeline Event Log redundancy and transient breaks): Resolved visual clutter in the Event Log where redundant desktop activity logs (e.g. Screen Locked, Went Idle) and their triggered break sessions (Lunch Break Started, etc.) were both listed at the exact same minute. Refactored WorkdayTimeline.tsx to: (1) filter out raw desktop activity logs if they correspond to a break session transition within 60 seconds; (2) hide transient break sessions that lasted less than 1 minute (e.g., brief 10-second screen locks) from the text log list, keeping the Event Log clean, structured, and easy to read.</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B41" s="2" t="str">
+        <v>TSK-ATT-023</v>
+      </c>
+      <c r="C41" s="2" t="str">
+        <v>Implement smart break event classification matching scheduled ranges in timeline logs</v>
+      </c>
+      <c r="D41" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E41" s="2" t="str">
+        <v>Implemented a smart visual mapping rule in WorkdayTimeline.tsx for logs and activity: (1) Locks, suspends, and idle times are classified as official breaks (e.g. Lunch Break, Tea Break) only if they overlap with the company's official break schedule ranges or were manually started from the web dashboard; (2) Lock/idle periods outside scheduled break hours are displayed with their actual telemetry descriptions (e.g., Screen Locked, Went Idle) instead of generic tea/lunch breaks, providing clear and accurate timelines.</v>
+      </c>
+      <c r="F41" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-023 (Implement smart break event classification matching scheduled ranges in timeline logs): Implemented a smart visual mapping rule in WorkdayTimeline.tsx for logs and activity: (1) Locks, suspends, and idle times are classified as official breaks (e.g. Lunch Break, Tea Break) only if they overlap with the company's official break schedule ranges or were manually started from the web dashboard; (2) Lock/idle periods outside scheduled break hours are displayed with their actual telemetry descriptions (e.g., Screen Locked, Went Idle) instead of generic tea/lunch breaks, providing clear and accurate timelines.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F41"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2163,7 +2203,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W59"/>
+  <dimension ref="A1:W61"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -5950,7 +5990,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W53" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
       </c>
     </row>
     <row r="54">
@@ -6021,7 +6061,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W54" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
       </c>
     </row>
     <row r="55">
@@ -6092,7 +6132,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W55" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
       </c>
     </row>
     <row r="56">
@@ -6163,7 +6203,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W56" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
       </c>
     </row>
     <row r="57">
@@ -6234,7 +6274,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W57" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
       </c>
     </row>
     <row r="58">
@@ -6305,7 +6345,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W58" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
       </c>
     </row>
     <row r="59">
@@ -6376,12 +6416,154 @@
         <v>2026-07-01</v>
       </c>
       <c r="W59" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools for CEO, MD, HR, and general employees. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event and cleaned up 9 previous days' break records mapped to Harshada Nichit's July 1st attendance.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B60" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C60" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D60" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E60" s="2" t="str">
+        <v>Attendance Page &amp; Timeline Modal</v>
+      </c>
+      <c r="F60" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G60" s="2" t="str">
+        <v>Timeline Redundancy Filter</v>
+      </c>
+      <c r="H60" s="2" t="str">
+        <v>TSK-ATT-022</v>
+      </c>
+      <c r="I60" s="2" t="str">
+        <v>Clean up Workday Timeline Event Log redundancy and transient breaks</v>
+      </c>
+      <c r="J60" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K60" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L60" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M60" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N60" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O60" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P60" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q60" s="2">
+        <v>1</v>
+      </c>
+      <c r="R60" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S60" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T60" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U60" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V60" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W60" s="2" t="str">
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B61" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C61" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D61" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E61" s="2" t="str">
+        <v>Attendance Page &amp; Timeline Modal</v>
+      </c>
+      <c r="F61" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G61" s="2" t="str">
+        <v>Smart Break Event Classification</v>
+      </c>
+      <c r="H61" s="2" t="str">
+        <v>TSK-ATT-023</v>
+      </c>
+      <c r="I61" s="2" t="str">
+        <v>Implement smart break event classification matching scheduled ranges in timeline logs</v>
+      </c>
+      <c r="J61" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K61" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L61" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M61" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N61" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O61" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P61" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q61" s="2">
+        <v>1</v>
+      </c>
+      <c r="R61" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S61" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T61" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U61" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V61" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W61" s="2" t="str">
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W61"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: resolve desktop client agent early reminder triggers
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1269,9 +1269,29 @@
         <v>* [COMPLETED] TSK-ATT-023 (Implement smart break event classification matching scheduled ranges in timeline logs): Implemented a smart visual mapping rule in WorkdayTimeline.tsx for logs and activity: (1) Locks, suspends, and idle times are classified as official breaks (e.g. Lunch Break, Tea Break) only if they overlap with the company's official break schedule ranges or were manually started from the web dashboard; (2) Lock/idle periods outside scheduled break hours are displayed with their actual telemetry descriptions (e.g., Screen Locked, Went Idle) instead of generic tea/lunch breaks, providing clear and accurate timelines.</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B42" s="2" t="str">
+        <v>TSK-ATT-024</v>
+      </c>
+      <c r="C42" s="2" t="str">
+        <v>Fix C# desktop agent break reminder popups triggering too early</v>
+      </c>
+      <c r="D42" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E42" s="2" t="str">
+        <v>Resolved a timing issue in the Windows C# desktop agent application where break reminder popups triggered 20-30 minutes early relative to their hardcoded notification strings (e.g. triggering Lunch Reminder at 12:30 PM instead of 1:00 PM). Refactored Program.cs to trigger break reminders based on the actual target schedules (10:45 AM for Morning Tea, 1:00 PM for Lunch, and 4:10 PM for Evening Tea) instead of using the shift's wide allowed window start bounds.</v>
+      </c>
+      <c r="F42" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-024 (Fix C# desktop agent break reminder popups triggering too early): Resolved a timing issue in the Windows C# desktop agent application where break reminder popups triggered 20-30 minutes early relative to their hardcoded notification strings (e.g. triggering Lunch Reminder at 12:30 PM instead of 1:00 PM). Refactored Program.cs to trigger break reminders based on the actual target schedules (10:45 AM for Morning Tea, 1:00 PM for Lunch, and 4:10 PM for Evening Tea) instead of using the shift's wide allowed window start bounds.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F42"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2203,7 +2223,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W61"/>
+  <dimension ref="A1:W62"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -5990,7 +6010,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W53" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
       </c>
     </row>
     <row r="54">
@@ -6061,7 +6081,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W54" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
       </c>
     </row>
     <row r="55">
@@ -6132,7 +6152,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W55" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
       </c>
     </row>
     <row r="56">
@@ -6203,7 +6223,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W56" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
       </c>
     </row>
     <row r="57">
@@ -6274,7 +6294,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W57" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
       </c>
     </row>
     <row r="58">
@@ -6345,7 +6365,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W58" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
       </c>
     </row>
     <row r="59">
@@ -6416,7 +6436,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W59" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
       </c>
     </row>
     <row r="60">
@@ -6487,7 +6507,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W60" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
       </c>
     </row>
     <row r="61">
@@ -6558,12 +6578,83 @@
         <v>2026-07-01</v>
       </c>
       <c r="W61" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts on both dashboards. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items and hid completed transient break sessions. (7) Classified locks and idle times as breaks only if they fall inside scheduled break hours, falling back to raw telemetry descriptions otherwise.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B62" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C62" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D62" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E62" s="2" t="str">
+        <v>Desktop Client App</v>
+      </c>
+      <c r="F62" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G62" s="2" t="str">
+        <v>Desktop Agent Reminders</v>
+      </c>
+      <c r="H62" s="2" t="str">
+        <v>TSK-ATT-024</v>
+      </c>
+      <c r="I62" s="2" t="str">
+        <v>Fix C# desktop agent break reminder popups triggering too early</v>
+      </c>
+      <c r="J62" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K62" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L62" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M62" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N62" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O62" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P62" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q62" s="2">
+        <v>1</v>
+      </c>
+      <c r="R62" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S62" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T62" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U62" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V62" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W62" s="2" t="str">
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W62"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
build: publish self-contained release and update download zip
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1289,9 +1289,29 @@
         <v>* [COMPLETED] TSK-ATT-024 (Fix C# desktop agent break reminder popups triggering too early): Resolved a timing issue in the Windows C# desktop agent application where break reminder popups triggered 20-30 minutes early relative to their hardcoded notification strings (e.g. triggering Lunch Reminder at 12:30 PM instead of 1:00 PM). Refactored Program.cs to trigger break reminders based on the actual target schedules (10:45 AM for Morning Tea, 1:00 PM for Lunch, and 4:10 PM for Evening Tea) instead of using the shift's wide allowed window start bounds.</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B43" s="2" t="str">
+        <v>TSK-ATT-025</v>
+      </c>
+      <c r="C43" s="2" t="str">
+        <v>Publish and package desktop agent binary zip for client deployment</v>
+      </c>
+      <c r="D43" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E43" s="2" t="str">
+        <v>Published a self-contained Release build of the Windows C# desktop agent application using the local .NET SDK. Packaged the compilation directory (including system dependencies and framework assemblies) into a zipped archive (HRMS_Agent.zip) and placed it in the frontend's public downloads directory, allowing seamless desktop client updates from the web dashboard.</v>
+      </c>
+      <c r="F43" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-025 (Publish and package desktop agent binary zip for client deployment): Published a self-contained Release build of the Windows C# desktop agent application using the local .NET SDK. Packaged the compilation directory (including system dependencies and framework assemblies) into a zipped archive (HRMS_Agent.zip) and placed it in the frontend's public downloads directory, allowing seamless desktop client updates from the web dashboard.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F43"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2223,7 +2243,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W62"/>
+  <dimension ref="A1:W63"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -6010,7 +6030,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W53" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
       </c>
     </row>
     <row r="54">
@@ -6081,7 +6101,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W54" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
       </c>
     </row>
     <row r="55">
@@ -6152,7 +6172,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W55" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
       </c>
     </row>
     <row r="56">
@@ -6223,7 +6243,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W56" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
       </c>
     </row>
     <row r="57">
@@ -6294,7 +6314,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W57" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
       </c>
     </row>
     <row r="58">
@@ -6365,7 +6385,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W58" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
       </c>
     </row>
     <row r="59">
@@ -6436,7 +6456,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W59" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
       </c>
     </row>
     <row r="60">
@@ -6507,7 +6527,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W60" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
       </c>
     </row>
     <row r="61">
@@ -6578,7 +6598,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W61" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
       </c>
     </row>
     <row r="62">
@@ -6649,12 +6669,83 @@
         <v>2026-07-01</v>
       </c>
       <c r="W62" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic in /desktop-event. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned C# desktop agent break reminder popup triggers to fire exactly at scheduled target break times.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B63" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C63" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D63" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E63" s="2" t="str">
+        <v>Desktop Client App</v>
+      </c>
+      <c r="F63" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G63" s="2" t="str">
+        <v>Packaging &amp; Deployment</v>
+      </c>
+      <c r="H63" s="2" t="str">
+        <v>TSK-ATT-025</v>
+      </c>
+      <c r="I63" s="2" t="str">
+        <v>Publish and package desktop agent binary zip for client deployment</v>
+      </c>
+      <c r="J63" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K63" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L63" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M63" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N63" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O63" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P63" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q63" s="2">
+        <v>1</v>
+      </c>
+      <c r="R63" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S63" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T63" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U63" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V63" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W63" s="2" t="str">
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W63"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: filter out historical desktop activity events in live status query
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1309,9 +1309,29 @@
         <v>* [COMPLETED] TSK-ATT-025 (Publish and package desktop agent binary zip for client deployment): Published a self-contained Release build of the Windows C# desktop agent application using the local .NET SDK. Packaged the compilation directory (including system dependencies and framework assemblies) into a zipped archive (HRMS_Agent.zip) and placed it in the frontend's public downloads directory, allowing seamless desktop client updates from the web dashboard.</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B44" s="2" t="str">
+        <v>TSK-ATT-026</v>
+      </c>
+      <c r="C44" s="2" t="str">
+        <v>Filter live-status activity logs query to the current date</v>
+      </c>
+      <c r="D44" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E44" s="2" t="str">
+        <v>Resolved a bug where employees who haven't sent desktop events today were showing old offline-synced sleep/lock times from previous days (e.g. June 26th) in their live status metadata and being incorrectly marked as AWAY. Refactored the GET /api/attendance/live-status endpoint in routes.ts to filter desktopActivityLogs selection to only include events occurring greater than or equal to the start of today.</v>
+      </c>
+      <c r="F44" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-026 (Filter live-status activity logs query to the current date): Resolved a bug where employees who haven't sent desktop events today were showing old offline-synced sleep/lock times from previous days (e.g. June 26th) in their live status metadata and being incorrectly marked as AWAY. Refactored the GET /api/attendance/live-status endpoint in routes.ts to filter desktopActivityLogs selection to only include events occurring greater than or equal to the start of today.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F44"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2243,7 +2263,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W63"/>
+  <dimension ref="A1:W64"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -6030,7 +6050,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W53" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
     <row r="54">
@@ -6101,7 +6121,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W54" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
     <row r="55">
@@ -6172,7 +6192,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W55" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
     <row r="56">
@@ -6243,7 +6263,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W56" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
     <row r="57">
@@ -6314,7 +6334,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W57" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
     <row r="58">
@@ -6385,7 +6405,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W58" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
     <row r="59">
@@ -6456,7 +6476,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W59" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
     <row r="60">
@@ -6527,7 +6547,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W60" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
     <row r="61">
@@ -6598,7 +6618,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W61" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
     <row r="62">
@@ -6669,7 +6689,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="W62" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
     <row r="63">
@@ -6740,12 +6760,83 @@
         <v>2026-07-01</v>
       </c>
       <c r="W63" s="2" t="str">
-        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build of the desktop agent (HRMS_Agent.zip) in the public downloads directory.</v>
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B64" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C64" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D64" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E64" s="2" t="str">
+        <v>Live Status Board / Active Workspace</v>
+      </c>
+      <c r="F64" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G64" s="2" t="str">
+        <v>Live Activity Query Filter</v>
+      </c>
+      <c r="H64" s="2" t="str">
+        <v>TSK-ATT-026</v>
+      </c>
+      <c r="I64" s="2" t="str">
+        <v>Filter live-status activity logs query to the current date</v>
+      </c>
+      <c r="J64" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K64" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L64" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M64" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="N64" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O64" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P64" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q64" s="2">
+        <v>1</v>
+      </c>
+      <c r="R64" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S64" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T64" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U64" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="V64" s="2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="W64" s="2" t="str">
+        <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W64"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>